<commit_message>
Corrige et enrichit TABLEAU_DE_BORD_CYCLES_OPERATOIRES.xlsx (taxonomie EOD/TFJ corrigee, 6 feuilles)
La version precedente utilisait encore "EOD Ventes" pour designer le
cycle de nuit reellement construit - corrige partout (c'est un TFJ).

Nouvelle feuille "Taxonomie complete" : les 14 types de traitement
bancaires reels (JOUR/NRT, TFJ, EOD, EOW, EOM, EOQ, EOY, CUTOFF,
REPLAY, PURGE, SIMULATION, REALTIME, ON_DEMAND) avec statut honnete
par type chez ECF.

Feuille "Cycle EOD Ventes" renommee "Cycles reels construits" et
etendue aux 5 exemples reels desormais construits (TFJ Ventes, EOD
Comptabilite, CUTOFF Achat, JOUR Ventes, PURGE Systeme) au lieu d'un
seul. Feuille "Objectifs par module" mise a jour (cycles suggeres
corriges module par module selon la taxonomie precise, statuts reels
pour CR/VT/CP/AH). Parite Control-M etendue avec les nouvelles lignes.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/TABLEAU_DE_BORD_CYCLES_OPERATOIRES.xlsx
+++ b/docs/TABLEAU_DE_BORD_CYCLES_OPERATOIRES.xlsx
@@ -8,20 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP PROBOOK\Documents\ECF\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DC1ACB2-BBEE-4861-BF4A-7BBF6A395159}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23F80ACD-A0BE-4D41-AD48-491CDF667316}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2472" yWindow="2472" windowWidth="17280" windowHeight="8880" xr2:uid="{7A3F6830-CDDC-4BD6-9DB9-E70917F562BA}"/>
+    <workbookView xWindow="2472" yWindow="2472" windowWidth="17280" windowHeight="8880" xr2:uid="{DDABEE53-8415-4B60-8DAA-76C5DBFE148E}"/>
   </bookViews>
   <sheets>
     <sheet name="Vue d'ensemble" sheetId="1" r:id="rId1"/>
     <sheet name="Objectifs par module" sheetId="2" r:id="rId2"/>
-    <sheet name="Cycle EOD Ventes (reel)" sheetId="3" r:id="rId3"/>
-    <sheet name="Scenario 50 traitements" sheetId="4" r:id="rId4"/>
-    <sheet name="Parite Control-M" sheetId="5" r:id="rId5"/>
+    <sheet name="Taxonomie complete" sheetId="3" r:id="rId3"/>
+    <sheet name="Cycles reels construits" sheetId="4" r:id="rId4"/>
+    <sheet name="Scenario 50 traitements" sheetId="5" r:id="rId5"/>
+    <sheet name="Parite Control-M" sheetId="6" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Objectifs par module'!$A$1:$G$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Scenario 50 traitements'!$A$3:$G$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Scenario 50 traitements'!$A$3:$G$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Taxonomie complete'!$A$3:$E$3</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,15 +44,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="349">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="572" uniqueCount="449">
   <si>
     <t>Tableau de bord des cycles operatoires - ERP_CRM_FACTORY</t>
   </si>
   <si>
-    <t>Ce classeur illustre, module par module, l'objectif metier reel poursuivi une fois un module Odoo active, et le cycle operatoire (EOD/EOM/TFJ/ON_DEMAND) qui le fait tourner en tache de fond - exactement comme le montre une session Control-M reelle (plusieurs chaines de jobs actives simultanement, chacune avec son propre calendrier).</t>
-  </si>
-  <si>
-    <t>STATUT reel (jamais survendu) : la colonne 'Statut' de la feuille 'Objectifs par module' distingue ce qui est CONSTRUIT ET VERIFIE (CRM, Ventes avec son cycle EOD complet, Achat) de ce qui reste A CONSTRUIRE sur le meme patron deja prouve. Voir docs/CONVENTION_NOMMAGE.md et docs/JOURNAL_TECHNIQUE.md dans le depot pour le detail technique complet de chaque decision.</t>
+    <t>Ce classeur illustre, module par module, l'objectif metier reel poursuivi une fois un module Odoo active, et le cycle operatoire qui le fait tourner en tache de fond - taxonomie bancaire complete (JOUR/NRT, TFJ, EOD, EOW, EOM, EOQ, EOY, CUTOFF, REPLAY, PURGE, SIMULATION, REALTIME, ON_DEMAND, voir la feuille 'Taxonomie complete'), exactement comme le montre une session Control-M reelle (plusieurs chaines de jobs actives simultanement, chacune avec son propre calendrier).</t>
+  </si>
+  <si>
+    <t>STATUT reel (jamais survendu) : la colonne 'Statut' de la feuille 'Objectifs par module' distingue ce qui est CONSTRUIT ET VERIFIE de ce qui reste A CONSTRUIRE sur le meme patron deja prouve. 5 cycles reels construits a ce jour, un par type (TFJ, EOD, CUTOFF, JOUR, PURGE) - voir la feuille 'Cycles reels construits'. Voir docs/CONVENTION_NOMMAGE.md et docs/JOURNAL_TECHNIQUE.md dans le depot pour le detail technique complet de chaque decision.</t>
   </si>
   <si>
     <t>Le moteur d'execution reel (orchestrator.sh) lance desormais tous les jobs prets d'une meme vague en parallele (MAX_PARALLEL_JOBS=6 par defaut, jamais un par un comme WAZ_ELK_FACTORY) - la feuille 'Scenario 50 traitements' simule ce comportement REEL (meme algorithme que le code, pas une illustration inventee) : environ 50 traitements reels lances, 6 demarrent simultanement, chaque emplacement se libere individuellement des qu'UN job finit.</t>
@@ -89,13 +91,13 @@
     <t>Installation et disponibilite de l'infrastructure Odoo complete</t>
   </si>
   <si>
-    <t>ON_DEMAND (deploiement)</t>
-  </si>
-  <si>
-    <t>Verification finale de bout en bout en parallele des modules</t>
-  </si>
-  <si>
-    <t>20 jobs BLD + ECFRVER (parallele)</t>
+    <t>ON_DEMAND (deploiement) + PURGE (mensuel)</t>
+  </si>
+  <si>
+    <t>Verification finale en parallele des modules - archivage a froid des fichiers arc/ &gt;90j</t>
+  </si>
+  <si>
+    <t>20 jobs BLD + ECFRVER (parallele) + ECFCPRG1 (PURGE</t>
   </si>
   <si>
     <t>CT</t>
@@ -128,582 +130,846 @@
     <t>Agenda partage et gestion des rendez-vous</t>
   </si>
   <si>
+    <t>JOUR/NRT</t>
+  </si>
+  <si>
+    <t>Envoi des rappels de rendez-vous du jour (toutes les heures)</t>
+  </si>
+  <si>
+    <t>ECFBCLAC/ECFBCLDE (activation seulement)</t>
+  </si>
+  <si>
+    <t>DS</t>
+  </si>
+  <si>
+    <t>Discuss</t>
+  </si>
+  <si>
+    <t>Messagerie interne et notifications entre utilisateurs</t>
+  </si>
+  <si>
+    <t>ON_DEMAND</t>
+  </si>
+  <si>
+    <t>Purge des messages archives anciens</t>
+  </si>
+  <si>
+    <t>ECFBDSAC/ECFBDSDE (activation seulement)</t>
+  </si>
+  <si>
+    <t>CR</t>
+  </si>
+  <si>
+    <t>CRM</t>
+  </si>
+  <si>
+    <t>Construit (Tier1 fichier)</t>
+  </si>
+  <si>
+    <t>Suivi des pistes et opportunites commerciales</t>
+  </si>
+  <si>
     <t>TFJ</t>
   </si>
   <si>
-    <t>Envoi des rappels de rendez-vous du jour</t>
-  </si>
-  <si>
-    <t>ECFBCLAC/ECFBCLDE (activation seulement)</t>
-  </si>
-  <si>
-    <t>DS</t>
-  </si>
-  <si>
-    <t>Discuss</t>
-  </si>
-  <si>
-    <t>Messagerie interne et notifications entre utilisateurs</t>
-  </si>
-  <si>
-    <t>ON_DEMAND</t>
-  </si>
-  <si>
-    <t>Purge des messages archives anciens</t>
-  </si>
-  <si>
-    <t>ECFBDSAC/ECFBDSDE (activation seulement)</t>
-  </si>
-  <si>
-    <t>CR</t>
-  </si>
-  <si>
-    <t>CRM</t>
-  </si>
-  <si>
-    <t>Construit (Tier1 fichier)</t>
-  </si>
-  <si>
-    <t>Suivi des pistes et opportunites commerciales</t>
+    <t>Relance automatique des pistes sans activite depuis 7 jours</t>
+  </si>
+  <si>
+    <t>5 jobs Tier1 (ECFRCRCL/CO/MV/WO/LO)</t>
+  </si>
+  <si>
+    <t>VT</t>
+  </si>
+  <si>
+    <t>Ventes</t>
+  </si>
+  <si>
+    <t>Construit (Tier1 + TFJ + JOUR reels)</t>
+  </si>
+  <si>
+    <t>Devis commandes et facturation client</t>
+  </si>
+  <si>
+    <t>TFJ (CONSTRUIT ET VERIFIE) + JOUR (CONSTRUIT)</t>
+  </si>
+  <si>
+    <t>TFJ : detection devis en attente (5j) - annulation devis perimes (30j) - rapport CA du jour. JOUR : suivi des devis envoyes sans reponse &gt;2h (8h-18h)</t>
+  </si>
+  <si>
+    <t>3 jobs Tier1 + cycle TFJ complet (ECFCVTRL/NT/RP) + ECFJVTSV (JOUR)</t>
+  </si>
+  <si>
+    <t>CP</t>
+  </si>
+  <si>
+    <t>Comptabilite</t>
+  </si>
+  <si>
+    <t>Construit (marqueur EOD reel)</t>
+  </si>
+  <si>
+    <t>Facturation et comptabilite de base</t>
+  </si>
+  <si>
+    <t>EOD (CONSTRUIT ET VERIFIE) + EOM</t>
+  </si>
+  <si>
+    <t>EOD : bascule quotidienne de la date valeur comptable J-&gt;J+1 (23h50). EOM (a construire) : cloture comptable mensuelle</t>
+  </si>
+  <si>
+    <t>ECFBCPAC/ECFBCPDE (activation) + ECFCEOD1 (EOD</t>
+  </si>
+  <si>
+    <t>AH</t>
+  </si>
+  <si>
+    <t>Achat</t>
+  </si>
+  <si>
+    <t>Construit (Tier1 + CUTOFF reel)</t>
+  </si>
+  <si>
+    <t>Commandes et appels d'offres fournisseurs</t>
+  </si>
+  <si>
+    <t>CUTOFF (CONSTRUIT ET VERIFIE) + EOM</t>
+  </si>
+  <si>
+    <t>CUTOFF : bascule J/J+1 des commandes fournisseurs a 15h. EOM (a construire) : reapprovisionnement mensuel base sur les seuils de stock</t>
+  </si>
+  <si>
+    <t>3 jobs Tier1 (ECFRAHPO/CF/RC) + ECFCCUT1 (CUTOFF</t>
+  </si>
+  <si>
+    <t>ST</t>
+  </si>
+  <si>
+    <t>Stock</t>
+  </si>
+  <si>
+    <t>Gestion des stocks et logistique</t>
+  </si>
+  <si>
+    <t>Alerte quotidienne des ruptures et sur-stocks</t>
+  </si>
+  <si>
+    <t>ECFBTAC/ECFBTDE (activation seulement)</t>
+  </si>
+  <si>
+    <t>MR</t>
+  </si>
+  <si>
+    <t>MRP</t>
+  </si>
+  <si>
+    <t>Ordres de fabrication et nomenclatures</t>
+  </si>
+  <si>
+    <t>Lancement des ordres de fabrication planifies (toutes les heures)</t>
+  </si>
+  <si>
+    <t>ECFBMRAC/ECFBMRDE (activation seulement)</t>
+  </si>
+  <si>
+    <t>RP</t>
+  </si>
+  <si>
+    <t>Reparation</t>
+  </si>
+  <si>
+    <t>Ordres de reparation (SAV/atelier)</t>
+  </si>
+  <si>
+    <t>Rapport quotidien des reparations en cours et terminees</t>
+  </si>
+  <si>
+    <t>ECFBRPAC/ECFBRPDE (activation seulement)</t>
+  </si>
+  <si>
+    <t>FL</t>
+  </si>
+  <si>
+    <t>Flotte vehicules</t>
+  </si>
+  <si>
+    <t>Gestion de parc de vehicules</t>
+  </si>
+  <si>
+    <t>Rapport mensuel d'entretien et de disponibilite des vehicules</t>
+  </si>
+  <si>
+    <t>ECFBFLAC/ECFBFLDE (activation seulement)</t>
+  </si>
+  <si>
+    <t>PS</t>
+  </si>
+  <si>
+    <t>Point de vente</t>
+  </si>
+  <si>
+    <t>Caisse (vente au comptoir)</t>
+  </si>
+  <si>
+    <t>Cloture de caisse quotidienne (rapprochement especes/carte)</t>
+  </si>
+  <si>
+    <t>ECFBPSAC/ECFBPSDE (activation seulement)</t>
+  </si>
+  <si>
+    <t>PR</t>
+  </si>
+  <si>
+    <t>POS Restaurant</t>
+  </si>
+  <si>
+    <t>Extensions caisse pour restauration</t>
+  </si>
+  <si>
+    <t>Cloture de service (midi/soir) avec ventilation par table</t>
+  </si>
+  <si>
+    <t>ECFBPRAC/ECFBPRDE (activation seulement)</t>
+  </si>
+  <si>
+    <t>SI</t>
+  </si>
+  <si>
+    <t>Site web</t>
+  </si>
+  <si>
+    <t>Constructeur de site web vitrine</t>
+  </si>
+  <si>
+    <t>Verification des liens morts et formulaires de contact</t>
+  </si>
+  <si>
+    <t>ECFBIAC/ECFBIDE (activation seulement)</t>
+  </si>
+  <si>
+    <t>EC</t>
+  </si>
+  <si>
+    <t>eCommerce</t>
+  </si>
+  <si>
+    <t>Boutique en ligne</t>
+  </si>
+  <si>
+    <t>Rapport quotidien des ventes en ligne et paniers abandonnes</t>
+  </si>
+  <si>
+    <t>ECFBECAC/ECFBECDE (activation seulement)</t>
+  </si>
+  <si>
+    <t>EV</t>
+  </si>
+  <si>
+    <t>Evenements</t>
+  </si>
+  <si>
+    <t>Publication et billetterie d'evenements</t>
+  </si>
+  <si>
+    <t>Rappel des evenements du jour aux inscrits</t>
+  </si>
+  <si>
+    <t>ECFBEVAC/ECFBEVDE (activation seulement)</t>
+  </si>
+  <si>
+    <t>EL</t>
+  </si>
+  <si>
+    <t>eLearning</t>
+  </si>
+  <si>
+    <t>Plateforme de formation en ligne</t>
+  </si>
+  <si>
+    <t>Rapport mensuel de progression des formations en cours</t>
+  </si>
+  <si>
+    <t>ECFBELAC/ECFBELDE (activation seulement)</t>
+  </si>
+  <si>
+    <t>JW</t>
+  </si>
+  <si>
+    <t>Offres emploi web</t>
+  </si>
+  <si>
+    <t>Offres d'emploi publiees en ligne</t>
+  </si>
+  <si>
+    <t>Depublication automatique des offres pourvues</t>
+  </si>
+  <si>
+    <t>ECFBJWAC/ECFBJWDE (activation seulement)</t>
+  </si>
+  <si>
+    <t>RH</t>
+  </si>
+  <si>
+    <t>Fiches employes</t>
+  </si>
+  <si>
+    <t>Rapport mensuel des effectifs et anciennete</t>
+  </si>
+  <si>
+    <t>ECFBRHAC/ECFBRHDE (activation seulement)</t>
+  </si>
+  <si>
+    <t>PN</t>
+  </si>
+  <si>
+    <t>Presences</t>
+  </si>
+  <si>
+    <t>Pointage des presences</t>
+  </si>
+  <si>
+    <t>Rapport quotidien des presences et anomalies (retards/absences)</t>
+  </si>
+  <si>
+    <t>ECFBPNAC/ECFBPNDE (activation seulement)</t>
+  </si>
+  <si>
+    <t>CG</t>
+  </si>
+  <si>
+    <t>Conges</t>
+  </si>
+  <si>
+    <t>Demandes de conges et absences</t>
+  </si>
+  <si>
+    <t>Relance des demandes en attente de validation (toutes les heures)</t>
+  </si>
+  <si>
+    <t>ECFBCGAC/ECFBCGDE (activation seulement)</t>
+  </si>
+  <si>
+    <t>ND</t>
+  </si>
+  <si>
+    <t>Notes de frais</t>
+  </si>
+  <si>
+    <t>Notes de frais employes</t>
+  </si>
+  <si>
+    <t>Rapport mensuel des depenses par employe et par categorie</t>
+  </si>
+  <si>
+    <t>ECFBNDAC/ECFBNDDE (activation seulement)</t>
+  </si>
+  <si>
+    <t>RC</t>
+  </si>
+  <si>
+    <t>Recrutement</t>
+  </si>
+  <si>
+    <t>Pipeline de recrutement</t>
+  </si>
+  <si>
+    <t>Relance quotidienne des candidatures en attente d'entretien</t>
+  </si>
+  <si>
+    <t>ECFBRCAC/ECFBRCDE (activation seulement)</t>
+  </si>
+  <si>
+    <t>CM</t>
+  </si>
+  <si>
+    <t>Competences</t>
+  </si>
+  <si>
+    <t>Competences et CV des employes</t>
+  </si>
+  <si>
+    <t>Rapport mensuel des ecarts de competences par equipe</t>
+  </si>
+  <si>
+    <t>ECFBCMAC/ECFBCMDE (activation seulement)</t>
+  </si>
+  <si>
+    <t>PJ</t>
+  </si>
+  <si>
+    <t>Projets</t>
+  </si>
+  <si>
+    <t>Gestion de projets</t>
+  </si>
+  <si>
+    <t>Rapport quotidien d'avancement des taches et jalons en retard</t>
+  </si>
+  <si>
+    <t>ECFBPJAC/ECFBPJDE (activation seulement)</t>
+  </si>
+  <si>
+    <t>TD</t>
+  </si>
+  <si>
+    <t>Todo</t>
+  </si>
+  <si>
+    <t>Listes de taches personnelles</t>
+  </si>
+  <si>
+    <t>Rappel des taches du jour non terminees (toutes les heures)</t>
+  </si>
+  <si>
+    <t>ECFBTDAC/ECFBTDDE (activation seulement)</t>
+  </si>
+  <si>
+    <t>MT</t>
+  </si>
+  <si>
+    <t>Maintenance</t>
+  </si>
+  <si>
+    <t>Suivi de maintenance des equipements</t>
+  </si>
+  <si>
+    <t>Planning de maintenance preventive du mois suivant</t>
+  </si>
+  <si>
+    <t>ECFBMTAC/ECFBMTDE (activation seulement)</t>
+  </si>
+  <si>
+    <t>SN</t>
+  </si>
+  <si>
+    <t>Sondages</t>
+  </si>
+  <si>
+    <t>Creation et diffusion de sondages</t>
+  </si>
+  <si>
+    <t>Cloture automatique des sondages arrives a echeance</t>
+  </si>
+  <si>
+    <t>ECFBNAC/ECFBNDE (activation seulement)</t>
+  </si>
+  <si>
+    <t>CN</t>
+  </si>
+  <si>
+    <t>Cantine</t>
+  </si>
+  <si>
+    <t>Commandes de repas internes</t>
+  </si>
+  <si>
+    <t>CUTOFF</t>
+  </si>
+  <si>
+    <t>Cutoff des commandes du jour (11h) avant envoi cuisine</t>
+  </si>
+  <si>
+    <t>ECFBCNAC/ECFBCNDE (activation seulement)</t>
+  </si>
+  <si>
+    <t>LC</t>
+  </si>
+  <si>
+    <t>Live chat</t>
+  </si>
+  <si>
+    <t>Chat en direct sur le site web</t>
+  </si>
+  <si>
+    <t>Rapport hebdomadaire (EOW) des conversations non traitees</t>
+  </si>
+  <si>
+    <t>ECFBLCAC/ECFBLCDE (activation seulement)</t>
+  </si>
+  <si>
+    <t>EM</t>
+  </si>
+  <si>
+    <t>Email marketing</t>
+  </si>
+  <si>
+    <t>Campagnes email marketing</t>
+  </si>
+  <si>
+    <t>Envoi des campagnes planifiees (toutes les heures)</t>
+  </si>
+  <si>
+    <t>ECFBEMAC/ECFBEMDE (activation seulement)</t>
+  </si>
+  <si>
+    <t>SM</t>
+  </si>
+  <si>
+    <t>SMS marketing</t>
+  </si>
+  <si>
+    <t>Campagnes SMS marketing</t>
+  </si>
+  <si>
+    <t>Envoi des campagnes SMS planifiees (toutes les heures)</t>
+  </si>
+  <si>
+    <t>ECFBMAC/ECFBMDE (activation seulement)</t>
+  </si>
+  <si>
+    <t>CK</t>
+  </si>
+  <si>
+    <t>Cartes marketing</t>
+  </si>
+  <si>
+    <t>Cartes marketing dynamiques partageables</t>
+  </si>
+  <si>
+    <t>Rapport de partage/engagement des cartes actives</t>
+  </si>
+  <si>
+    <t>ECFBCKAC/ECFBCKDE (activation seulement)</t>
+  </si>
+  <si>
+    <t>RY</t>
+  </si>
+  <si>
+    <t>Recyclage donnees</t>
+  </si>
+  <si>
+    <t>Detection et archivage des donnees perimees</t>
+  </si>
+  <si>
+    <t>Detection mensuelle des donnees perimees (distinct du PURGE systeme deja construit)</t>
+  </si>
+  <si>
+    <t>ECFBRYAC/ECFBRYDE (activation seulement)</t>
+  </si>
+  <si>
+    <t>Taxonomie complete des cycles operatoires (vocabulaire bancaire reel - CBS Amplitude/SAB/Temenos)</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Nature du declenchement</t>
+  </si>
+  <si>
+    <t>Frequence</t>
+  </si>
+  <si>
+    <t>Cas d'usage</t>
+  </si>
+  <si>
+    <t>Statut chez ECF</t>
+  </si>
+  <si>
+    <t>JOUR / NRT</t>
+  </si>
+  <si>
+    <t>Automatique frequence fixe (ex. toutes les heures) ou micro-batch 5-15 min</t>
+  </si>
+  <si>
+    <t>Quotidienne pendant les heures ouvrees</t>
+  </si>
+  <si>
+    <t>Synchronisations d'interfaces sauvegardes a chaud alertes temps reel</t>
+  </si>
+  <si>
+    <t>CONSTRUIT (ECFJVTSV</t>
+  </si>
+  <si>
+    <t>Automatique a la fermeture (guichets/agences)</t>
+  </si>
+  <si>
+    <t>Quotidienne fenetre nocturne</t>
+  </si>
+  <si>
+    <t>Chaine d'orchestration de fin de journee : gel transactions reconciliations soldes</t>
+  </si>
+  <si>
+    <t>CONSTRUIT (ECFCVTRL/NT/RP</t>
   </si>
   <si>
     <t>EOD</t>
   </si>
   <si>
-    <t>Relance automatique des pistes sans activite depuis 7 jours</t>
-  </si>
-  <si>
-    <t>5 jobs Tier1 (ECFRCRCL/CO/MV/WO/LO)</t>
-  </si>
-  <si>
-    <t>VT</t>
-  </si>
-  <si>
-    <t>Ventes</t>
-  </si>
-  <si>
-    <t>Construit (Tier1 + cycle EOD reel)</t>
-  </si>
-  <si>
-    <t>Devis commandes et facturation client</t>
-  </si>
-  <si>
-    <t>EOD (CONSTRUIT ET VERIFIE)</t>
-  </si>
-  <si>
-    <t>Detection devis en attente (5j) - annulation devis perimes (30j) - rapport CA du jour</t>
-  </si>
-  <si>
-    <t>3 jobs Tier1 + cycle EOD complet (ECFCVTRL/NT/RP)</t>
-  </si>
-  <si>
-    <t>CP</t>
-  </si>
-  <si>
-    <t>Comptabilite</t>
-  </si>
-  <si>
-    <t>Facturation et comptabilite de base</t>
-  </si>
-  <si>
-    <t>EOM + TFJ</t>
-  </si>
-  <si>
-    <t>Cloture comptable mensuelle - relance quotidienne des factures impayees &gt;30j</t>
-  </si>
-  <si>
-    <t>ECFBCPAC/ECFBCPDE (activation seulement)</t>
-  </si>
-  <si>
-    <t>AH</t>
-  </si>
-  <si>
-    <t>Achat</t>
-  </si>
-  <si>
-    <t>Commandes et appels d'offres fournisseurs</t>
-  </si>
-  <si>
-    <t>Reapprovisionnement automatique base sur les seuils de stock minimum</t>
-  </si>
-  <si>
-    <t>3 jobs Tier1 (ECFRAHPO/CF/RC)</t>
-  </si>
-  <si>
-    <t>ST</t>
-  </si>
-  <si>
-    <t>Stock</t>
-  </si>
-  <si>
-    <t>Gestion des stocks et logistique</t>
-  </si>
-  <si>
-    <t>Alerte quotidienne des ruptures et sur-stocks</t>
-  </si>
-  <si>
-    <t>ECFBTAC/ECFBTDE (activation seulement)</t>
-  </si>
-  <si>
-    <t>MR</t>
-  </si>
-  <si>
-    <t>MRP</t>
-  </si>
-  <si>
-    <t>Ordres de fabrication et nomenclatures</t>
-  </si>
-  <si>
-    <t>Lancement des ordres de fabrication planifies du jour</t>
-  </si>
-  <si>
-    <t>ECFBMRAC/ECFBMRDE (activation seulement)</t>
-  </si>
-  <si>
-    <t>RP</t>
-  </si>
-  <si>
-    <t>Reparation</t>
-  </si>
-  <si>
-    <t>Ordres de reparation (SAV/atelier)</t>
-  </si>
-  <si>
-    <t>Rapport quotidien des reparations en cours et terminees</t>
-  </si>
-  <si>
-    <t>ECFBRPAC/ECFBRPDE (activation seulement)</t>
-  </si>
-  <si>
-    <t>FL</t>
-  </si>
-  <si>
-    <t>Flotte vehicules</t>
-  </si>
-  <si>
-    <t>Gestion de parc de vehicules</t>
-  </si>
-  <si>
-    <t>Rapport mensuel d'entretien et de disponibilite des vehicules</t>
-  </si>
-  <si>
-    <t>ECFBFLAC/ECFBFLDE (activation seulement)</t>
-  </si>
-  <si>
-    <t>PS</t>
-  </si>
-  <si>
-    <t>Point de vente</t>
-  </si>
-  <si>
-    <t>Caisse (vente au comptoir)</t>
-  </si>
-  <si>
-    <t>Cloture de caisse quotidienne (rapprochement especes/carte)</t>
-  </si>
-  <si>
-    <t>ECFBPSAC/ECFBPSDE (activation seulement)</t>
-  </si>
-  <si>
-    <t>PR</t>
-  </si>
-  <si>
-    <t>POS Restaurant</t>
-  </si>
-  <si>
-    <t>Extensions caisse pour restauration</t>
-  </si>
-  <si>
-    <t>Cloture de service (midi/soir) avec ventilation par table</t>
-  </si>
-  <si>
-    <t>ECFBPRAC/ECFBPRDE (activation seulement)</t>
-  </si>
-  <si>
-    <t>SI</t>
-  </si>
-  <si>
-    <t>Site web</t>
-  </si>
-  <si>
-    <t>Constructeur de site web vitrine</t>
-  </si>
-  <si>
-    <t>Verification des liens morts et formulaires de contact</t>
-  </si>
-  <si>
-    <t>ECFBIAC/ECFBIDE (activation seulement)</t>
-  </si>
-  <si>
-    <t>EC</t>
-  </si>
-  <si>
-    <t>eCommerce</t>
-  </si>
-  <si>
-    <t>Boutique en ligne</t>
-  </si>
-  <si>
-    <t>Rapport quotidien des ventes en ligne et paniers abandonnes</t>
-  </si>
-  <si>
-    <t>ECFBECAC/ECFBECDE (activation seulement)</t>
-  </si>
-  <si>
-    <t>EV</t>
-  </si>
-  <si>
-    <t>Evenements</t>
-  </si>
-  <si>
-    <t>Publication et billetterie d'evenements</t>
-  </si>
-  <si>
-    <t>Rappel des evenements du jour aux inscrits</t>
-  </si>
-  <si>
-    <t>ECFBEVAC/ECFBEVDE (activation seulement)</t>
-  </si>
-  <si>
-    <t>EL</t>
-  </si>
-  <si>
-    <t>eLearning</t>
-  </si>
-  <si>
-    <t>Plateforme de formation en ligne</t>
-  </si>
-  <si>
-    <t>Rapport mensuel de progression des formations en cours</t>
-  </si>
-  <si>
-    <t>ECFBELAC/ECFBELDE (activation seulement)</t>
-  </si>
-  <si>
-    <t>JW</t>
-  </si>
-  <si>
-    <t>Offres emploi web</t>
-  </si>
-  <si>
-    <t>Offres d'emploi publiees en ligne</t>
-  </si>
-  <si>
-    <t>Depublication automatique des offres pourvues</t>
-  </si>
-  <si>
-    <t>ECFBJWAC/ECFBJWDE (activation seulement)</t>
-  </si>
-  <si>
-    <t>RH</t>
-  </si>
-  <si>
-    <t>Fiches employes</t>
-  </si>
-  <si>
-    <t>Rapport mensuel des effectifs et anciennete</t>
-  </si>
-  <si>
-    <t>ECFBRHAC/ECFBRHDE (activation seulement)</t>
-  </si>
-  <si>
-    <t>PN</t>
-  </si>
-  <si>
-    <t>Presences</t>
-  </si>
-  <si>
-    <t>Pointage des presences</t>
-  </si>
-  <si>
-    <t>Rapport quotidien des presences et anomalies (retards/absences)</t>
-  </si>
-  <si>
-    <t>ECFBPNAC/ECFBPNDE (activation seulement)</t>
-  </si>
-  <si>
-    <t>CG</t>
-  </si>
-  <si>
-    <t>Conges</t>
-  </si>
-  <si>
-    <t>Demandes de conges et absences</t>
-  </si>
-  <si>
-    <t>Relance quotidienne des demandes en attente de validation</t>
-  </si>
-  <si>
-    <t>ECFBCGAC/ECFBCGDE (activation seulement)</t>
-  </si>
-  <si>
-    <t>ND</t>
-  </si>
-  <si>
-    <t>Notes de frais</t>
-  </si>
-  <si>
-    <t>Notes de frais employes</t>
-  </si>
-  <si>
-    <t>Rapport mensuel des depenses par employe et par categorie</t>
-  </si>
-  <si>
-    <t>ECFBNDAC/ECFBNDDE (activation seulement)</t>
-  </si>
-  <si>
-    <t>RC</t>
-  </si>
-  <si>
-    <t>Recrutement</t>
-  </si>
-  <si>
-    <t>Pipeline de recrutement</t>
-  </si>
-  <si>
-    <t>Relance quotidienne des candidatures en attente d'entretien</t>
-  </si>
-  <si>
-    <t>ECFBRCAC/ECFBRCDE (activation seulement)</t>
-  </si>
-  <si>
-    <t>CM</t>
-  </si>
-  <si>
-    <t>Competences</t>
-  </si>
-  <si>
-    <t>Competences et CV des employes</t>
-  </si>
-  <si>
-    <t>Rapport mensuel des ecarts de competences par equipe</t>
-  </si>
-  <si>
-    <t>ECFBCMAC/ECFBCMDE (activation seulement)</t>
-  </si>
-  <si>
-    <t>PJ</t>
-  </si>
-  <si>
-    <t>Projets</t>
-  </si>
-  <si>
-    <t>Gestion de projets</t>
-  </si>
-  <si>
-    <t>Rapport quotidien d'avancement des taches et jalons en retard</t>
-  </si>
-  <si>
-    <t>ECFBPJAC/ECFBPJDE (activation seulement)</t>
-  </si>
-  <si>
-    <t>TD</t>
-  </si>
-  <si>
-    <t>Todo</t>
-  </si>
-  <si>
-    <t>Listes de taches personnelles</t>
-  </si>
-  <si>
-    <t>Rappel des taches du jour non terminees</t>
-  </si>
-  <si>
-    <t>ECFBTDAC/ECFBTDDE (activation seulement)</t>
-  </si>
-  <si>
-    <t>MT</t>
-  </si>
-  <si>
-    <t>Maintenance</t>
-  </si>
-  <si>
-    <t>Suivi de maintenance des equipements</t>
-  </si>
-  <si>
-    <t>Planning de maintenance preventive du mois suivant</t>
-  </si>
-  <si>
-    <t>ECFBMTAC/ECFBMTDE (activation seulement)</t>
-  </si>
-  <si>
-    <t>SN</t>
-  </si>
-  <si>
-    <t>Sondages</t>
-  </si>
-  <si>
-    <t>Creation et diffusion de sondages</t>
-  </si>
-  <si>
-    <t>Cloture automatique des sondages arrives a echeance</t>
-  </si>
-  <si>
-    <t>ECFBNAC/ECFBNDE (activation seulement)</t>
-  </si>
-  <si>
-    <t>CN</t>
-  </si>
-  <si>
-    <t>Cantine</t>
-  </si>
-  <si>
-    <t>Commandes de repas internes</t>
-  </si>
-  <si>
-    <t>Cloture des commandes du jour avant envoi cuisine</t>
-  </si>
-  <si>
-    <t>ECFBCNAC/ECFBCNDE (activation seulement)</t>
-  </si>
-  <si>
-    <t>LC</t>
-  </si>
-  <si>
-    <t>Live chat</t>
-  </si>
-  <si>
-    <t>Chat en direct sur le site web</t>
-  </si>
-  <si>
-    <t>Rapport hebdomadaire des conversations non traitees</t>
-  </si>
-  <si>
-    <t>ECFBLCAC/ECFBLCDE (activation seulement)</t>
-  </si>
-  <si>
-    <t>EM</t>
-  </si>
-  <si>
-    <t>Email marketing</t>
-  </si>
-  <si>
-    <t>Campagnes email marketing</t>
-  </si>
-  <si>
-    <t>Envoi des campagnes planifiees du jour</t>
-  </si>
-  <si>
-    <t>ECFBEMAC/ECFBEMDE (activation seulement)</t>
-  </si>
-  <si>
-    <t>SM</t>
-  </si>
-  <si>
-    <t>SMS marketing</t>
-  </si>
-  <si>
-    <t>Campagnes SMS marketing</t>
-  </si>
-  <si>
-    <t>Envoi des campagnes SMS planifiees du jour</t>
-  </si>
-  <si>
-    <t>ECFBMAC/ECFBMDE (activation seulement)</t>
-  </si>
-  <si>
-    <t>CK</t>
-  </si>
-  <si>
-    <t>Cartes marketing</t>
-  </si>
-  <si>
-    <t>Cartes marketing dynamiques partageables</t>
-  </si>
-  <si>
-    <t>Rapport de partage/engagement des cartes actives</t>
-  </si>
-  <si>
-    <t>ECFBCKAC/ECFBCKDE (activation seulement)</t>
-  </si>
-  <si>
-    <t>RY</t>
-  </si>
-  <si>
-    <t>Recyclage donnees</t>
-  </si>
-  <si>
-    <t>Detection et archivage des donnees perimees</t>
-  </si>
-  <si>
-    <t>Purge mensuelle des donnees perimees detectees</t>
-  </si>
-  <si>
-    <t>ECFBRYAC/ECFBRYDE (activation seulement)</t>
-  </si>
-  <si>
-    <t>Cycle EOD Ventes - seul cycle calendaire CONSTRUIT ET VERIFIE a ce jour</t>
+    <t>Horodate (ex. 23h50)</t>
+  </si>
+  <si>
+    <t>Quotidienne</t>
+  </si>
+  <si>
+    <t>Marqueur logique unique - bascule de la date valeur comptable de J a J+1</t>
+  </si>
+  <si>
+    <t>CONSTRUIT (ECFCEOD1</t>
+  </si>
+  <si>
+    <t>EOW</t>
+  </si>
+  <si>
+    <t>Automatique (vendredi soir/samedi)</t>
+  </si>
+  <si>
+    <t>Hebdomadaire</t>
+  </si>
+  <si>
+    <t>Positions moyennes consolidation des risques hebdomadaires</t>
+  </si>
+  <si>
+    <t>MECANISME PRET (WEEKLY) - aucun exemple construit</t>
+  </si>
+  <si>
+    <t>Calendaire (dernier jour du mois)</t>
+  </si>
+  <si>
+    <t>Mensuelle</t>
+  </si>
+  <si>
+    <t>Paies amortissements arretes comptables rapports reglementaires</t>
+  </si>
+  <si>
+    <t>MECANISME PRET (MONTHLY) - aucun exemple construit</t>
+  </si>
+  <si>
+    <t>EOQ</t>
+  </si>
+  <si>
+    <t>Automatique (fin de trimestre)</t>
+  </si>
+  <si>
+    <t>Trimestrielle</t>
+  </si>
+  <si>
+    <t>Ratios prudentiels reporting reglementaire</t>
+  </si>
+  <si>
+    <t>MECANISME PRET (QUARTERLY) - aucun exemple construit</t>
+  </si>
+  <si>
+    <t>EOY</t>
+  </si>
+  <si>
+    <t>Automatique (31 decembre)</t>
+  </si>
+  <si>
+    <t>Annuelle</t>
+  </si>
+  <si>
+    <t>Bascule d'exercice comptable amortissements annuels etats fiscaux</t>
+  </si>
+  <si>
+    <t>MECANISME PRET (YEARLY) - aucun exemple construit</t>
+  </si>
+  <si>
+    <t>Horaire legal strict (ex. 15h)</t>
+  </si>
+  <si>
+    <t>Heure limite de prise en compte des ordres - bascule automatique en J+1 apres</t>
+  </si>
+  <si>
+    <t>CONSTRUIT (ECFCCUT1</t>
+  </si>
+  <si>
+    <t>REPLAY</t>
+  </si>
+  <si>
+    <t>Exceptionnel manuel ou incident</t>
+  </si>
+  <si>
+    <t>Ponctuelle</t>
+  </si>
+  <si>
+    <t>Rejeu d'une chaine en erreur apres correction d'un bug</t>
+  </si>
+  <si>
+    <t>DEJA COUVERT (bin/rerun_job.sh bin/order_job.sh)</t>
+  </si>
+  <si>
+    <t>PURGE</t>
+  </si>
+  <si>
+    <t>Periodique (depassement de retention)</t>
+  </si>
+  <si>
+    <t>Periodique</t>
+  </si>
+  <si>
+    <t>Nettoyage de tables temporaires archivage a froid</t>
+  </si>
+  <si>
+    <t>CONSTRUIT (ECFCPRG1</t>
+  </si>
+  <si>
+    <t>SIMULATION</t>
+  </si>
+  <si>
+    <t>Sur environnement miroir/sandbox</t>
+  </si>
+  <si>
+    <t>Stress test impact d'une hypothese sur le portefeuille</t>
+  </si>
+  <si>
+    <t>HORS PERIMETRE - necessite un environnement dedie</t>
+  </si>
+  <si>
+    <t>REALTIME</t>
+  </si>
+  <si>
+    <t>Continu evenementiel (Kafka webhooks)</t>
+  </si>
+  <si>
+    <t>Fil de l'eau</t>
+  </si>
+  <si>
+    <t>Anti-fraude transaction autorisation immediate</t>
+  </si>
+  <si>
+    <t>HORS PERIMETRE - architecture evenementielle incompatible avec un ordonnanceur batch</t>
+  </si>
+  <si>
+    <t>Manuel (operateur) ou webhook/API</t>
+  </si>
+  <si>
+    <t>Reexecution d'un batch en erreur export specifique pour audit</t>
+  </si>
+  <si>
+    <t>DEJA COUVERT (jobs Tier1 pilotes par fichier + bin/run_now.sh)</t>
+  </si>
+  <si>
+    <t>5 cycles reels construits et verifies a ce jour - un par type de mecanisme</t>
+  </si>
+  <si>
+    <t>JOB_ID</t>
+  </si>
+  <si>
+    <t>Nom</t>
+  </si>
+  <si>
+    <t>Role</t>
+  </si>
+  <si>
+    <t>Detail</t>
+  </si>
+  <si>
+    <t>TFJ (0/3)</t>
+  </si>
+  <si>
+    <t>bin/montee_au_plan.sh</t>
+  </si>
+  <si>
+    <t>Montee au plan (New Day)</t>
+  </si>
+  <si>
+    <t>Ouvre la fenetre chaque nuit (00:05)</t>
+  </si>
+  <si>
+    <t>TFJ_VENTES_WINDOW_OPEN</t>
+  </si>
+  <si>
+    <t>TFJ (1/3)</t>
+  </si>
+  <si>
+    <t>ECFCVTRL</t>
+  </si>
+  <si>
+    <t>ECF_VENTE_CYC_RELANCE</t>
+  </si>
+  <si>
+    <t>Detecte les devis en attente depuis plus de 5 jours</t>
+  </si>
+  <si>
+    <t>TFJ_VENTES_RELANCE_OK</t>
+  </si>
+  <si>
+    <t>TFJ (2/3)</t>
+  </si>
+  <si>
+    <t>ECFCVTNT</t>
+  </si>
+  <si>
+    <t>ECF_VENTE_CYC_NETTOYAGE</t>
+  </si>
+  <si>
+    <t>Annule automatiquement les devis perimes depuis plus de 30 jours</t>
+  </si>
+  <si>
+    <t>TFJ_VENTES_NETTOYAGE_OK</t>
+  </si>
+  <si>
+    <t>TFJ (3/3)</t>
+  </si>
+  <si>
+    <t>ECFCVTRP</t>
+  </si>
+  <si>
+    <t>ECF_VENTE_CYC_RAPPORT</t>
+  </si>
+  <si>
+    <t>JOB TERMINAL - rapport de fin de journee (commandes et CA du jour)</t>
+  </si>
+  <si>
+    <t>TFJ_VENTES_TERMINE</t>
+  </si>
+  <si>
+    <t>ECFCEOD1</t>
+  </si>
+  <si>
+    <t>ECF_COMPTA_EOD_BASCULE</t>
+  </si>
+  <si>
+    <t>Marqueur horodate (23h50, minuteur dedie) - bascule la date valeur comptable J-&gt;J+1</t>
+  </si>
+  <si>
+    <t>state/valeur_comptable_courante.txt</t>
+  </si>
+  <si>
+    <t>ECFCCUT1</t>
+  </si>
+  <si>
+    <t>ECF_ACHAT_CUTOFF_ORDRES</t>
+  </si>
+  <si>
+    <t>Marqueur horodate (15h) - fixe J ou J+1 pour les futures commandes fournisseurs</t>
+  </si>
+  <si>
+    <t>state/cutoff_achat_date_valeur.txt</t>
+  </si>
+  <si>
+    <t>ECFJVTSV</t>
+  </si>
+  <si>
+    <t>ECF_VENTE_JOUR_SUIVI</t>
+  </si>
+  <si>
+    <t>Suivi intraday des devis envoyes sans reponse &gt;2h (garde horaire 8h-18h)</t>
+  </si>
+  <si>
+    <t>OUT_COND=NONE, invoque toutes les 15 min</t>
+  </si>
+  <si>
+    <t>ECFCPRG1</t>
+  </si>
+  <si>
+    <t>ECF_SYS_CYC_PURGE</t>
+  </si>
+  <si>
+    <t>Archivage a froid des fichiers arc/ de plus de 90 jours (cadence mensuelle)</t>
+  </si>
+  <si>
+    <t>PURGE_ARC_TERMINE</t>
+  </si>
+  <si>
+    <t>TFJ/EOM/EOW/EOQ/EOY partagent le meme mecanisme (bin/montee_au_plan.sh, CYCLE_WINDOWS, un jalon reel remis a zero par periode). EOD/CUTOFF suivent un patron different : un marqueur horodate unique, son propre minuteur systemd a heure fixe, jamais celui de montee_au_plan.sh. JOUR/NRT n'a besoin d'aucun minuteur dedie : un job Tier 1 classique (OUT_COND=NONE) avec sa propre garde horaire interne, invoque par le minuteur periodique de l'orchestrateur (15 min).</t>
+  </si>
+  <si>
+    <t>Simulation reelle : ~50 traitements sous MAX_PARALLEL_JOBS=6 (meme algorithme que orchestrator.sh)</t>
   </si>
   <si>
     <t>Ordre</t>
   </si>
   <si>
-    <t>JOB_ID</t>
-  </si>
-  <si>
-    <t>Nom</t>
-  </si>
-  <si>
-    <t>Role</t>
-  </si>
-  <si>
-    <t>Sortie produite</t>
-  </si>
-  <si>
-    <t>bin/montee_au_plan.sh</t>
-  </si>
-  <si>
-    <t>Montee au plan (New Day)</t>
-  </si>
-  <si>
-    <t>Ouvre la fenetre du jour (00:05, quotidien)</t>
-  </si>
-  <si>
-    <t>EOD_VENTES_WINDOW_OPEN</t>
-  </si>
-  <si>
-    <t>ECFCVTRL</t>
-  </si>
-  <si>
-    <t>ECF_VENTE_CYC_RELANCE</t>
-  </si>
-  <si>
-    <t>Detecte les devis en attente depuis plus de 5 jours, ecrit un rapport dans /vt/snd</t>
-  </si>
-  <si>
-    <t>EOD_VENTES_RELANCE_OK</t>
-  </si>
-  <si>
-    <t>ECFCVTNT</t>
-  </si>
-  <si>
-    <t>ECF_VENTE_CYC_NETTOYAGE</t>
-  </si>
-  <si>
-    <t>Annule automatiquement les devis perimes depuis plus de 30 jours</t>
-  </si>
-  <si>
-    <t>EOD_VENTES_NETTOYAGE_OK</t>
-  </si>
-  <si>
-    <t>ECFCVTRP</t>
-  </si>
-  <si>
-    <t>ECF_VENTE_CYC_RAPPORT</t>
-  </si>
-  <si>
-    <t>JOB TERMINAL - rapport de fin de journee (commandes et CA du jour)</t>
-  </si>
-  <si>
-    <t>EOD_VENTES_TERMINE</t>
-  </si>
-  <si>
-    <t>Le lendemain, bin/montee_au_plan.sh archive EOD_VENTES_TERMINE (state/plan/history/), l'efface, et rouvre EOD_VENTES_WINDOW_OPEN - la chaine redevient eligible, sans intervention humaine.</t>
-  </si>
-  <si>
-    <t>Simulation reelle : ~50 traitements sous MAX_PARALLEL_JOBS=6 (meme algorithme que orchestrator.sh)</t>
-  </si>
-  <si>
     <t>Service</t>
   </si>
   <si>
@@ -1061,10 +1327,46 @@
     <t>CONSTRUIT - state/history/&lt;JOB_ID&gt;/, bin/view_history.sh</t>
   </si>
   <si>
-    <t>Calendrier (jobs EOD/EOM/TFJ auto-declenches)</t>
-  </si>
-  <si>
-    <t>CONSTRUIT - bin/montee_au_plan.sh, 1 cycle reel (Ventes EOD), 30+ modules restants sur le meme patron</t>
+    <t>Calendrier TFJ/EOM/EOW/EOQ/EOY (chaines auto-declenchees)</t>
+  </si>
+  <si>
+    <t>CONSTRUIT - bin/montee_au_plan.sh (5 cadences), 1 cycle TFJ + 1 cycle PURGE reels</t>
+  </si>
+  <si>
+    <t>EOD/CUTOFF (marqueur horodate, heure fixe)</t>
+  </si>
+  <si>
+    <t>CONSTRUIT - ECFCEOD1 (Comptabilite, 23h50) et ECFCCUT1 (Achat, 15h)</t>
+  </si>
+  <si>
+    <t>JOUR/NRT (intraday, garde horaire interne)</t>
+  </si>
+  <si>
+    <t>CONSTRUIT - ECFJVTSV (Ventes)</t>
+  </si>
+  <si>
+    <t>REPLAY (rejeu apres incident)</t>
+  </si>
+  <si>
+    <t>DEJA COUVERT - bin/rerun_job.sh / bin/order_job.sh</t>
+  </si>
+  <si>
+    <t>PURGE (archivage a froid periodique)</t>
+  </si>
+  <si>
+    <t>CONSTRUIT - ECFCPRG1</t>
+  </si>
+  <si>
+    <t>SIMULATION (stress test sur miroir)</t>
+  </si>
+  <si>
+    <t>A CONSTRUIRE - necessite un environnement miroir/sandbox dedie</t>
+  </si>
+  <si>
+    <t>REALTIME (evenementiel, Kafka/webhooks)</t>
+  </si>
+  <si>
+    <t>HORS PERIMETRE - architecture evenementielle incompatible avec un ordonnanceur batch bash/CSV</t>
   </si>
   <si>
     <t>Montee au plan / New Day (snapshot quotidien)</t>
@@ -1130,7 +1432,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1149,6 +1451,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEEEDF0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC0C0C0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -1162,7 +1476,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1173,6 +1487,14 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1501,7 +1823,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40EA069E-C37E-4E35-9D07-E3E8FDB1E4FC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C44B503F-E54F-48F8-B3E8-05AE9262FFDB}">
   <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1527,14 +1849,14 @@
       <c r="F2" s="1"/>
     </row>
     <row r="3" spans="1:6" ht="55.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="12"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="12"/>
+      <c r="B3" s="16"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="16"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
@@ -1545,12 +1867,12 @@
       <c r="F4" s="1"/>
     </row>
     <row r="5" spans="1:6" ht="55.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="12"/>
-      <c r="B5" s="12"/>
-      <c r="C5" s="12"/>
-      <c r="D5" s="12"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="12"/>
+      <c r="A5" s="16"/>
+      <c r="B5" s="16"/>
+      <c r="C5" s="16"/>
+      <c r="D5" s="16"/>
+      <c r="E5" s="16"/>
+      <c r="F5" s="16"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
@@ -1561,14 +1883,14 @@
       <c r="F6" s="1"/>
     </row>
     <row r="7" spans="1:6" ht="55.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="12"/>
-      <c r="C7" s="12"/>
-      <c r="D7" s="12"/>
-      <c r="E7" s="12"/>
-      <c r="F7" s="12"/>
+      <c r="B7" s="16"/>
+      <c r="C7" s="16"/>
+      <c r="D7" s="16"/>
+      <c r="E7" s="16"/>
+      <c r="F7" s="16"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -1579,12 +1901,12 @@
       <c r="F8" s="1"/>
     </row>
     <row r="9" spans="1:6" ht="55.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="12"/>
-      <c r="B9" s="12"/>
-      <c r="C9" s="12"/>
-      <c r="D9" s="12"/>
-      <c r="E9" s="12"/>
-      <c r="F9" s="12"/>
+      <c r="A9" s="16"/>
+      <c r="B9" s="16"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="16"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
@@ -1595,14 +1917,14 @@
       <c r="F10" s="1"/>
     </row>
     <row r="11" spans="1:6" ht="55.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="12" t="s">
+      <c r="A11" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="B11" s="12"/>
-      <c r="C11" s="12"/>
-      <c r="D11" s="12"/>
-      <c r="E11" s="12"/>
-      <c r="F11" s="12"/>
+      <c r="B11" s="16"/>
+      <c r="C11" s="16"/>
+      <c r="D11" s="16"/>
+      <c r="E11" s="16"/>
+      <c r="F11" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -1618,17 +1940,17 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37157928-76FF-4E37-BD23-CB91E81F6830}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDE1AE77-44A1-469E-A35D-801DD77B2B4C}">
   <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.77734375" customWidth="1"/>
     <col min="2" max="2" width="18.77734375" customWidth="1"/>
-    <col min="3" max="3" width="20.77734375" customWidth="1"/>
+    <col min="3" max="3" width="24.77734375" customWidth="1"/>
     <col min="4" max="4" width="45.77734375" customWidth="1"/>
-    <col min="5" max="5" width="16.77734375" customWidth="1"/>
-    <col min="6" max="6" width="45.77734375" customWidth="1"/>
-    <col min="7" max="7" width="35.77734375" customWidth="1"/>
+    <col min="5" max="5" width="22.77734375" customWidth="1"/>
+    <col min="6" max="6" width="55.77734375" customWidth="1"/>
+    <col min="7" max="7" width="40.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
@@ -1654,7 +1976,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="79.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="106.2" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>11</v>
       </c>
@@ -1700,7 +2022,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="53.4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" ht="79.8" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>25</v>
       </c>
@@ -1769,7 +2091,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="27" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" ht="40.200000000000003" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>44</v>
       </c>
@@ -1793,698 +2115,698 @@
       </c>
     </row>
     <row r="8" spans="1:7" ht="27" x14ac:dyDescent="0.3">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C8" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="D8" s="7" t="s">
+      <c r="C8" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="D8" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="E8" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="G8" s="7" t="s">
+      <c r="F8" s="6" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" ht="27" x14ac:dyDescent="0.3">
+      <c r="G8" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="40.200000000000003" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>22</v>
+        <v>62</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="27" x14ac:dyDescent="0.3">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>20</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E10" s="7" t="s">
         <v>41</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="27" x14ac:dyDescent="0.3">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>20</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E11" s="7" t="s">
         <v>28</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="27" x14ac:dyDescent="0.3">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>20</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="E12" s="7" t="s">
         <v>41</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="27" x14ac:dyDescent="0.3">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>20</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E13" s="7" t="s">
         <v>22</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="27" x14ac:dyDescent="0.3">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>20</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="E14" s="7" t="s">
         <v>41</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="27" x14ac:dyDescent="0.3">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="C15" s="5" t="s">
         <v>20</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="E15" s="7" t="s">
         <v>41</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="27" x14ac:dyDescent="0.3">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="C16" s="5" t="s">
         <v>20</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E16" s="7" t="s">
         <v>34</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="27" x14ac:dyDescent="0.3">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="C17" s="5" t="s">
         <v>20</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="E17" s="7" t="s">
         <v>41</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="27" x14ac:dyDescent="0.3">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="C18" s="5" t="s">
         <v>20</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E18" s="7" t="s">
         <v>28</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" ht="27" x14ac:dyDescent="0.3">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="C19" s="5" t="s">
         <v>20</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="E19" s="7" t="s">
         <v>22</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="27" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="C20" s="5" t="s">
         <v>20</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="E20" s="7" t="s">
         <v>34</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" ht="27" x14ac:dyDescent="0.3">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="C21" s="5" t="s">
         <v>20</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="E21" s="7" t="s">
         <v>22</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="G21" s="7" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" ht="27" x14ac:dyDescent="0.3">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="C22" s="5" t="s">
         <v>20</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="E22" s="7" t="s">
         <v>41</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="G22" s="7" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" ht="27" x14ac:dyDescent="0.3">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="C23" s="5" t="s">
         <v>20</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="E23" s="7" t="s">
         <v>28</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="G23" s="7" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" ht="27" x14ac:dyDescent="0.3">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="5" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="C24" s="5" t="s">
         <v>20</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="E24" s="7" t="s">
         <v>22</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="G24" s="7" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" ht="27" x14ac:dyDescent="0.3">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="C25" s="5" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="E25" s="7" t="s">
         <v>41</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" ht="27" x14ac:dyDescent="0.3">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="C26" s="5" t="s">
         <v>20</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="E26" s="7" t="s">
         <v>22</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="G26" s="7" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" ht="27" x14ac:dyDescent="0.3">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="C27" s="5" t="s">
         <v>20</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="E27" s="7" t="s">
         <v>41</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="G27" s="7" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" ht="27" x14ac:dyDescent="0.3">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="C28" s="5" t="s">
         <v>20</v>
       </c>
       <c r="D28" s="7" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="E28" s="7" t="s">
         <v>28</v>
       </c>
       <c r="F28" s="7" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="G28" s="7" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" ht="27" x14ac:dyDescent="0.3">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" s="5" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="C29" s="5" t="s">
         <v>20</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="E29" s="7" t="s">
         <v>22</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="G29" s="7" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" ht="27" x14ac:dyDescent="0.3">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" s="5" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="C30" s="5" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="7" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="E30" s="7" t="s">
         <v>34</v>
       </c>
       <c r="F30" s="7" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="G30" s="7" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" ht="27" x14ac:dyDescent="0.3">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" s="5" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="C31" s="5" t="s">
         <v>20</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="E31" s="7" t="s">
-        <v>28</v>
+        <v>172</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="G31" s="7" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" ht="27" x14ac:dyDescent="0.3">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" s="5" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="C32" s="5" t="s">
         <v>20</v>
       </c>
       <c r="D32" s="7" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="E32" s="7" t="s">
         <v>34</v>
       </c>
       <c r="F32" s="7" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="G32" s="7" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" ht="27" x14ac:dyDescent="0.3">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" s="5" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="C33" s="5" t="s">
         <v>20</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="E33" s="7" t="s">
         <v>28</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="G33" s="7" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" ht="27" x14ac:dyDescent="0.3">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" s="5" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="C34" s="5" t="s">
         <v>20</v>
       </c>
       <c r="D34" s="7" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="E34" s="7" t="s">
         <v>28</v>
       </c>
       <c r="F34" s="7" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="G34" s="7" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" ht="27" x14ac:dyDescent="0.3">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" s="5" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="C35" s="5" t="s">
         <v>20</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="E35" s="7" t="s">
         <v>34</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="G35" s="7" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="27" x14ac:dyDescent="0.3">
       <c r="A36" s="5" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="C36" s="5" t="s">
         <v>20</v>
       </c>
       <c r="D36" s="7" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="E36" s="7" t="s">
         <v>22</v>
       </c>
       <c r="F36" s="7" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="G36" s="7" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G1" xr:uid="{37157928-76FF-4E37-BD23-CB91E81F6830}"/>
+  <autoFilter ref="A1:G1" xr:uid="{FDE1AE77-44A1-469E-A35D-801DD77B2B4C}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB3D4F7A-4BAB-468D-BC40-D440E658C2C9}">
-  <dimension ref="A1:E9"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0DE62E72-034C-49A6-8154-6E7EB4598AA7}">
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.77734375" customWidth="1"/>
-    <col min="2" max="2" width="20.77734375" customWidth="1"/>
-    <col min="3" max="3" width="26.77734375" customWidth="1"/>
-    <col min="4" max="4" width="55.77734375" customWidth="1"/>
-    <col min="5" max="5" width="24.77734375" customWidth="1"/>
+    <col min="1" max="1" width="14.77734375" customWidth="1"/>
+    <col min="2" max="2" width="40.77734375" customWidth="1"/>
+    <col min="3" max="3" width="22.77734375" customWidth="1"/>
+    <col min="4" max="4" width="45.77734375" customWidth="1"/>
+    <col min="5" max="5" width="40.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A1" s="9" t="s">
-        <v>196</v>
-      </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
+      <c r="A1" s="13" t="s">
+        <v>200</v>
+      </c>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="5"/>
@@ -2494,117 +2816,460 @@
       <c r="E2" s="5"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="8" t="s">
-        <v>197</v>
-      </c>
-      <c r="B3" s="8" t="s">
-        <v>198</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>199</v>
-      </c>
-      <c r="D3" s="8" t="s">
-        <v>200</v>
-      </c>
-      <c r="E3" s="8" t="s">
+      <c r="A3" s="3" t="s">
         <v>201</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" ht="27" x14ac:dyDescent="0.3">
-      <c r="A4" s="7">
-        <v>0</v>
-      </c>
-      <c r="B4" s="7" t="s">
+      <c r="B3" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C3" s="3" t="s">
         <v>203</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D3" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E3" s="3" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="27" x14ac:dyDescent="0.3">
-      <c r="A5" s="7">
-        <v>1</v>
-      </c>
-      <c r="B5" s="7" t="s">
+    <row r="4" spans="1:5" ht="93" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
         <v>206</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="B4" s="6" t="s">
         <v>207</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="C4" s="6" t="s">
         <v>208</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="D4" s="6" t="s">
         <v>209</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" ht="27" x14ac:dyDescent="0.3">
-      <c r="A6" s="7">
-        <v>2</v>
-      </c>
-      <c r="B6" s="7" t="s">
+      <c r="E4" s="6" t="s">
         <v>210</v>
       </c>
-      <c r="C6" s="7" t="s">
+    </row>
+    <row r="5" spans="1:5" ht="93" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B5" s="6" t="s">
         <v>211</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="C5" s="6" t="s">
         <v>212</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="D5" s="6" t="s">
         <v>213</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" ht="27" x14ac:dyDescent="0.3">
-      <c r="A7" s="7">
-        <v>3</v>
+      <c r="E5" s="6" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="106.2" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>216</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>217</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>218</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="79.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="5" t="s">
+        <v>220</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>214</v>
+        <v>221</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>216</v>
+        <v>223</v>
       </c>
       <c r="E7" s="7" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="27" x14ac:dyDescent="0.3">
+      <c r="A8" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>225</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>226</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>227</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="27" x14ac:dyDescent="0.3">
+      <c r="A9" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>230</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="27" x14ac:dyDescent="0.3">
+      <c r="A10" s="5" t="s">
+        <v>234</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>235</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>236</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="27" x14ac:dyDescent="0.3">
+      <c r="A11" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="C11" s="6" t="s">
         <v>217</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="5"/>
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
-    </row>
-    <row r="9" spans="1:5" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="11" t="s">
-        <v>218</v>
-      </c>
-      <c r="B9" s="11"/>
-      <c r="C9" s="11"/>
-      <c r="D9" s="11"/>
-      <c r="E9" s="11"/>
+      <c r="D11" s="6" t="s">
+        <v>240</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="27" x14ac:dyDescent="0.3">
+      <c r="A12" s="8" t="s">
+        <v>242</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>243</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>244</v>
+      </c>
+      <c r="D12" s="10" t="s">
+        <v>245</v>
+      </c>
+      <c r="E12" s="10" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>248</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>249</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>250</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="27" x14ac:dyDescent="0.3">
+      <c r="A14" s="9" t="s">
+        <v>252</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>253</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>244</v>
+      </c>
+      <c r="D14" s="11" t="s">
+        <v>254</v>
+      </c>
+      <c r="E14" s="11" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="40.200000000000003" x14ac:dyDescent="0.3">
+      <c r="A15" s="9" t="s">
+        <v>256</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>257</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>258</v>
+      </c>
+      <c r="D15" s="11" t="s">
+        <v>259</v>
+      </c>
+      <c r="E15" s="11" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="27" x14ac:dyDescent="0.3">
+      <c r="A16" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B16" s="10" t="s">
+        <v>261</v>
+      </c>
+      <c r="C16" s="10" t="s">
+        <v>244</v>
+      </c>
+      <c r="D16" s="10" t="s">
+        <v>262</v>
+      </c>
+      <c r="E16" s="10" t="s">
+        <v>263</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <autoFilter ref="A3:E3" xr:uid="{0DE62E72-034C-49A6-8154-6E7EB4598AA7}"/>
+  <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A9:E9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C4400B9-DF3B-4693-9AF8-03147BAE59A2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FFCD391-2710-44F2-9FB7-551D10D1FEFA}">
+  <dimension ref="A1:E13"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="12.77734375" customWidth="1"/>
+    <col min="2" max="2" width="20.77734375" customWidth="1"/>
+    <col min="3" max="3" width="26.77734375" customWidth="1"/>
+    <col min="4" max="4" width="55.77734375" customWidth="1"/>
+    <col min="5" max="5" width="30.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="13" t="s">
+        <v>264</v>
+      </c>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="5"/>
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="12" t="s">
+        <v>201</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>265</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>266</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>267</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="7" t="s">
+        <v>269</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>270</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>271</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>272</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="7" t="s">
+        <v>274</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>275</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>277</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="27" x14ac:dyDescent="0.3">
+      <c r="A6" s="7" t="s">
+        <v>279</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>282</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="27" x14ac:dyDescent="0.3">
+      <c r="A7" s="7" t="s">
+        <v>284</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>285</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>286</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>287</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="27" x14ac:dyDescent="0.3">
+      <c r="A8" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>289</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>290</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>291</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="27" x14ac:dyDescent="0.3">
+      <c r="A9" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>293</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>294</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>295</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="27" x14ac:dyDescent="0.3">
+      <c r="A10" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>297</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>298</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>299</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="27" x14ac:dyDescent="0.3">
+      <c r="A11" s="7" t="s">
+        <v>247</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>301</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>302</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>303</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="5"/>
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+    </row>
+    <row r="13" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="15" t="s">
+        <v>305</v>
+      </c>
+      <c r="B13" s="15"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="15"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A13:E13"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{520B399C-294A-4A60-8313-782D6DB2BE13}">
   <dimension ref="A1:G56"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -2618,15 +3283,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="9" t="s">
-        <v>219</v>
-      </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
+      <c r="A1" s="13" t="s">
+        <v>306</v>
+      </c>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="5"/>
@@ -2639,25 +3304,25 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>197</v>
+        <v>307</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>198</v>
+        <v>265</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>220</v>
+        <v>308</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>221</v>
+        <v>309</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>222</v>
+        <v>310</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>223</v>
+        <v>311</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>224</v>
+        <v>312</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="53.4" x14ac:dyDescent="0.3">
@@ -2665,13 +3330,13 @@
         <v>1</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>225</v>
+        <v>313</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>37</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>226</v>
+        <v>314</v>
       </c>
       <c r="E4" s="4">
         <v>45</v>
@@ -2688,13 +3353,13 @@
         <v>2</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>227</v>
+        <v>315</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>37</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>228</v>
+        <v>316</v>
       </c>
       <c r="E5" s="4">
         <v>20</v>
@@ -2711,13 +3376,13 @@
         <v>3</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>229</v>
+        <v>317</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>44</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>230</v>
+        <v>318</v>
       </c>
       <c r="E6" s="4">
         <v>30</v>
@@ -2734,13 +3399,13 @@
         <v>4</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>231</v>
+        <v>319</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>44</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>232</v>
+        <v>320</v>
       </c>
       <c r="E7" s="4">
         <v>25</v>
@@ -2757,13 +3422,13 @@
         <v>5</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>233</v>
+        <v>321</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>44</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>234</v>
+        <v>322</v>
       </c>
       <c r="E8" s="4">
         <v>40</v>
@@ -2780,13 +3445,13 @@
         <v>6</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>206</v>
+        <v>275</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>44</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>235</v>
+        <v>323</v>
       </c>
       <c r="E9" s="4">
         <v>35</v>
@@ -2803,13 +3468,13 @@
         <v>7</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>210</v>
+        <v>280</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>44</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>236</v>
+        <v>324</v>
       </c>
       <c r="E10" s="5">
         <v>20</v>
@@ -2826,13 +3491,13 @@
         <v>8</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>214</v>
+        <v>285</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>44</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>237</v>
+        <v>325</v>
       </c>
       <c r="E11" s="5">
         <v>15</v>
@@ -2849,13 +3514,13 @@
         <v>9</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>238</v>
+        <v>326</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>239</v>
+        <v>327</v>
       </c>
       <c r="E12" s="5">
         <v>30</v>
@@ -2872,13 +3537,13 @@
         <v>10</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>240</v>
+        <v>328</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>241</v>
+        <v>329</v>
       </c>
       <c r="E13" s="5">
         <v>20</v>
@@ -2895,13 +3560,13 @@
         <v>11</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>242</v>
+        <v>330</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>243</v>
+        <v>331</v>
       </c>
       <c r="E14" s="5">
         <v>50</v>
@@ -2918,13 +3583,13 @@
         <v>12</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>244</v>
+        <v>332</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>245</v>
+        <v>333</v>
       </c>
       <c r="E15" s="5">
         <v>25</v>
@@ -2941,13 +3606,13 @@
         <v>13</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>246</v>
+        <v>334</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>247</v>
+        <v>335</v>
       </c>
       <c r="E16" s="5">
         <v>60</v>
@@ -2964,13 +3629,13 @@
         <v>14</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>248</v>
+        <v>336</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>249</v>
+        <v>337</v>
       </c>
       <c r="E17" s="5">
         <v>90</v>
@@ -2987,13 +3652,13 @@
         <v>15</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>250</v>
+        <v>338</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>251</v>
+        <v>339</v>
       </c>
       <c r="E18" s="5">
         <v>20</v>
@@ -3010,13 +3675,13 @@
         <v>16</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>252</v>
+        <v>340</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>253</v>
+        <v>341</v>
       </c>
       <c r="E19" s="5">
         <v>35</v>
@@ -3033,13 +3698,13 @@
         <v>17</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>254</v>
+        <v>342</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>255</v>
+        <v>343</v>
       </c>
       <c r="E20" s="5">
         <v>15</v>
@@ -3056,13 +3721,13 @@
         <v>18</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>256</v>
+        <v>344</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>257</v>
+        <v>345</v>
       </c>
       <c r="E21" s="5">
         <v>20</v>
@@ -3079,13 +3744,13 @@
         <v>19</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>258</v>
+        <v>346</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>259</v>
+        <v>347</v>
       </c>
       <c r="E22" s="5">
         <v>30</v>
@@ -3102,13 +3767,13 @@
         <v>20</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>260</v>
+        <v>348</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>261</v>
+        <v>349</v>
       </c>
       <c r="E23" s="5">
         <v>10</v>
@@ -3125,13 +3790,13 @@
         <v>21</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>262</v>
+        <v>350</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>263</v>
+        <v>351</v>
       </c>
       <c r="E24" s="5">
         <v>40</v>
@@ -3148,13 +3813,13 @@
         <v>22</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>264</v>
+        <v>352</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>265</v>
+        <v>353</v>
       </c>
       <c r="E25" s="5">
         <v>25</v>
@@ -3171,13 +3836,13 @@
         <v>23</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>266</v>
+        <v>354</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>267</v>
+        <v>355</v>
       </c>
       <c r="E26" s="5">
         <v>20</v>
@@ -3194,13 +3859,13 @@
         <v>24</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>268</v>
+        <v>356</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>269</v>
+        <v>357</v>
       </c>
       <c r="E27" s="5">
         <v>15</v>
@@ -3217,13 +3882,13 @@
         <v>25</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>270</v>
+        <v>358</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="D28" s="7" t="s">
-        <v>271</v>
+        <v>359</v>
       </c>
       <c r="E28" s="5">
         <v>30</v>
@@ -3240,13 +3905,13 @@
         <v>26</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>272</v>
+        <v>360</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>273</v>
+        <v>361</v>
       </c>
       <c r="E29" s="5">
         <v>20</v>
@@ -3263,13 +3928,13 @@
         <v>27</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>274</v>
+        <v>362</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="D30" s="7" t="s">
-        <v>275</v>
+        <v>363</v>
       </c>
       <c r="E30" s="5">
         <v>35</v>
@@ -3286,13 +3951,13 @@
         <v>28</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>276</v>
+        <v>364</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>277</v>
+        <v>365</v>
       </c>
       <c r="E31" s="5">
         <v>45</v>
@@ -3309,13 +3974,13 @@
         <v>29</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>278</v>
+        <v>366</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="D32" s="7" t="s">
-        <v>279</v>
+        <v>367</v>
       </c>
       <c r="E32" s="5">
         <v>10</v>
@@ -3332,13 +3997,13 @@
         <v>30</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>280</v>
+        <v>368</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>281</v>
+        <v>369</v>
       </c>
       <c r="E33" s="5">
         <v>30</v>
@@ -3355,13 +4020,13 @@
         <v>31</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>282</v>
+        <v>370</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="D34" s="7" t="s">
-        <v>283</v>
+        <v>371</v>
       </c>
       <c r="E34" s="5">
         <v>15</v>
@@ -3378,13 +4043,13 @@
         <v>32</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>284</v>
+        <v>372</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>285</v>
+        <v>373</v>
       </c>
       <c r="E35" s="5">
         <v>10</v>
@@ -3401,13 +4066,13 @@
         <v>33</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>286</v>
+        <v>374</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="D36" s="7" t="s">
-        <v>287</v>
+        <v>375</v>
       </c>
       <c r="E36" s="5">
         <v>20</v>
@@ -3424,13 +4089,13 @@
         <v>34</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>288</v>
+        <v>376</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="D37" s="7" t="s">
-        <v>289</v>
+        <v>377</v>
       </c>
       <c r="E37" s="5">
         <v>60</v>
@@ -3447,13 +4112,13 @@
         <v>35</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>290</v>
+        <v>378</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="D38" s="7" t="s">
-        <v>291</v>
+        <v>379</v>
       </c>
       <c r="E38" s="5">
         <v>30</v>
@@ -3470,13 +4135,13 @@
         <v>36</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>292</v>
+        <v>380</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="D39" s="7" t="s">
-        <v>293</v>
+        <v>381</v>
       </c>
       <c r="E39" s="5">
         <v>15</v>
@@ -3493,13 +4158,13 @@
         <v>37</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>294</v>
+        <v>382</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="D40" s="7" t="s">
-        <v>295</v>
+        <v>383</v>
       </c>
       <c r="E40" s="5">
         <v>50</v>
@@ -3516,13 +4181,13 @@
         <v>38</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>296</v>
+        <v>384</v>
       </c>
       <c r="C41" s="5" t="s">
         <v>18</v>
       </c>
       <c r="D41" s="7" t="s">
-        <v>297</v>
+        <v>385</v>
       </c>
       <c r="E41" s="5">
         <v>40</v>
@@ -3539,13 +4204,13 @@
         <v>39</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>298</v>
+        <v>386</v>
       </c>
       <c r="C42" s="5" t="s">
         <v>25</v>
       </c>
       <c r="D42" s="7" t="s">
-        <v>299</v>
+        <v>387</v>
       </c>
       <c r="E42" s="5">
         <v>10</v>
@@ -3562,13 +4227,13 @@
         <v>40</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>300</v>
+        <v>388</v>
       </c>
       <c r="C43" s="5" t="s">
         <v>31</v>
       </c>
       <c r="D43" s="7" t="s">
-        <v>301</v>
+        <v>389</v>
       </c>
       <c r="E43" s="5">
         <v>20</v>
@@ -3585,13 +4250,13 @@
         <v>41</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>302</v>
+        <v>390</v>
       </c>
       <c r="C44" s="5" t="s">
         <v>51</v>
       </c>
       <c r="D44" s="7" t="s">
-        <v>303</v>
+        <v>391</v>
       </c>
       <c r="E44" s="5">
         <v>35</v>
@@ -3608,13 +4273,13 @@
         <v>42</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>304</v>
+        <v>392</v>
       </c>
       <c r="C45" s="5" t="s">
         <v>51</v>
       </c>
       <c r="D45" s="7" t="s">
-        <v>305</v>
+        <v>393</v>
       </c>
       <c r="E45" s="5">
         <v>120</v>
@@ -3631,13 +4296,13 @@
         <v>43</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>306</v>
+        <v>394</v>
       </c>
       <c r="C46" s="5" t="s">
         <v>37</v>
       </c>
       <c r="D46" s="7" t="s">
-        <v>307</v>
+        <v>395</v>
       </c>
       <c r="E46" s="5">
         <v>15</v>
@@ -3654,13 +4319,13 @@
         <v>44</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>308</v>
+        <v>396</v>
       </c>
       <c r="C47" s="5" t="s">
         <v>37</v>
       </c>
       <c r="D47" s="7" t="s">
-        <v>309</v>
+        <v>397</v>
       </c>
       <c r="E47" s="5">
         <v>10</v>
@@ -3677,13 +4342,13 @@
         <v>45</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>310</v>
+        <v>398</v>
       </c>
       <c r="C48" s="5" t="s">
         <v>37</v>
       </c>
       <c r="D48" s="7" t="s">
-        <v>311</v>
+        <v>399</v>
       </c>
       <c r="E48" s="5">
         <v>10</v>
@@ -3700,13 +4365,13 @@
         <v>46</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>312</v>
+        <v>400</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D49" s="7" t="s">
-        <v>313</v>
+        <v>401</v>
       </c>
       <c r="E49" s="5">
         <v>25</v>
@@ -3723,13 +4388,13 @@
         <v>47</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>314</v>
+        <v>402</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="D50" s="7" t="s">
-        <v>315</v>
+        <v>403</v>
       </c>
       <c r="E50" s="5">
         <v>10</v>
@@ -3746,13 +4411,13 @@
         <v>48</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>316</v>
+        <v>404</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="D51" s="7" t="s">
-        <v>317</v>
+        <v>405</v>
       </c>
       <c r="E51" s="5">
         <v>20</v>
@@ -3769,13 +4434,13 @@
         <v>49</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>318</v>
+        <v>406</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="D52" s="7" t="s">
-        <v>319</v>
+        <v>407</v>
       </c>
       <c r="E52" s="5">
         <v>35</v>
@@ -3792,13 +4457,13 @@
         <v>50</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>320</v>
+        <v>408</v>
       </c>
       <c r="C53" s="5" t="s">
         <v>44</v>
       </c>
       <c r="D53" s="7" t="s">
-        <v>321</v>
+        <v>409</v>
       </c>
       <c r="E53" s="5">
         <v>45</v>
@@ -3815,13 +4480,13 @@
         <v>51</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>322</v>
+        <v>410</v>
       </c>
       <c r="C54" s="5" t="s">
         <v>37</v>
       </c>
       <c r="D54" s="7" t="s">
-        <v>323</v>
+        <v>411</v>
       </c>
       <c r="E54" s="5">
         <v>30</v>
@@ -3834,18 +4499,18 @@
       </c>
     </row>
     <row r="56" spans="1:7" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="10" t="s">
-        <v>324</v>
-      </c>
-      <c r="B56" s="10"/>
-      <c r="C56" s="10"/>
-      <c r="D56" s="10"/>
-      <c r="E56" s="10"/>
-      <c r="F56" s="10"/>
-      <c r="G56" s="10"/>
+      <c r="A56" s="14" t="s">
+        <v>412</v>
+      </c>
+      <c r="B56" s="14"/>
+      <c r="C56" s="14"/>
+      <c r="D56" s="14"/>
+      <c r="E56" s="14"/>
+      <c r="F56" s="14"/>
+      <c r="G56" s="14"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:G3" xr:uid="{5C4400B9-DF3B-4693-9AF8-03147BAE59A2}"/>
+  <autoFilter ref="A3:G3" xr:uid="{520B399C-294A-4A60-8313-782D6DB2BE13}"/>
   <mergeCells count="2">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A56:G56"/>
@@ -3854,109 +4519,157 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2779DD9-7244-4588-8575-FB9548F3D43C}">
-  <dimension ref="A1:B12"/>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1A2ADCF-A946-4A47-B45D-055F07B86754}">
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="45.77734375" customWidth="1"/>
-    <col min="2" max="2" width="70.77734375" customWidth="1"/>
+    <col min="1" max="1" width="48.77734375" customWidth="1"/>
+    <col min="2" max="2" width="75.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>325</v>
+        <v>413</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>326</v>
+        <v>414</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="93" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>327</v>
+        <v>415</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>328</v>
+        <v>416</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="79.8" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>329</v>
+        <v>417</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>330</v>
+        <v>418</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="93" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
-        <v>331</v>
+        <v>419</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>332</v>
+        <v>420</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="93" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>333</v>
+        <v>421</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>334</v>
+        <v>422</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>335</v>
+        <v>423</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>336</v>
+        <v>424</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
-        <v>337</v>
+        <v>425</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>338</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="27" x14ac:dyDescent="0.3">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
-        <v>339</v>
+        <v>427</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>340</v>
+        <v>428</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>341</v>
+        <v>429</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>342</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="27" x14ac:dyDescent="0.3">
-      <c r="A10" s="5" t="s">
-        <v>343</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>344</v>
+        <v>430</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>432</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A11" s="5" t="s">
-        <v>345</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>346</v>
+      <c r="A11" s="4" t="s">
+        <v>433</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>434</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A12" s="5" t="s">
-        <v>347</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>348</v>
+      <c r="A12" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" s="5" t="s">
+        <v>437</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="27" x14ac:dyDescent="0.3">
+      <c r="A14" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" s="4" t="s">
+        <v>441</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="27" x14ac:dyDescent="0.3">
+      <c r="A16" s="5" t="s">
+        <v>443</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" s="5" t="s">
+        <v>445</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" s="5" t="s">
+        <v>447</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>448</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Met a jour le catalogue des operations : 5 operations passees de A CONSTRUIRE a CONSTRUIT
Reflete le lot de jobs metier construit dans cbe5038 (cycle TFJ
Comptabilite, EOM Comptabilite+Ventes, EOQ) - chaque ligne pointe
maintenant vers le vrai JOB_ID et precise honnetement le perimetre
reellement couvert par la version simplifiee construite (ex: EOM
Comptabilite sans provisions ni verrouillage de periode). 8 operations
HAUTE priorite restantes (22 CONSTRUIT au total desormais, contre 17).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/TABLEAU_DE_BORD_CYCLES_OPERATOIRES.xlsx
+++ b/docs/TABLEAU_DE_BORD_CYCLES_OPERATOIRES.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP PROBOOK\Documents\ECF\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8138107C-9D87-4E9C-8B29-C49E44750E9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{91A7DED7-92AE-444D-9247-EB5D370DAB08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2472" yWindow="2472" windowWidth="17280" windowHeight="8880" xr2:uid="{C551928C-355D-43F7-977C-D22A6F84B241}"/>
+    <workbookView xWindow="2472" yWindow="2472" windowWidth="17280" windowHeight="8880" xr2:uid="{1C8EC45E-BD1F-45DD-8D0B-DA7242E61BEC}"/>
   </bookViews>
   <sheets>
     <sheet name="Vue d'ensemble" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1100" uniqueCount="560">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1104" uniqueCount="564">
   <si>
     <t>Tableau de bord des cycles operatoires - ERP_CRM_FACTORY</t>
   </si>
@@ -928,6 +928,9 @@
     <t>Lineaire (consolidation - calcul commissions - validation - verrouillage - rapport)</t>
   </si>
   <si>
+    <t>ECFCVTEM1 deja construit (version simplifiee : CA et repartition par commercial - sans verrouillage de periode)</t>
+  </si>
+  <si>
     <t>Cloture quotidienne TFJ Ventes (doit avoir tourne chaque jour du mois)</t>
   </si>
   <si>
@@ -961,6 +964,9 @@
     <t>Lineaire (import releve - rapprochement auto - exceptions - validation - rapport)</t>
   </si>
   <si>
+    <t>ECFCCPRB1 deja construit (detection des lignes non rapprochees - pas encore l'import automatique du releve lui-meme)</t>
+  </si>
+  <si>
     <t>Relance factures impayees</t>
   </si>
   <si>
@@ -970,6 +976,9 @@
     <t>Lineaire (detection - relance)</t>
   </si>
   <si>
+    <t>ECFCCPFI1 deja construit (detection et rapport - relance email non automatisee - meme choix que ECFCVTRL cote Ventes)</t>
+  </si>
+  <si>
     <t>Generation de releves de compte PDF volumineux</t>
   </si>
   <si>
@@ -1009,7 +1018,7 @@
     <t>Lineaire (verif soldes - lettrage auto - provisions - balance - validation - verrouillage periode - export - notification - archivage)</t>
   </si>
   <si>
-    <t>Chaine lourde representative d'une vraie cloture bancaire</t>
+    <t>ECFCCPEM1 deja construit (version simplifiee : CA facture/encaisse/balance agee - sans provisions ni verrouillage de periode)</t>
   </si>
   <si>
     <t>Reconciliation bancaire quotidienne + Marqueur EOD (chaque jour du mois)</t>
@@ -1024,6 +1033,9 @@
     <t>Lineaire (extraction - calcul ratios - validation - generation etat - controle - transmission)</t>
   </si>
   <si>
+    <t>ECFCCPEQ1 deja construit (TVA collectee/deductible/nette simplifiee - pas encore les ratios prudentiels)</t>
+  </si>
+  <si>
     <t>Cloture comptable mensuelle (les 3 mois du trimestre)</t>
   </si>
   <si>
@@ -1525,7 +1537,7 @@
     <t>Distinct du PURGE systeme global (ECFCPRG1) - specifique au module data_recycle</t>
   </si>
   <si>
-    <t>TOTAL : 88 operations reelles cataloguees, 233 jobs estimes au total (lineaires + paralleles cumules) - 17 operations deja CONSTRUITES ET VERIFIEES (vert), 13 en PRIORITE HAUTE a construire ensuite (jaune - operations quotidiennes/critiques des modules coeur), le reste sur le meme patron deja prouve. Ces chiffres sont des estimations architecturales raisonnees (jamais un decompte de jobs reellement ecrits pour les operations encore A CONSTRUIRE). Priorite : HAUTE = necessaire des le premier cycle d'exploitation reel (quotidien/critique sur un module coeur) - MOYENNE = utile mais differable - BASSE = illustratif/complementaire. Colonne 'Depend de' : chaine de dependance metier reelle (pas une IN_COND technique) - l'operation en amont qui doit exister avant que celle-ci ait un sens operationnel.</t>
+    <t>TOTAL : 88 operations reelles cataloguees, 233 jobs estimes au total (lineaires + paralleles cumules) - 22 operations deja CONSTRUITES ET VERIFIEES (vert), 8 en PRIORITE HAUTE a construire ensuite (jaune - operations quotidiennes/critiques des modules coeur), le reste sur le meme patron deja prouve. Ces chiffres sont des estimations architecturales raisonnees (jamais un decompte de jobs reellement ecrits pour les operations encore A CONSTRUIRE). Priorite : HAUTE = necessaire des le premier cycle d'exploitation reel (quotidien/critique sur un module coeur) - MOYENNE = utile mais differable - BASSE = illustratif/complementaire. Colonne 'Depend de' : chaine de dependance metier reelle (pas une IN_COND technique) - l'operation en amont qui doit exister avant que celle-ci ait un sens operationnel.</t>
   </si>
   <si>
     <t>Maintien en condition operationnelle - preuves d'efficacite reelles</t>
@@ -1588,7 +1600,7 @@
     <t>Couverture du catalogue d'operations</t>
   </si>
   <si>
-    <t>17 des 88 operations cataloguees deja construites</t>
+    <t>22 des 88 operations cataloguees deja construites</t>
   </si>
   <si>
     <t>233 jobs estimes au total sur l'ensemble du catalogue si tout etait construit - roadmap explicite, jamais presente comme deja fait.</t>
@@ -2082,14 +2094,14 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>17</c:v>
+                  <c:v>22</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-2CC8-4026-803E-2CEC4622D482}"/>
+              <c16:uniqueId val="{00000000-0DA8-451D-8A19-4D353F89230A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2195,14 +2207,14 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>69</c:v>
+                  <c:v>64</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-2CC8-4026-803E-2CEC4622D482}"/>
+              <c16:uniqueId val="{00000002-0DA8-451D-8A19-4D353F89230A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2315,7 +2327,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-2CC8-4026-803E-2CEC4622D482}"/>
+              <c16:uniqueId val="{00000003-0DA8-451D-8A19-4D353F89230A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2992,7 +3004,7 @@
         <xdr:cNvPr id="2" name="Graphique 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B91864DB-0385-4353-B721-EC56A4533CA5}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D8CB4A2C-0ACF-4293-980B-DB6D33F055DD}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3309,7 +3321,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82667C35-C0E1-4D6B-B224-A5207098906E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49005E43-6F93-4C86-A4CE-3B9E95856FFA}">
   <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -3498,7 +3510,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66D78C55-1DD8-4428-80B7-D978393E723A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDE00EBB-670F-4983-9E58-B2E3B1026B64}">
   <dimension ref="A1:K93"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -4541,36 +4553,38 @@
       </c>
     </row>
     <row r="32" spans="1:11" ht="159" x14ac:dyDescent="0.3">
-      <c r="A32" s="22" t="s">
+      <c r="A32" s="11" t="s">
         <v>278</v>
       </c>
-      <c r="B32" s="22" t="s">
+      <c r="B32" s="11" t="s">
         <v>130</v>
       </c>
-      <c r="C32" s="23" t="s">
+      <c r="C32" s="14" t="s">
         <v>291</v>
       </c>
-      <c r="D32" s="23" t="s">
+      <c r="D32" s="14" t="s">
         <v>292</v>
       </c>
-      <c r="E32" s="23" t="s">
+      <c r="E32" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="F32" s="23">
+      <c r="F32" s="14">
         <v>5</v>
       </c>
-      <c r="G32" s="23" t="s">
+      <c r="G32" s="14" t="s">
         <v>293</v>
       </c>
-      <c r="H32" s="23" t="s">
-        <v>204</v>
-      </c>
-      <c r="I32" s="23" t="s">
-        <v>270</v>
-      </c>
-      <c r="J32" s="23"/>
-      <c r="K32" s="23" t="s">
+      <c r="H32" s="14" t="s">
+        <v>189</v>
+      </c>
+      <c r="I32" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="J32" s="14" t="s">
         <v>294</v>
+      </c>
+      <c r="K32" s="14" t="s">
+        <v>295</v>
       </c>
     </row>
     <row r="33" spans="1:11" ht="119.4" x14ac:dyDescent="0.3">
@@ -4581,10 +4595,10 @@
         <v>130</v>
       </c>
       <c r="C33" s="15" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D33" s="15" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E33" s="15" t="s">
         <v>37</v>
@@ -4603,21 +4617,21 @@
       </c>
       <c r="J33" s="15"/>
       <c r="K33" s="15" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
     </row>
     <row r="34" spans="1:11" ht="159" x14ac:dyDescent="0.3">
       <c r="A34" s="11" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B34" s="11" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C34" s="14" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="D34" s="14" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="E34" s="14" t="s">
         <v>22</v>
@@ -4641,93 +4655,97 @@
         <v>192</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="145.80000000000001" x14ac:dyDescent="0.3">
-      <c r="A35" s="22" t="s">
-        <v>298</v>
-      </c>
-      <c r="B35" s="22" t="s">
+    <row r="35" spans="1:11" ht="159" x14ac:dyDescent="0.3">
+      <c r="A35" s="11" t="s">
         <v>299</v>
       </c>
-      <c r="C35" s="23" t="s">
-        <v>302</v>
-      </c>
-      <c r="D35" s="23" t="s">
+      <c r="B35" s="11" t="s">
+        <v>300</v>
+      </c>
+      <c r="C35" s="14" t="s">
         <v>303</v>
       </c>
-      <c r="E35" s="23" t="s">
+      <c r="D35" s="14" t="s">
+        <v>304</v>
+      </c>
+      <c r="E35" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="F35" s="23">
+      <c r="F35" s="14">
         <v>5</v>
       </c>
-      <c r="G35" s="23" t="s">
-        <v>304</v>
-      </c>
-      <c r="H35" s="23" t="s">
-        <v>204</v>
-      </c>
-      <c r="I35" s="23" t="s">
-        <v>270</v>
-      </c>
-      <c r="J35" s="23"/>
-      <c r="K35" s="23" t="s">
+      <c r="G35" s="14" t="s">
+        <v>305</v>
+      </c>
+      <c r="H35" s="14" t="s">
+        <v>189</v>
+      </c>
+      <c r="I35" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="J35" s="14" t="s">
+        <v>306</v>
+      </c>
+      <c r="K35" s="14" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="93" x14ac:dyDescent="0.3">
-      <c r="A36" s="22" t="s">
-        <v>298</v>
-      </c>
-      <c r="B36" s="22" t="s">
+    <row r="36" spans="1:11" ht="159" x14ac:dyDescent="0.3">
+      <c r="A36" s="11" t="s">
         <v>299</v>
       </c>
-      <c r="C36" s="23" t="s">
-        <v>305</v>
-      </c>
-      <c r="D36" s="23" t="s">
-        <v>306</v>
-      </c>
-      <c r="E36" s="23" t="s">
+      <c r="B36" s="11" t="s">
+        <v>300</v>
+      </c>
+      <c r="C36" s="14" t="s">
+        <v>307</v>
+      </c>
+      <c r="D36" s="14" t="s">
+        <v>308</v>
+      </c>
+      <c r="E36" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="F36" s="23">
+      <c r="F36" s="14">
         <v>2</v>
       </c>
-      <c r="G36" s="23" t="s">
-        <v>307</v>
-      </c>
-      <c r="H36" s="23" t="s">
-        <v>204</v>
-      </c>
-      <c r="I36" s="23" t="s">
-        <v>270</v>
-      </c>
-      <c r="J36" s="23"/>
-      <c r="K36" s="23" t="s">
+      <c r="G36" s="14" t="s">
+        <v>309</v>
+      </c>
+      <c r="H36" s="14" t="s">
+        <v>189</v>
+      </c>
+      <c r="I36" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="J36" s="14" t="s">
+        <v>310</v>
+      </c>
+      <c r="K36" s="14" t="s">
         <v>192</v>
       </c>
     </row>
     <row r="37" spans="1:11" ht="132.6" x14ac:dyDescent="0.3">
       <c r="A37" s="9" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B37" s="9" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C37" s="15" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="D37" s="15" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="E37" s="15" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="F37" s="15">
         <v>2</v>
       </c>
       <c r="G37" s="15" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="H37" s="15" t="s">
         <v>204</v>
@@ -4736,7 +4754,7 @@
         <v>205</v>
       </c>
       <c r="J37" s="15" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K37" s="15" t="s">
         <v>192</v>
@@ -4744,25 +4762,25 @@
     </row>
     <row r="38" spans="1:11" ht="145.80000000000001" x14ac:dyDescent="0.3">
       <c r="A38" s="9" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C38" s="15" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="D38" s="15" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="E38" s="15" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="F38" s="15">
         <v>3</v>
       </c>
       <c r="G38" s="15" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="H38" s="15" t="s">
         <v>204</v>
@@ -4771,92 +4789,94 @@
         <v>205</v>
       </c>
       <c r="J38" s="15" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="K38" s="15" t="s">
         <v>192</v>
       </c>
     </row>
     <row r="39" spans="1:11" ht="211.8" x14ac:dyDescent="0.3">
-      <c r="A39" s="22" t="s">
-        <v>298</v>
-      </c>
-      <c r="B39" s="22" t="s">
+      <c r="A39" s="11" t="s">
         <v>299</v>
       </c>
-      <c r="C39" s="23" t="s">
-        <v>318</v>
-      </c>
-      <c r="D39" s="23" t="s">
-        <v>319</v>
-      </c>
-      <c r="E39" s="23" t="s">
+      <c r="B39" s="11" t="s">
+        <v>300</v>
+      </c>
+      <c r="C39" s="14" t="s">
+        <v>321</v>
+      </c>
+      <c r="D39" s="14" t="s">
+        <v>322</v>
+      </c>
+      <c r="E39" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="F39" s="23">
+      <c r="F39" s="14">
         <v>9</v>
       </c>
-      <c r="G39" s="23" t="s">
-        <v>320</v>
-      </c>
-      <c r="H39" s="23" t="s">
-        <v>204</v>
-      </c>
-      <c r="I39" s="23" t="s">
-        <v>270</v>
-      </c>
-      <c r="J39" s="23" t="s">
-        <v>321</v>
-      </c>
-      <c r="K39" s="23" t="s">
-        <v>322</v>
+      <c r="G39" s="14" t="s">
+        <v>323</v>
+      </c>
+      <c r="H39" s="14" t="s">
+        <v>189</v>
+      </c>
+      <c r="I39" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="J39" s="14" t="s">
+        <v>324</v>
+      </c>
+      <c r="K39" s="14" t="s">
+        <v>325</v>
       </c>
     </row>
     <row r="40" spans="1:11" ht="132.6" x14ac:dyDescent="0.3">
-      <c r="A40" s="22" t="s">
-        <v>298</v>
-      </c>
-      <c r="B40" s="22" t="s">
+      <c r="A40" s="11" t="s">
         <v>299</v>
       </c>
-      <c r="C40" s="23" t="s">
-        <v>323</v>
-      </c>
-      <c r="D40" s="23" t="s">
-        <v>324</v>
-      </c>
-      <c r="E40" s="23" t="s">
+      <c r="B40" s="11" t="s">
+        <v>300</v>
+      </c>
+      <c r="C40" s="14" t="s">
+        <v>326</v>
+      </c>
+      <c r="D40" s="14" t="s">
+        <v>327</v>
+      </c>
+      <c r="E40" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="F40" s="23">
+      <c r="F40" s="14">
         <v>6</v>
       </c>
-      <c r="G40" s="23" t="s">
-        <v>325</v>
-      </c>
-      <c r="H40" s="23" t="s">
-        <v>204</v>
-      </c>
-      <c r="I40" s="23" t="s">
-        <v>270</v>
-      </c>
-      <c r="J40" s="23"/>
-      <c r="K40" s="23" t="s">
-        <v>326</v>
+      <c r="G40" s="14" t="s">
+        <v>328</v>
+      </c>
+      <c r="H40" s="14" t="s">
+        <v>189</v>
+      </c>
+      <c r="I40" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="J40" s="14" t="s">
+        <v>329</v>
+      </c>
+      <c r="K40" s="14" t="s">
+        <v>330</v>
       </c>
     </row>
     <row r="41" spans="1:11" ht="225" x14ac:dyDescent="0.3">
       <c r="A41" s="9" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C41" s="15" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="D41" s="15" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="E41" s="15" t="s">
         <v>42</v>
@@ -4865,7 +4885,7 @@
         <v>12</v>
       </c>
       <c r="G41" s="15" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
       <c r="H41" s="15" t="s">
         <v>204</v>
@@ -4874,24 +4894,24 @@
         <v>205</v>
       </c>
       <c r="J41" s="15" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="K41" s="15" t="s">
-        <v>331</v>
+        <v>335</v>
       </c>
     </row>
     <row r="42" spans="1:11" ht="93" x14ac:dyDescent="0.3">
       <c r="A42" s="11" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="B42" s="11" t="s">
         <v>140</v>
       </c>
       <c r="C42" s="14" t="s">
-        <v>333</v>
+        <v>337</v>
       </c>
       <c r="D42" s="14" t="s">
-        <v>334</v>
+        <v>338</v>
       </c>
       <c r="E42" s="14" t="s">
         <v>70</v>
@@ -4917,7 +4937,7 @@
     </row>
     <row r="43" spans="1:11" ht="106.2" x14ac:dyDescent="0.3">
       <c r="A43" s="11" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="B43" s="11" t="s">
         <v>140</v>
@@ -4926,7 +4946,7 @@
         <v>281</v>
       </c>
       <c r="D43" s="14" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="E43" s="14" t="s">
         <v>70</v>
@@ -4952,7 +4972,7 @@
     </row>
     <row r="44" spans="1:11" ht="66.599999999999994" x14ac:dyDescent="0.3">
       <c r="A44" s="11" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="B44" s="11" t="s">
         <v>140</v>
@@ -4961,7 +4981,7 @@
         <v>145</v>
       </c>
       <c r="D44" s="14" t="s">
-        <v>336</v>
+        <v>340</v>
       </c>
       <c r="E44" s="14" t="s">
         <v>70</v>
@@ -4987,16 +5007,16 @@
     </row>
     <row r="45" spans="1:11" ht="159" x14ac:dyDescent="0.3">
       <c r="A45" s="11" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="B45" s="11" t="s">
         <v>140</v>
       </c>
       <c r="C45" s="14" t="s">
-        <v>337</v>
+        <v>341</v>
       </c>
       <c r="D45" s="14" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="E45" s="14" t="s">
         <v>47</v>
@@ -5022,16 +5042,16 @@
     </row>
     <row r="46" spans="1:11" ht="172.2" x14ac:dyDescent="0.3">
       <c r="A46" s="22" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="B46" s="22" t="s">
         <v>140</v>
       </c>
       <c r="C46" s="23" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="D46" s="23" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
       <c r="E46" s="23" t="s">
         <v>17</v>
@@ -5040,7 +5060,7 @@
         <v>4</v>
       </c>
       <c r="G46" s="23" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="H46" s="23" t="s">
         <v>204</v>
@@ -5055,16 +5075,16 @@
     </row>
     <row r="47" spans="1:11" ht="93" x14ac:dyDescent="0.3">
       <c r="A47" s="9" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="B47" s="9" t="s">
         <v>140</v>
       </c>
       <c r="C47" s="15" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="D47" s="15" t="s">
-        <v>343</v>
+        <v>347</v>
       </c>
       <c r="E47" s="15" t="s">
         <v>32</v>
@@ -5083,21 +5103,21 @@
       </c>
       <c r="J47" s="15"/>
       <c r="K47" s="15" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="48" spans="1:11" ht="93" x14ac:dyDescent="0.3">
       <c r="A48" s="22" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
       <c r="B48" s="22" t="s">
         <v>147</v>
       </c>
       <c r="C48" s="23" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="D48" s="23" t="s">
-        <v>347</v>
+        <v>351</v>
       </c>
       <c r="E48" s="23" t="s">
         <v>224</v>
@@ -5121,16 +5141,16 @@
     </row>
     <row r="49" spans="1:11" ht="119.4" x14ac:dyDescent="0.3">
       <c r="A49" s="22" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
       <c r="B49" s="22" t="s">
         <v>147</v>
       </c>
       <c r="C49" s="23" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
       <c r="D49" s="23" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
       <c r="E49" s="23" t="s">
         <v>17</v>
@@ -5139,7 +5159,7 @@
         <v>6</v>
       </c>
       <c r="G49" s="23" t="s">
-        <v>350</v>
+        <v>354</v>
       </c>
       <c r="H49" s="23" t="s">
         <v>204</v>
@@ -5154,16 +5174,16 @@
     </row>
     <row r="50" spans="1:11" ht="79.8" x14ac:dyDescent="0.3">
       <c r="A50" s="9" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
       <c r="B50" s="9" t="s">
         <v>147</v>
       </c>
       <c r="C50" s="15" t="s">
-        <v>351</v>
+        <v>355</v>
       </c>
       <c r="D50" s="15" t="s">
-        <v>352</v>
+        <v>356</v>
       </c>
       <c r="E50" s="15" t="s">
         <v>32</v>
@@ -5182,21 +5202,21 @@
       </c>
       <c r="J50" s="15"/>
       <c r="K50" s="15" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
     </row>
     <row r="51" spans="1:11" ht="106.2" x14ac:dyDescent="0.3">
       <c r="A51" s="9" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
       <c r="B51" s="9" t="s">
         <v>147</v>
       </c>
       <c r="C51" s="15" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="D51" s="15" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
       <c r="E51" s="15" t="s">
         <v>37</v>
@@ -5215,30 +5235,30 @@
       </c>
       <c r="J51" s="15"/>
       <c r="K51" s="15" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
     </row>
     <row r="52" spans="1:11" ht="119.4" x14ac:dyDescent="0.3">
       <c r="A52" s="9" t="s">
-        <v>357</v>
+        <v>361</v>
       </c>
       <c r="B52" s="9" t="s">
         <v>152</v>
       </c>
       <c r="C52" s="15" t="s">
-        <v>358</v>
+        <v>362</v>
       </c>
       <c r="D52" s="15" t="s">
-        <v>359</v>
+        <v>363</v>
       </c>
       <c r="E52" s="15" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="F52" s="15">
         <v>3</v>
       </c>
       <c r="G52" s="15" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
       <c r="H52" s="15" t="s">
         <v>204</v>
@@ -5253,16 +5273,16 @@
     </row>
     <row r="53" spans="1:11" ht="145.80000000000001" x14ac:dyDescent="0.3">
       <c r="A53" s="9" t="s">
-        <v>357</v>
+        <v>361</v>
       </c>
       <c r="B53" s="9" t="s">
         <v>152</v>
       </c>
       <c r="C53" s="15" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="D53" s="15" t="s">
-        <v>362</v>
+        <v>366</v>
       </c>
       <c r="E53" s="15" t="s">
         <v>17</v>
@@ -5286,16 +5306,16 @@
     </row>
     <row r="54" spans="1:11" ht="93" x14ac:dyDescent="0.3">
       <c r="A54" s="9" t="s">
-        <v>357</v>
+        <v>361</v>
       </c>
       <c r="B54" s="9" t="s">
         <v>152</v>
       </c>
       <c r="C54" s="15" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="D54" s="15" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="E54" s="15" t="s">
         <v>32</v>
@@ -5319,16 +5339,16 @@
     </row>
     <row r="55" spans="1:11" ht="106.2" x14ac:dyDescent="0.3">
       <c r="A55" s="9" t="s">
-        <v>365</v>
+        <v>369</v>
       </c>
       <c r="B55" s="9" t="s">
         <v>155</v>
       </c>
       <c r="C55" s="15" t="s">
-        <v>366</v>
+        <v>370</v>
       </c>
       <c r="D55" s="15" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="E55" s="15" t="s">
         <v>107</v>
@@ -5352,16 +5372,16 @@
     </row>
     <row r="56" spans="1:11" ht="79.8" x14ac:dyDescent="0.3">
       <c r="A56" s="9" t="s">
-        <v>365</v>
+        <v>369</v>
       </c>
       <c r="B56" s="9" t="s">
         <v>155</v>
       </c>
       <c r="C56" s="15" t="s">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="D56" s="15" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="E56" s="15" t="s">
         <v>17</v>
@@ -5385,16 +5405,16 @@
     </row>
     <row r="57" spans="1:11" ht="93" x14ac:dyDescent="0.3">
       <c r="A57" s="9" t="s">
-        <v>370</v>
+        <v>374</v>
       </c>
       <c r="B57" s="9" t="s">
         <v>158</v>
       </c>
       <c r="C57" s="15" t="s">
-        <v>371</v>
+        <v>375</v>
       </c>
       <c r="D57" s="15" t="s">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="E57" s="15" t="s">
         <v>252</v>
@@ -5418,16 +5438,16 @@
     </row>
     <row r="58" spans="1:11" ht="79.8" x14ac:dyDescent="0.3">
       <c r="A58" s="9" t="s">
-        <v>370</v>
+        <v>374</v>
       </c>
       <c r="B58" s="9" t="s">
         <v>158</v>
       </c>
       <c r="C58" s="15" t="s">
-        <v>373</v>
+        <v>377</v>
       </c>
       <c r="D58" s="15" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
       <c r="E58" s="15" t="s">
         <v>32</v>
@@ -5451,16 +5471,16 @@
     </row>
     <row r="59" spans="1:11" ht="119.4" x14ac:dyDescent="0.3">
       <c r="A59" s="22" t="s">
-        <v>375</v>
+        <v>379</v>
       </c>
       <c r="B59" s="22" t="s">
         <v>161</v>
       </c>
       <c r="C59" s="23" t="s">
-        <v>376</v>
+        <v>380</v>
       </c>
       <c r="D59" s="23" t="s">
-        <v>377</v>
+        <v>381</v>
       </c>
       <c r="E59" s="23" t="s">
         <v>17</v>
@@ -5469,7 +5489,7 @@
         <v>4</v>
       </c>
       <c r="G59" s="23" t="s">
-        <v>378</v>
+        <v>382</v>
       </c>
       <c r="H59" s="23" t="s">
         <v>204</v>
@@ -5484,16 +5504,16 @@
     </row>
     <row r="60" spans="1:11" ht="66.599999999999994" x14ac:dyDescent="0.3">
       <c r="A60" s="9" t="s">
-        <v>375</v>
+        <v>379</v>
       </c>
       <c r="B60" s="9" t="s">
         <v>161</v>
       </c>
       <c r="C60" s="15" t="s">
-        <v>379</v>
+        <v>383</v>
       </c>
       <c r="D60" s="15" t="s">
-        <v>380</v>
+        <v>384</v>
       </c>
       <c r="E60" s="15" t="s">
         <v>32</v>
@@ -5517,16 +5537,16 @@
     </row>
     <row r="61" spans="1:11" ht="93" x14ac:dyDescent="0.3">
       <c r="A61" s="9" t="s">
-        <v>381</v>
+        <v>385</v>
       </c>
       <c r="B61" s="9" t="s">
         <v>164</v>
       </c>
       <c r="C61" s="15" t="s">
-        <v>382</v>
+        <v>386</v>
       </c>
       <c r="D61" s="15" t="s">
-        <v>383</v>
+        <v>387</v>
       </c>
       <c r="E61" s="15" t="s">
         <v>17</v>
@@ -5550,16 +5570,16 @@
     </row>
     <row r="62" spans="1:11" ht="119.4" x14ac:dyDescent="0.3">
       <c r="A62" s="9" t="s">
-        <v>384</v>
+        <v>388</v>
       </c>
       <c r="B62" s="9" t="s">
-        <v>385</v>
+        <v>389</v>
       </c>
       <c r="C62" s="15" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
       <c r="D62" s="15" t="s">
-        <v>387</v>
+        <v>391</v>
       </c>
       <c r="E62" s="15" t="s">
         <v>27</v>
@@ -5583,16 +5603,16 @@
     </row>
     <row r="63" spans="1:11" ht="106.2" x14ac:dyDescent="0.3">
       <c r="A63" s="9" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="B63" s="9" t="s">
         <v>167</v>
       </c>
       <c r="C63" s="15" t="s">
-        <v>389</v>
+        <v>393</v>
       </c>
       <c r="D63" s="15" t="s">
-        <v>390</v>
+        <v>394</v>
       </c>
       <c r="E63" s="15" t="s">
         <v>17</v>
@@ -5616,16 +5636,16 @@
     </row>
     <row r="64" spans="1:11" ht="106.2" x14ac:dyDescent="0.3">
       <c r="A64" s="9" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="B64" s="9" t="s">
         <v>167</v>
       </c>
       <c r="C64" s="15" t="s">
-        <v>391</v>
+        <v>395</v>
       </c>
       <c r="D64" s="15" t="s">
-        <v>392</v>
+        <v>396</v>
       </c>
       <c r="E64" s="15" t="s">
         <v>107</v>
@@ -5634,7 +5654,7 @@
         <v>2</v>
       </c>
       <c r="G64" s="15" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="H64" s="15" t="s">
         <v>204</v>
@@ -5649,16 +5669,16 @@
     </row>
     <row r="65" spans="1:11" ht="66.599999999999994" x14ac:dyDescent="0.3">
       <c r="A65" s="9" t="s">
-        <v>393</v>
+        <v>397</v>
       </c>
       <c r="B65" s="9" t="s">
         <v>170</v>
       </c>
       <c r="C65" s="15" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="D65" s="15" t="s">
-        <v>395</v>
+        <v>399</v>
       </c>
       <c r="E65" s="15" t="s">
         <v>252</v>
@@ -5682,16 +5702,16 @@
     </row>
     <row r="66" spans="1:11" ht="93" x14ac:dyDescent="0.3">
       <c r="A66" s="9" t="s">
-        <v>393</v>
+        <v>397</v>
       </c>
       <c r="B66" s="9" t="s">
         <v>170</v>
       </c>
       <c r="C66" s="15" t="s">
-        <v>396</v>
+        <v>400</v>
       </c>
       <c r="D66" s="15" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="E66" s="15" t="s">
         <v>32</v>
@@ -5715,16 +5735,16 @@
     </row>
     <row r="67" spans="1:11" ht="93" x14ac:dyDescent="0.3">
       <c r="A67" s="9" t="s">
-        <v>398</v>
+        <v>402</v>
       </c>
       <c r="B67" s="9" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
       <c r="C67" s="15" t="s">
-        <v>400</v>
+        <v>404</v>
       </c>
       <c r="D67" s="15" t="s">
-        <v>401</v>
+        <v>405</v>
       </c>
       <c r="E67" s="15" t="s">
         <v>32</v>
@@ -5748,16 +5768,16 @@
     </row>
     <row r="68" spans="1:11" ht="145.80000000000001" x14ac:dyDescent="0.3">
       <c r="A68" s="9" t="s">
-        <v>402</v>
+        <v>406</v>
       </c>
       <c r="B68" s="9" t="s">
-        <v>403</v>
+        <v>407</v>
       </c>
       <c r="C68" s="15" t="s">
-        <v>404</v>
+        <v>408</v>
       </c>
       <c r="D68" s="15" t="s">
-        <v>405</v>
+        <v>409</v>
       </c>
       <c r="E68" s="15" t="s">
         <v>252</v>
@@ -5781,16 +5801,16 @@
     </row>
     <row r="69" spans="1:11" ht="93" x14ac:dyDescent="0.3">
       <c r="A69" s="9" t="s">
-        <v>406</v>
+        <v>410</v>
       </c>
       <c r="B69" s="9" t="s">
-        <v>406</v>
+        <v>410</v>
       </c>
       <c r="C69" s="15" t="s">
-        <v>407</v>
+        <v>411</v>
       </c>
       <c r="D69" s="15" t="s">
-        <v>408</v>
+        <v>412</v>
       </c>
       <c r="E69" s="15" t="s">
         <v>32</v>
@@ -5814,16 +5834,16 @@
     </row>
     <row r="70" spans="1:11" ht="79.8" x14ac:dyDescent="0.3">
       <c r="A70" s="9" t="s">
-        <v>406</v>
+        <v>410</v>
       </c>
       <c r="B70" s="9" t="s">
-        <v>406</v>
+        <v>410</v>
       </c>
       <c r="C70" s="15" t="s">
-        <v>409</v>
+        <v>413</v>
       </c>
       <c r="D70" s="15" t="s">
-        <v>410</v>
+        <v>414</v>
       </c>
       <c r="E70" s="15" t="s">
         <v>42</v>
@@ -5842,21 +5862,21 @@
       </c>
       <c r="J70" s="15"/>
       <c r="K70" s="15" t="s">
-        <v>411</v>
+        <v>415</v>
       </c>
     </row>
     <row r="71" spans="1:11" ht="277.8" x14ac:dyDescent="0.3">
       <c r="A71" s="22" t="s">
-        <v>406</v>
+        <v>410</v>
       </c>
       <c r="B71" s="22" t="s">
-        <v>406</v>
+        <v>410</v>
       </c>
       <c r="C71" s="23" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="D71" s="23" t="s">
-        <v>413</v>
+        <v>417</v>
       </c>
       <c r="E71" s="23" t="s">
         <v>17</v>
@@ -5865,7 +5885,7 @@
         <v>2</v>
       </c>
       <c r="G71" s="23" t="s">
-        <v>414</v>
+        <v>418</v>
       </c>
       <c r="H71" s="23" t="s">
         <v>204</v>
@@ -5874,7 +5894,7 @@
         <v>270</v>
       </c>
       <c r="J71" s="23" t="s">
-        <v>415</v>
+        <v>419</v>
       </c>
       <c r="K71" s="23" t="s">
         <v>192</v>
@@ -5882,16 +5902,16 @@
     </row>
     <row r="72" spans="1:11" ht="225" x14ac:dyDescent="0.3">
       <c r="A72" s="9" t="s">
-        <v>406</v>
+        <v>410</v>
       </c>
       <c r="B72" s="9" t="s">
-        <v>406</v>
+        <v>410</v>
       </c>
       <c r="C72" s="15" t="s">
-        <v>416</v>
+        <v>420</v>
       </c>
       <c r="D72" s="15" t="s">
-        <v>417</v>
+        <v>421</v>
       </c>
       <c r="E72" s="15" t="s">
         <v>70</v>
@@ -5900,7 +5920,7 @@
         <v>3</v>
       </c>
       <c r="G72" s="15" t="s">
-        <v>418</v>
+        <v>422</v>
       </c>
       <c r="H72" s="15" t="s">
         <v>204</v>
@@ -5909,24 +5929,24 @@
         <v>205</v>
       </c>
       <c r="J72" s="15" t="s">
-        <v>419</v>
+        <v>423</v>
       </c>
       <c r="K72" s="15" t="s">
-        <v>420</v>
+        <v>424</v>
       </c>
     </row>
     <row r="73" spans="1:11" ht="66.599999999999994" x14ac:dyDescent="0.3">
       <c r="A73" s="9" t="s">
-        <v>421</v>
+        <v>425</v>
       </c>
       <c r="B73" s="9" t="s">
-        <v>422</v>
+        <v>426</v>
       </c>
       <c r="C73" s="15" t="s">
-        <v>423</v>
+        <v>427</v>
       </c>
       <c r="D73" s="15" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="E73" s="15" t="s">
         <v>17</v>
@@ -5950,16 +5970,16 @@
     </row>
     <row r="74" spans="1:11" ht="93" x14ac:dyDescent="0.3">
       <c r="A74" s="22" t="s">
-        <v>421</v>
+        <v>425</v>
       </c>
       <c r="B74" s="22" t="s">
-        <v>422</v>
+        <v>426</v>
       </c>
       <c r="C74" s="23" t="s">
-        <v>425</v>
+        <v>429</v>
       </c>
       <c r="D74" s="23" t="s">
-        <v>426</v>
+        <v>430</v>
       </c>
       <c r="E74" s="23" t="s">
         <v>32</v>
@@ -5968,7 +5988,7 @@
         <v>4</v>
       </c>
       <c r="G74" s="23" t="s">
-        <v>427</v>
+        <v>431</v>
       </c>
       <c r="H74" s="23" t="s">
         <v>204</v>
@@ -5978,21 +5998,21 @@
       </c>
       <c r="J74" s="23"/>
       <c r="K74" s="23" t="s">
-        <v>428</v>
+        <v>432</v>
       </c>
     </row>
     <row r="75" spans="1:11" ht="119.4" x14ac:dyDescent="0.3">
       <c r="A75" s="9" t="s">
-        <v>429</v>
+        <v>433</v>
       </c>
       <c r="B75" s="9" t="s">
-        <v>430</v>
+        <v>434</v>
       </c>
       <c r="C75" s="15" t="s">
-        <v>431</v>
+        <v>435</v>
       </c>
       <c r="D75" s="15" t="s">
-        <v>432</v>
+        <v>436</v>
       </c>
       <c r="E75" s="15" t="s">
         <v>107</v>
@@ -6016,16 +6036,16 @@
     </row>
     <row r="76" spans="1:11" ht="106.2" x14ac:dyDescent="0.3">
       <c r="A76" s="9" t="s">
-        <v>429</v>
+        <v>433</v>
       </c>
       <c r="B76" s="9" t="s">
-        <v>430</v>
+        <v>434</v>
       </c>
       <c r="C76" s="15" t="s">
-        <v>433</v>
+        <v>437</v>
       </c>
       <c r="D76" s="15" t="s">
-        <v>434</v>
+        <v>438</v>
       </c>
       <c r="E76" s="15" t="s">
         <v>42</v>
@@ -6049,16 +6069,16 @@
     </row>
     <row r="77" spans="1:11" ht="106.2" x14ac:dyDescent="0.3">
       <c r="A77" s="9" t="s">
-        <v>435</v>
+        <v>439</v>
       </c>
       <c r="B77" s="9" t="s">
-        <v>436</v>
+        <v>440</v>
       </c>
       <c r="C77" s="15" t="s">
-        <v>437</v>
+        <v>441</v>
       </c>
       <c r="D77" s="15" t="s">
-        <v>438</v>
+        <v>442</v>
       </c>
       <c r="E77" s="15" t="s">
         <v>32</v>
@@ -6082,16 +6102,16 @@
     </row>
     <row r="78" spans="1:11" ht="93" x14ac:dyDescent="0.3">
       <c r="A78" s="9" t="s">
-        <v>439</v>
+        <v>443</v>
       </c>
       <c r="B78" s="9" t="s">
-        <v>440</v>
+        <v>444</v>
       </c>
       <c r="C78" s="15" t="s">
-        <v>441</v>
+        <v>445</v>
       </c>
       <c r="D78" s="15" t="s">
-        <v>442</v>
+        <v>446</v>
       </c>
       <c r="E78" s="15" t="s">
         <v>17</v>
@@ -6115,16 +6135,16 @@
     </row>
     <row r="79" spans="1:11" ht="119.4" x14ac:dyDescent="0.3">
       <c r="A79" s="9" t="s">
-        <v>443</v>
+        <v>447</v>
       </c>
       <c r="B79" s="9" t="s">
-        <v>444</v>
+        <v>448</v>
       </c>
       <c r="C79" s="15" t="s">
-        <v>445</v>
+        <v>449</v>
       </c>
       <c r="D79" s="15" t="s">
-        <v>446</v>
+        <v>450</v>
       </c>
       <c r="E79" s="15" t="s">
         <v>32</v>
@@ -6148,16 +6168,16 @@
     </row>
     <row r="80" spans="1:11" ht="106.2" x14ac:dyDescent="0.3">
       <c r="A80" s="9" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="B80" s="9" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="C80" s="15" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="D80" s="15" t="s">
-        <v>450</v>
+        <v>454</v>
       </c>
       <c r="E80" s="15" t="s">
         <v>17</v>
@@ -6181,16 +6201,16 @@
     </row>
     <row r="81" spans="1:11" ht="106.2" x14ac:dyDescent="0.3">
       <c r="A81" s="22" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="B81" s="22" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="C81" s="23" t="s">
-        <v>451</v>
+        <v>455</v>
       </c>
       <c r="D81" s="23" t="s">
-        <v>452</v>
+        <v>456</v>
       </c>
       <c r="E81" s="23" t="s">
         <v>32</v>
@@ -6214,16 +6234,16 @@
     </row>
     <row r="82" spans="1:11" ht="79.8" x14ac:dyDescent="0.3">
       <c r="A82" s="9" t="s">
-        <v>453</v>
+        <v>457</v>
       </c>
       <c r="B82" s="9" t="s">
-        <v>454</v>
+        <v>458</v>
       </c>
       <c r="C82" s="15" t="s">
-        <v>455</v>
+        <v>459</v>
       </c>
       <c r="D82" s="15" t="s">
-        <v>456</v>
+        <v>460</v>
       </c>
       <c r="E82" s="15" t="s">
         <v>107</v>
@@ -6247,16 +6267,16 @@
     </row>
     <row r="83" spans="1:11" ht="119.4" x14ac:dyDescent="0.3">
       <c r="A83" s="9" t="s">
-        <v>457</v>
+        <v>461</v>
       </c>
       <c r="B83" s="9" t="s">
-        <v>458</v>
+        <v>462</v>
       </c>
       <c r="C83" s="15" t="s">
-        <v>459</v>
+        <v>463</v>
       </c>
       <c r="D83" s="15" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="E83" s="15" t="s">
         <v>32</v>
@@ -6280,16 +6300,16 @@
     </row>
     <row r="84" spans="1:11" ht="93" x14ac:dyDescent="0.3">
       <c r="A84" s="9" t="s">
-        <v>461</v>
+        <v>465</v>
       </c>
       <c r="B84" s="9" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
       <c r="C84" s="15" t="s">
-        <v>463</v>
+        <v>467</v>
       </c>
       <c r="D84" s="15" t="s">
-        <v>464</v>
+        <v>468</v>
       </c>
       <c r="E84" s="15" t="s">
         <v>70</v>
@@ -6313,16 +6333,16 @@
     </row>
     <row r="85" spans="1:11" ht="145.80000000000001" x14ac:dyDescent="0.3">
       <c r="A85" s="9" t="s">
-        <v>465</v>
+        <v>469</v>
       </c>
       <c r="B85" s="9" t="s">
-        <v>466</v>
+        <v>470</v>
       </c>
       <c r="C85" s="15" t="s">
-        <v>467</v>
+        <v>471</v>
       </c>
       <c r="D85" s="15" t="s">
-        <v>468</v>
+        <v>472</v>
       </c>
       <c r="E85" s="15" t="s">
         <v>47</v>
@@ -6346,16 +6366,16 @@
     </row>
     <row r="86" spans="1:11" ht="106.2" x14ac:dyDescent="0.3">
       <c r="A86" s="9" t="s">
-        <v>469</v>
+        <v>473</v>
       </c>
       <c r="B86" s="9" t="s">
-        <v>470</v>
+        <v>474</v>
       </c>
       <c r="C86" s="15" t="s">
-        <v>471</v>
+        <v>475</v>
       </c>
       <c r="D86" s="15" t="s">
-        <v>472</v>
+        <v>476</v>
       </c>
       <c r="E86" s="15" t="s">
         <v>27</v>
@@ -6379,16 +6399,16 @@
     </row>
     <row r="87" spans="1:11" ht="93" x14ac:dyDescent="0.3">
       <c r="A87" s="9" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B87" s="9" t="s">
-        <v>474</v>
+        <v>478</v>
       </c>
       <c r="C87" s="15" t="s">
-        <v>475</v>
+        <v>479</v>
       </c>
       <c r="D87" s="15" t="s">
-        <v>476</v>
+        <v>480</v>
       </c>
       <c r="E87" s="15" t="s">
         <v>107</v>
@@ -6397,7 +6417,7 @@
         <v>2</v>
       </c>
       <c r="G87" s="15" t="s">
-        <v>477</v>
+        <v>481</v>
       </c>
       <c r="H87" s="15" t="s">
         <v>204</v>
@@ -6412,16 +6432,16 @@
     </row>
     <row r="88" spans="1:11" ht="119.4" x14ac:dyDescent="0.3">
       <c r="A88" s="9" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B88" s="9" t="s">
-        <v>474</v>
+        <v>478</v>
       </c>
       <c r="C88" s="15" t="s">
-        <v>478</v>
+        <v>482</v>
       </c>
       <c r="D88" s="15" t="s">
-        <v>479</v>
+        <v>483</v>
       </c>
       <c r="E88" s="15" t="s">
         <v>32</v>
@@ -6445,16 +6465,16 @@
     </row>
     <row r="89" spans="1:11" ht="93" x14ac:dyDescent="0.3">
       <c r="A89" s="9" t="s">
-        <v>480</v>
+        <v>484</v>
       </c>
       <c r="B89" s="9" t="s">
-        <v>481</v>
+        <v>485</v>
       </c>
       <c r="C89" s="15" t="s">
-        <v>482</v>
+        <v>486</v>
       </c>
       <c r="D89" s="15" t="s">
-        <v>483</v>
+        <v>487</v>
       </c>
       <c r="E89" s="15" t="s">
         <v>107</v>
@@ -6478,16 +6498,16 @@
     </row>
     <row r="90" spans="1:11" ht="119.4" x14ac:dyDescent="0.3">
       <c r="A90" s="9" t="s">
-        <v>484</v>
+        <v>488</v>
       </c>
       <c r="B90" s="9" t="s">
-        <v>485</v>
+        <v>489</v>
       </c>
       <c r="C90" s="15" t="s">
-        <v>486</v>
+        <v>490</v>
       </c>
       <c r="D90" s="15" t="s">
-        <v>487</v>
+        <v>491</v>
       </c>
       <c r="E90" s="15" t="s">
         <v>27</v>
@@ -6511,16 +6531,16 @@
     </row>
     <row r="91" spans="1:11" ht="159" x14ac:dyDescent="0.3">
       <c r="A91" s="9" t="s">
-        <v>488</v>
+        <v>492</v>
       </c>
       <c r="B91" s="9" t="s">
-        <v>489</v>
+        <v>493</v>
       </c>
       <c r="C91" s="15" t="s">
-        <v>490</v>
+        <v>494</v>
       </c>
       <c r="D91" s="15" t="s">
-        <v>491</v>
+        <v>495</v>
       </c>
       <c r="E91" s="15" t="s">
         <v>32</v>
@@ -6538,7 +6558,7 @@
         <v>226</v>
       </c>
       <c r="J91" s="15" t="s">
-        <v>492</v>
+        <v>496</v>
       </c>
       <c r="K91" s="15" t="s">
         <v>192</v>
@@ -6546,7 +6566,7 @@
     </row>
     <row r="93" spans="1:11" ht="85.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A93" s="21" t="s">
-        <v>493</v>
+        <v>497</v>
       </c>
       <c r="B93" s="1"/>
       <c r="C93" s="1"/>
@@ -6560,7 +6580,7 @@
       <c r="K93" s="1"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:K3" xr:uid="{66D78C55-1DD8-4428-80B7-D978393E723A}"/>
+  <autoFilter ref="A3:K3" xr:uid="{CDE00EBB-670F-4983-9E58-B2E3B1026B64}"/>
   <mergeCells count="2">
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A93:K93"/>
@@ -6570,7 +6590,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3320E27B-962F-476C-99E3-6E9F568D33FD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E01783F-2C0A-4160-A5B8-C3AEC1586AD7}">
   <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -6836,7 +6856,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:E3" xr:uid="{3320E27B-962F-476C-99E3-6E9F568D33FD}"/>
+  <autoFilter ref="A3:E3" xr:uid="{5E01783F-2C0A-4160-A5B8-C3AEC1586AD7}"/>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
   </mergeCells>
@@ -6845,7 +6865,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E09837FE-036D-4FB3-BAA5-EC4087018752}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AB71E9C-31E0-4DC6-BFCA-3BEE75F95328}">
   <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -7051,7 +7071,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27A49328-CDC9-45AE-A439-B26F90F8A78A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{751F6249-8DC4-4EF8-9465-E8BFDF814697}">
   <dimension ref="A1:D47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -7062,7 +7082,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="18" x14ac:dyDescent="0.35">
       <c r="A1" s="20" t="s">
-        <v>494</v>
+        <v>498</v>
       </c>
       <c r="B1" s="20"/>
       <c r="C1" s="20"/>
@@ -7075,106 +7095,106 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
-        <v>495</v>
+        <v>499</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>496</v>
+        <v>500</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>497</v>
+        <v>501</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
-        <v>498</v>
+        <v>502</v>
       </c>
       <c r="B4" s="25" t="s">
-        <v>499</v>
+        <v>503</v>
       </c>
       <c r="C4" s="25" t="s">
-        <v>500</v>
+        <v>504</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
-        <v>501</v>
+        <v>505</v>
       </c>
       <c r="B5" s="25" t="s">
-        <v>502</v>
+        <v>506</v>
       </c>
       <c r="C5" s="25" t="s">
-        <v>503</v>
+        <v>507</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
-        <v>504</v>
+        <v>508</v>
       </c>
       <c r="B6" s="25" t="s">
-        <v>505</v>
+        <v>509</v>
       </c>
       <c r="C6" s="25" t="s">
-        <v>506</v>
+        <v>510</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
-        <v>507</v>
+        <v>511</v>
       </c>
       <c r="B7" s="25" t="s">
-        <v>508</v>
+        <v>512</v>
       </c>
       <c r="C7" s="25" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="B8" s="25" t="s">
-        <v>511</v>
+        <v>515</v>
       </c>
       <c r="C8" s="25" t="s">
-        <v>512</v>
+        <v>516</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
-        <v>513</v>
+        <v>517</v>
       </c>
       <c r="B9" s="25" t="s">
-        <v>514</v>
+        <v>518</v>
       </c>
       <c r="C9" s="25" t="s">
-        <v>515</v>
+        <v>519</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
-        <v>516</v>
+        <v>520</v>
       </c>
       <c r="B10" s="25" t="s">
-        <v>517</v>
+        <v>521</v>
       </c>
       <c r="C10" s="25" t="s">
-        <v>518</v>
+        <v>522</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="7" t="s">
-        <v>519</v>
+        <v>523</v>
       </c>
       <c r="B11" s="25" t="s">
-        <v>520</v>
+        <v>524</v>
       </c>
       <c r="C11" s="25" t="s">
-        <v>521</v>
+        <v>525</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="21" t="s">
-        <v>522</v>
+        <v>526</v>
       </c>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
@@ -7184,7 +7204,7 @@
         <v>180</v>
       </c>
       <c r="B14" s="26" t="s">
-        <v>523</v>
+        <v>527</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
@@ -7192,7 +7212,7 @@
         <v>189</v>
       </c>
       <c r="B15" s="9">
-        <v>17</v>
+        <v>22</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
@@ -7200,7 +7220,7 @@
         <v>204</v>
       </c>
       <c r="B16" s="9">
-        <v>69</v>
+        <v>64</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
@@ -7213,153 +7233,153 @@
     </row>
     <row r="28" spans="1:3" ht="17.399999999999999" x14ac:dyDescent="0.35">
       <c r="A28" s="5" t="s">
-        <v>524</v>
+        <v>528</v>
       </c>
       <c r="B28" s="5"/>
       <c r="C28" s="5"/>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" s="10" t="s">
-        <v>525</v>
+        <v>529</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>526</v>
+        <v>530</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="11" t="s">
-        <v>527</v>
+        <v>531</v>
       </c>
       <c r="B31" s="14" t="s">
-        <v>528</v>
+        <v>532</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="11" t="s">
-        <v>529</v>
+        <v>533</v>
       </c>
       <c r="B32" s="14" t="s">
-        <v>530</v>
+        <v>534</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="11" t="s">
-        <v>520</v>
+        <v>524</v>
       </c>
       <c r="B33" s="14" t="s">
-        <v>531</v>
+        <v>535</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="11" t="s">
-        <v>532</v>
+        <v>536</v>
       </c>
       <c r="B34" s="14" t="s">
-        <v>533</v>
+        <v>537</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="11" t="s">
-        <v>534</v>
+        <v>538</v>
       </c>
       <c r="B35" s="14" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="11" t="s">
-        <v>536</v>
+        <v>540</v>
       </c>
       <c r="B36" s="14" t="s">
-        <v>537</v>
+        <v>541</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="11" t="s">
-        <v>538</v>
+        <v>542</v>
       </c>
       <c r="B37" s="14" t="s">
-        <v>539</v>
+        <v>543</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="11" t="s">
-        <v>540</v>
+        <v>544</v>
       </c>
       <c r="B38" s="14" t="s">
-        <v>541</v>
+        <v>545</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="11" t="s">
-        <v>542</v>
+        <v>546</v>
       </c>
       <c r="B39" s="14" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="11" t="s">
-        <v>544</v>
+        <v>548</v>
       </c>
       <c r="B40" s="14" t="s">
-        <v>545</v>
+        <v>549</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="11" t="s">
-        <v>546</v>
+        <v>550</v>
       </c>
       <c r="B41" s="14" t="s">
-        <v>547</v>
+        <v>551</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="9" t="s">
-        <v>548</v>
+        <v>552</v>
       </c>
       <c r="B42" s="15" t="s">
-        <v>549</v>
+        <v>553</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="9" t="s">
-        <v>550</v>
+        <v>554</v>
       </c>
       <c r="B43" s="15" t="s">
-        <v>551</v>
+        <v>555</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="11" t="s">
-        <v>552</v>
+        <v>556</v>
       </c>
       <c r="B44" s="14" t="s">
-        <v>553</v>
+        <v>557</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="9" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="B45" s="15" t="s">
-        <v>555</v>
+        <v>559</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="9" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="B46" s="15" t="s">
-        <v>557</v>
+        <v>561</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="9" t="s">
-        <v>558</v>
+        <v>562</v>
       </c>
       <c r="B47" s="15" t="s">
-        <v>559</v>
+        <v>563</v>
       </c>
     </row>
   </sheetData>
@@ -7374,7 +7394,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A95DC96-FAC5-4233-862B-9887027141F4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A5DB6D1-7BF2-44D1-B601-A2507581CBEE}">
   <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -7902,7 +7922,7 @@
       <c r="G25" s="1"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:G3" xr:uid="{4A95DC96-FAC5-4233-862B-9887027141F4}"/>
+  <autoFilter ref="A3:G3" xr:uid="{7A5DB6D1-7BF2-44D1-B601-A2507581CBEE}"/>
   <mergeCells count="2">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A25:G25"/>

</xml_diff>

<commit_message>
Ajouter la feuille "Operations par type traitement" au tableau de bord
Meme limitation reelle qu'un plan Excel n'a qu'un seul axe de pliage par
feuille (deja rencontree pour le dossier d'exploitation) : la feuille
"Catalogue des operations" groupe par module, donc "combien d'operations
TFJ/EOM/etc. au total sur les 88 ?" ne s'y lit pas d'un coup d'oeil.

Nouvelle feuille jumelle, memes 88 lignes, groupees par Type de traitement
et triees par nombre decroissant (EOM 20, TFJ 15, ON_DEMAND 14, JOUR/NRT 10,
EOW 5, NRT/JOUR/EOY 4, EOQ 3, INTRADAY/CUTOFF 2, SIMULATION/REALTIME/PURGE/
EOD/DIFFERE 1) - verifie ligne par ligne via COM (88/88 lignes de detail
retrouvees, aucune perdue).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/TABLEAU_DE_BORD_CYCLES_OPERATOIRES.xlsx
+++ b/docs/TABLEAU_DE_BORD_CYCLES_OPERATOIRES.xlsx
@@ -8,22 +8,24 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP PROBOOK\Documents\ECF\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{74D2DBD9-2160-4AFE-99A1-1A04A938936E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5AB24D01-363C-4578-A742-ED10BD157361}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2472" yWindow="2472" windowWidth="17280" windowHeight="8880" xr2:uid="{5FF0A2E3-D62D-4FC9-AC61-E6D22B7FCF7A}"/>
+    <workbookView xWindow="2472" yWindow="2472" windowWidth="17280" windowHeight="8880" xr2:uid="{03B8B241-4607-456B-A423-362F3C32F81C}"/>
   </bookViews>
   <sheets>
     <sheet name="Vue d'ensemble" sheetId="1" r:id="rId1"/>
     <sheet name="Catalogue des operations" sheetId="5" r:id="rId2"/>
-    <sheet name="Taxonomie complete" sheetId="2" r:id="rId3"/>
-    <sheet name="Cycles reels construits" sheetId="3" r:id="rId4"/>
-    <sheet name="Exploitation MCO - efficacite" sheetId="6" r:id="rId5"/>
-    <sheet name="Scenario 50 traitements" sheetId="4" r:id="rId6"/>
+    <sheet name="Operations par type traitement" sheetId="6" r:id="rId3"/>
+    <sheet name="Taxonomie complete" sheetId="2" r:id="rId4"/>
+    <sheet name="Cycles reels construits" sheetId="3" r:id="rId5"/>
+    <sheet name="Exploitation MCO - efficacite" sheetId="7" r:id="rId6"/>
+    <sheet name="Scenario 50 traitements" sheetId="4" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Catalogue des operations'!$A$3:$K$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Scenario 50 traitements'!$A$3:$G$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Taxonomie complete'!$A$3:$E$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Operations par type traitement'!$A$3:$K$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Scenario 50 traitements'!$A$3:$G$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Taxonomie complete'!$A$3:$E$3</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1180" uniqueCount="591">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2057" uniqueCount="607">
   <si>
     <t>Tableau de bord des cycles operatoires - ERP_CRM_FACTORY</t>
   </si>
@@ -1619,6 +1621,54 @@
   </si>
   <si>
     <t>TOTAL : 88 operations reelles cataloguees, 233 jobs estimes au total (lineaires + paralleles cumules) - 30 operations deja CONSTRUITES ET VERIFIEES (vert), 0 en PRIORITE HAUTE a construire ensuite (jaune - operations quotidiennes/critiques des modules coeur), le reste sur le meme patron deja prouve. Ces chiffres sont des estimations architecturales raisonnees (jamais un decompte de jobs reellement ecrits pour les operations encore A CONSTRUIRE). Priorite : HAUTE = necessaire des le premier cycle d'exploitation reel (quotidien/critique sur un module coeur) - MOYENNE = utile mais differable - BASSE = illustratif/complementaire. Colonne 'Depend de' : chaine de dependance metier reelle (pas une IN_COND technique) - l'operation en amont qui doit exister avant que celle-ci ait un sens operationnel.</t>
+  </si>
+  <si>
+    <t>Memes 88 operations, groupees par type de traitement (TFJ/EOM/ON_DEMAND/...) - pour repondre a 'combien d'operations TFJ au total ?'</t>
+  </si>
+  <si>
+    <t>20 operations - 4 construite(s) - 59 jobs estimes (deplier pour voir le detail)</t>
+  </si>
+  <si>
+    <t>15 operations - 8 construite(s) - 46 jobs estimes (deplier pour voir le detail)</t>
+  </si>
+  <si>
+    <t>14 operations - 11 construite(s) - 38 jobs estimes (deplier pour voir le detail)</t>
+  </si>
+  <si>
+    <t>10 operations - 2 construite(s) - 14 jobs estimes (deplier pour voir le detail)</t>
+  </si>
+  <si>
+    <t>5 operations - 0 construite(s) - 9 jobs estimes (deplier pour voir le detail)</t>
+  </si>
+  <si>
+    <t>4 operations - 0 construite(s) - 5 jobs estimes (deplier pour voir le detail)</t>
+  </si>
+  <si>
+    <t>4 operations - 1 construite(s) - 9 jobs estimes (deplier pour voir le detail)</t>
+  </si>
+  <si>
+    <t>4 operations - 0 construite(s) - 21 jobs estimes (deplier pour voir le detail)</t>
+  </si>
+  <si>
+    <t>3 operations - 1 construite(s) - 13 jobs estimes (deplier pour voir le detail)</t>
+  </si>
+  <si>
+    <t>2 operations - 0 construite(s) - 6 jobs estimes (deplier pour voir le detail)</t>
+  </si>
+  <si>
+    <t>2 operations - 1 construite(s) - 2 jobs estimes (deplier pour voir le detail)</t>
+  </si>
+  <si>
+    <t>1 operation - 0 construite(s) - 2 jobs estimes (deplier pour voir le detail)</t>
+  </si>
+  <si>
+    <t>1 operation - 0 construite(s) - 6 jobs estimes (deplier pour voir le detail)</t>
+  </si>
+  <si>
+    <t>1 operation - 0 construite(s) - 1 jobs estimes (deplier pour voir le detail)</t>
+  </si>
+  <si>
+    <t>1 operation - 1 construite(s) - 1 jobs estimes (deplier pour voir le detail)</t>
   </si>
   <si>
     <t>Maintien en condition operationnelle - preuves d'efficacite reelles</t>
@@ -2200,7 +2250,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-BDBB-4559-A8D0-940529E41D84}"/>
+              <c16:uniqueId val="{00000000-1B25-465B-B328-6C6F1E9EC643}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2313,7 +2363,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-BDBB-4559-A8D0-940529E41D84}"/>
+              <c16:uniqueId val="{00000002-1B25-465B-B328-6C6F1E9EC643}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2426,7 +2476,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-BDBB-4559-A8D0-940529E41D84}"/>
+              <c16:uniqueId val="{00000003-1B25-465B-B328-6C6F1E9EC643}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3103,7 +3153,7 @@
         <xdr:cNvPr id="2" name="Graphique 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BA5D2A91-2795-4F8F-B812-158618510B19}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{77622F8B-2DE7-4D72-A27C-08C704AAA420}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3420,7 +3470,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BEA3A266-F89F-4F14-AA83-40942C948E58}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83412779-CC28-47E7-9A4C-5D35CBDAC71D}">
   <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -3609,7 +3659,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E15E1F3-362E-4514-B137-131D17BF05EF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D4FF926-5CAC-497A-8E37-6D37AAC9CEF4}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
@@ -7289,7 +7339,7 @@
       <c r="K128" s="1"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:K3" xr:uid="{2E15E1F3-362E-4514-B137-131D17BF05EF}"/>
+  <autoFilter ref="A3:K3" xr:uid="{6D4FF926-5CAC-497A-8E37-6D37AAC9CEF4}"/>
   <mergeCells count="37">
     <mergeCell ref="A128:K128"/>
     <mergeCell ref="C114:K114"/>
@@ -7334,7 +7384,3374 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27130E95-0811-4A0B-A01B-CAF6D9C8D224}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D3B3E0A-BA90-4939-991F-4C9A794F6191}">
+  <sheetPr>
+    <outlinePr summaryBelow="0"/>
+  </sheetPr>
+  <dimension ref="A1:K107"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" outlineLevelRow="1" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16.77734375" customWidth="1"/>
+    <col min="2" max="2" width="8.77734375" customWidth="1"/>
+    <col min="3" max="3" width="32.77734375" customWidth="1"/>
+    <col min="4" max="4" width="55.77734375" customWidth="1"/>
+    <col min="5" max="5" width="14.77734375" customWidth="1"/>
+    <col min="6" max="6" width="10.77734375" customWidth="1"/>
+    <col min="7" max="7" width="40.77734375" customWidth="1"/>
+    <col min="8" max="8" width="14.77734375" customWidth="1"/>
+    <col min="9" max="9" width="10.77734375" customWidth="1"/>
+    <col min="10" max="10" width="35.77734375" customWidth="1"/>
+    <col min="11" max="11" width="40.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A1" s="8" t="s">
+        <v>525</v>
+      </c>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
+      <c r="I1" s="8"/>
+      <c r="J1" s="8"/>
+      <c r="K1" s="8"/>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A2" s="9"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="9"/>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A3" s="10" t="s">
+        <v>174</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>175</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>176</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>177</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>178</v>
+      </c>
+      <c r="G3" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="H3" s="10" t="s">
+        <v>180</v>
+      </c>
+      <c r="I3" s="10" t="s">
+        <v>181</v>
+      </c>
+      <c r="J3" s="10" t="s">
+        <v>182</v>
+      </c>
+      <c r="K3" s="10" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" collapsed="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="24" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" s="22"/>
+      <c r="C4" s="25" t="s">
+        <v>526</v>
+      </c>
+      <c r="D4" s="23"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="23"/>
+      <c r="G4" s="23"/>
+      <c r="H4" s="23"/>
+      <c r="I4" s="23"/>
+      <c r="J4" s="23"/>
+      <c r="K4" s="23"/>
+    </row>
+    <row r="5" spans="1:11" ht="119.4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="9" t="s">
+        <v>214</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>216</v>
+      </c>
+      <c r="C5" s="15" t="s">
+        <v>221</v>
+      </c>
+      <c r="D5" s="15" t="s">
+        <v>222</v>
+      </c>
+      <c r="E5" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="F5" s="15">
+        <v>4</v>
+      </c>
+      <c r="G5" s="15" t="s">
+        <v>223</v>
+      </c>
+      <c r="H5" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I5" s="15" t="s">
+        <v>206</v>
+      </c>
+      <c r="J5" s="15"/>
+      <c r="K5" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="79.8" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="9" t="s">
+        <v>232</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="C6" s="15" t="s">
+        <v>245</v>
+      </c>
+      <c r="D6" s="15" t="s">
+        <v>246</v>
+      </c>
+      <c r="E6" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="F6" s="15">
+        <v>1</v>
+      </c>
+      <c r="G6" s="15" t="s">
+        <v>237</v>
+      </c>
+      <c r="H6" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I6" s="15" t="s">
+        <v>228</v>
+      </c>
+      <c r="J6" s="15"/>
+      <c r="K6" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="106.2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="9" t="s">
+        <v>247</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="C7" s="15" t="s">
+        <v>258</v>
+      </c>
+      <c r="D7" s="15" t="s">
+        <v>259</v>
+      </c>
+      <c r="E7" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="F7" s="15">
+        <v>1</v>
+      </c>
+      <c r="G7" s="15" t="s">
+        <v>237</v>
+      </c>
+      <c r="H7" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I7" s="15" t="s">
+        <v>228</v>
+      </c>
+      <c r="J7" s="15"/>
+      <c r="K7" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="159" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="11" t="s">
+        <v>282</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>297</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>298</v>
+      </c>
+      <c r="E8" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="F8" s="14">
+        <v>5</v>
+      </c>
+      <c r="G8" s="14" t="s">
+        <v>299</v>
+      </c>
+      <c r="H8" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="I8" s="14" t="s">
+        <v>191</v>
+      </c>
+      <c r="J8" s="14" t="s">
+        <v>300</v>
+      </c>
+      <c r="K8" s="14" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="211.8" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="11" t="s">
+        <v>305</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>307</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>329</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>330</v>
+      </c>
+      <c r="E9" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="F9" s="14">
+        <v>9</v>
+      </c>
+      <c r="G9" s="14" t="s">
+        <v>331</v>
+      </c>
+      <c r="H9" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="I9" s="14" t="s">
+        <v>191</v>
+      </c>
+      <c r="J9" s="14" t="s">
+        <v>332</v>
+      </c>
+      <c r="K9" s="14" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="93" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="9" t="s">
+        <v>344</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>356</v>
+      </c>
+      <c r="D10" s="15" t="s">
+        <v>357</v>
+      </c>
+      <c r="E10" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="F10" s="15">
+        <v>3</v>
+      </c>
+      <c r="G10" s="15" t="s">
+        <v>200</v>
+      </c>
+      <c r="H10" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I10" s="15" t="s">
+        <v>206</v>
+      </c>
+      <c r="J10" s="15"/>
+      <c r="K10" s="15" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="79.8" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="9" t="s">
+        <v>359</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>147</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>368</v>
+      </c>
+      <c r="D11" s="15" t="s">
+        <v>369</v>
+      </c>
+      <c r="E11" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="F11" s="15">
+        <v>5</v>
+      </c>
+      <c r="G11" s="15" t="s">
+        <v>200</v>
+      </c>
+      <c r="H11" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I11" s="15" t="s">
+        <v>206</v>
+      </c>
+      <c r="J11" s="15"/>
+      <c r="K11" s="15" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="93" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="9" t="s">
+        <v>374</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="C12" s="15" t="s">
+        <v>381</v>
+      </c>
+      <c r="D12" s="15" t="s">
+        <v>382</v>
+      </c>
+      <c r="E12" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="F12" s="15">
+        <v>2</v>
+      </c>
+      <c r="G12" s="15" t="s">
+        <v>200</v>
+      </c>
+      <c r="H12" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I12" s="15" t="s">
+        <v>228</v>
+      </c>
+      <c r="J12" s="15"/>
+      <c r="K12" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="79.8" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="9" t="s">
+        <v>389</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>158</v>
+      </c>
+      <c r="C13" s="15" t="s">
+        <v>392</v>
+      </c>
+      <c r="D13" s="15" t="s">
+        <v>393</v>
+      </c>
+      <c r="E13" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="F13" s="15">
+        <v>2</v>
+      </c>
+      <c r="G13" s="15" t="s">
+        <v>200</v>
+      </c>
+      <c r="H13" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I13" s="15" t="s">
+        <v>228</v>
+      </c>
+      <c r="J13" s="15"/>
+      <c r="K13" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="66.599999999999994" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="9" t="s">
+        <v>394</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="C14" s="15" t="s">
+        <v>400</v>
+      </c>
+      <c r="D14" s="15" t="s">
+        <v>401</v>
+      </c>
+      <c r="E14" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="F14" s="15">
+        <v>3</v>
+      </c>
+      <c r="G14" s="15" t="s">
+        <v>200</v>
+      </c>
+      <c r="H14" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I14" s="15" t="s">
+        <v>206</v>
+      </c>
+      <c r="J14" s="15"/>
+      <c r="K14" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="93" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="9" t="s">
+        <v>417</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>170</v>
+      </c>
+      <c r="C15" s="15" t="s">
+        <v>420</v>
+      </c>
+      <c r="D15" s="15" t="s">
+        <v>421</v>
+      </c>
+      <c r="E15" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="F15" s="15">
+        <v>2</v>
+      </c>
+      <c r="G15" s="15" t="s">
+        <v>200</v>
+      </c>
+      <c r="H15" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I15" s="15" t="s">
+        <v>228</v>
+      </c>
+      <c r="J15" s="15"/>
+      <c r="K15" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="93" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="9" t="s">
+        <v>422</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>423</v>
+      </c>
+      <c r="C16" s="15" t="s">
+        <v>424</v>
+      </c>
+      <c r="D16" s="15" t="s">
+        <v>425</v>
+      </c>
+      <c r="E16" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="F16" s="15">
+        <v>2</v>
+      </c>
+      <c r="G16" s="15" t="s">
+        <v>200</v>
+      </c>
+      <c r="H16" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I16" s="15" t="s">
+        <v>228</v>
+      </c>
+      <c r="J16" s="15"/>
+      <c r="K16" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="93" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="9" t="s">
+        <v>431</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>431</v>
+      </c>
+      <c r="C17" s="15" t="s">
+        <v>433</v>
+      </c>
+      <c r="D17" s="15" t="s">
+        <v>434</v>
+      </c>
+      <c r="E17" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="F17" s="15">
+        <v>2</v>
+      </c>
+      <c r="G17" s="15" t="s">
+        <v>200</v>
+      </c>
+      <c r="H17" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I17" s="15" t="s">
+        <v>206</v>
+      </c>
+      <c r="J17" s="15"/>
+      <c r="K17" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="93" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="11" t="s">
+        <v>447</v>
+      </c>
+      <c r="B18" s="11" t="s">
+        <v>449</v>
+      </c>
+      <c r="C18" s="14" t="s">
+        <v>452</v>
+      </c>
+      <c r="D18" s="14" t="s">
+        <v>453</v>
+      </c>
+      <c r="E18" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="F18" s="14">
+        <v>4</v>
+      </c>
+      <c r="G18" s="14" t="s">
+        <v>454</v>
+      </c>
+      <c r="H18" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="I18" s="14" t="s">
+        <v>191</v>
+      </c>
+      <c r="J18" s="14" t="s">
+        <v>455</v>
+      </c>
+      <c r="K18" s="14" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="106.2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="9" t="s">
+        <v>463</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>464</v>
+      </c>
+      <c r="C19" s="15" t="s">
+        <v>465</v>
+      </c>
+      <c r="D19" s="15" t="s">
+        <v>466</v>
+      </c>
+      <c r="E19" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="F19" s="15">
+        <v>3</v>
+      </c>
+      <c r="G19" s="15" t="s">
+        <v>200</v>
+      </c>
+      <c r="H19" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I19" s="15" t="s">
+        <v>206</v>
+      </c>
+      <c r="J19" s="15"/>
+      <c r="K19" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="119.4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="9" t="s">
+        <v>471</v>
+      </c>
+      <c r="B20" s="9" t="s">
+        <v>472</v>
+      </c>
+      <c r="C20" s="15" t="s">
+        <v>473</v>
+      </c>
+      <c r="D20" s="15" t="s">
+        <v>474</v>
+      </c>
+      <c r="E20" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="F20" s="15">
+        <v>2</v>
+      </c>
+      <c r="G20" s="15" t="s">
+        <v>200</v>
+      </c>
+      <c r="H20" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I20" s="15" t="s">
+        <v>228</v>
+      </c>
+      <c r="J20" s="15"/>
+      <c r="K20" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="145.80000000000001" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="11" t="s">
+        <v>475</v>
+      </c>
+      <c r="B21" s="11" t="s">
+        <v>477</v>
+      </c>
+      <c r="C21" s="14" t="s">
+        <v>480</v>
+      </c>
+      <c r="D21" s="14" t="s">
+        <v>481</v>
+      </c>
+      <c r="E21" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="F21" s="14">
+        <v>3</v>
+      </c>
+      <c r="G21" s="14" t="s">
+        <v>200</v>
+      </c>
+      <c r="H21" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="I21" s="14" t="s">
+        <v>191</v>
+      </c>
+      <c r="J21" s="14" t="s">
+        <v>482</v>
+      </c>
+      <c r="K21" s="14" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" ht="119.4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="9" t="s">
+        <v>487</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>488</v>
+      </c>
+      <c r="C22" s="15" t="s">
+        <v>489</v>
+      </c>
+      <c r="D22" s="15" t="s">
+        <v>490</v>
+      </c>
+      <c r="E22" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="F22" s="15">
+        <v>2</v>
+      </c>
+      <c r="G22" s="15" t="s">
+        <v>200</v>
+      </c>
+      <c r="H22" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I22" s="15" t="s">
+        <v>228</v>
+      </c>
+      <c r="J22" s="15"/>
+      <c r="K22" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="119.4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="9" t="s">
+        <v>503</v>
+      </c>
+      <c r="B23" s="9" t="s">
+        <v>505</v>
+      </c>
+      <c r="C23" s="15" t="s">
+        <v>509</v>
+      </c>
+      <c r="D23" s="15" t="s">
+        <v>510</v>
+      </c>
+      <c r="E23" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="F23" s="15">
+        <v>2</v>
+      </c>
+      <c r="G23" s="15" t="s">
+        <v>200</v>
+      </c>
+      <c r="H23" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I23" s="15" t="s">
+        <v>228</v>
+      </c>
+      <c r="J23" s="15"/>
+      <c r="K23" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" ht="159" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="9" t="s">
+        <v>519</v>
+      </c>
+      <c r="B24" s="9" t="s">
+        <v>520</v>
+      </c>
+      <c r="C24" s="15" t="s">
+        <v>521</v>
+      </c>
+      <c r="D24" s="15" t="s">
+        <v>522</v>
+      </c>
+      <c r="E24" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="F24" s="15">
+        <v>2</v>
+      </c>
+      <c r="G24" s="15" t="s">
+        <v>200</v>
+      </c>
+      <c r="H24" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I24" s="15" t="s">
+        <v>228</v>
+      </c>
+      <c r="J24" s="15" t="s">
+        <v>523</v>
+      </c>
+      <c r="K24" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" collapsed="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="B25" s="22"/>
+      <c r="C25" s="25" t="s">
+        <v>527</v>
+      </c>
+      <c r="D25" s="23"/>
+      <c r="E25" s="23"/>
+      <c r="F25" s="23"/>
+      <c r="G25" s="23"/>
+      <c r="H25" s="23"/>
+      <c r="I25" s="23"/>
+      <c r="J25" s="23"/>
+      <c r="K25" s="23"/>
+    </row>
+    <row r="26" spans="1:11" ht="172.2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="11" t="s">
+        <v>260</v>
+      </c>
+      <c r="B26" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="C26" s="14" t="s">
+        <v>272</v>
+      </c>
+      <c r="D26" s="14" t="s">
+        <v>273</v>
+      </c>
+      <c r="E26" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="F26" s="14">
+        <v>3</v>
+      </c>
+      <c r="G26" s="14" t="s">
+        <v>274</v>
+      </c>
+      <c r="H26" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="I26" s="14" t="s">
+        <v>191</v>
+      </c>
+      <c r="J26" s="14" t="s">
+        <v>275</v>
+      </c>
+      <c r="K26" s="14" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" ht="119.4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="11" t="s">
+        <v>282</v>
+      </c>
+      <c r="B27" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="C27" s="14" t="s">
+        <v>290</v>
+      </c>
+      <c r="D27" s="14" t="s">
+        <v>291</v>
+      </c>
+      <c r="E27" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="F27" s="14">
+        <v>3</v>
+      </c>
+      <c r="G27" s="14" t="s">
+        <v>292</v>
+      </c>
+      <c r="H27" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="I27" s="14" t="s">
+        <v>191</v>
+      </c>
+      <c r="J27" s="14" t="s">
+        <v>293</v>
+      </c>
+      <c r="K27" s="14" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" ht="159" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="11" t="s">
+        <v>305</v>
+      </c>
+      <c r="B28" s="11" t="s">
+        <v>307</v>
+      </c>
+      <c r="C28" s="14" t="s">
+        <v>311</v>
+      </c>
+      <c r="D28" s="14" t="s">
+        <v>312</v>
+      </c>
+      <c r="E28" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="F28" s="14">
+        <v>5</v>
+      </c>
+      <c r="G28" s="14" t="s">
+        <v>313</v>
+      </c>
+      <c r="H28" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="I28" s="14" t="s">
+        <v>191</v>
+      </c>
+      <c r="J28" s="14" t="s">
+        <v>314</v>
+      </c>
+      <c r="K28" s="14" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" ht="172.2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="11" t="s">
+        <v>305</v>
+      </c>
+      <c r="B29" s="11" t="s">
+        <v>307</v>
+      </c>
+      <c r="C29" s="14" t="s">
+        <v>315</v>
+      </c>
+      <c r="D29" s="14" t="s">
+        <v>316</v>
+      </c>
+      <c r="E29" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="F29" s="14">
+        <v>2</v>
+      </c>
+      <c r="G29" s="14" t="s">
+        <v>317</v>
+      </c>
+      <c r="H29" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="I29" s="14" t="s">
+        <v>191</v>
+      </c>
+      <c r="J29" s="14" t="s">
+        <v>318</v>
+      </c>
+      <c r="K29" s="14" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" ht="172.2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="11" t="s">
+        <v>344</v>
+      </c>
+      <c r="B30" s="11" t="s">
+        <v>140</v>
+      </c>
+      <c r="C30" s="14" t="s">
+        <v>352</v>
+      </c>
+      <c r="D30" s="14" t="s">
+        <v>353</v>
+      </c>
+      <c r="E30" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="F30" s="14">
+        <v>4</v>
+      </c>
+      <c r="G30" s="14" t="s">
+        <v>354</v>
+      </c>
+      <c r="H30" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="I30" s="14" t="s">
+        <v>191</v>
+      </c>
+      <c r="J30" s="14" t="s">
+        <v>355</v>
+      </c>
+      <c r="K30" s="14" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" ht="185.4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="11" t="s">
+        <v>359</v>
+      </c>
+      <c r="B31" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="C31" s="14" t="s">
+        <v>364</v>
+      </c>
+      <c r="D31" s="14" t="s">
+        <v>365</v>
+      </c>
+      <c r="E31" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="F31" s="14">
+        <v>6</v>
+      </c>
+      <c r="G31" s="14" t="s">
+        <v>366</v>
+      </c>
+      <c r="H31" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="I31" s="14" t="s">
+        <v>191</v>
+      </c>
+      <c r="J31" s="14" t="s">
+        <v>367</v>
+      </c>
+      <c r="K31" s="14" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" ht="145.80000000000001" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="9" t="s">
+        <v>374</v>
+      </c>
+      <c r="B32" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="C32" s="15" t="s">
+        <v>379</v>
+      </c>
+      <c r="D32" s="15" t="s">
+        <v>380</v>
+      </c>
+      <c r="E32" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="F32" s="15">
+        <v>4</v>
+      </c>
+      <c r="G32" s="15" t="s">
+        <v>200</v>
+      </c>
+      <c r="H32" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I32" s="15" t="s">
+        <v>206</v>
+      </c>
+      <c r="J32" s="15"/>
+      <c r="K32" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" ht="79.8" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="9" t="s">
+        <v>383</v>
+      </c>
+      <c r="B33" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="C33" s="15" t="s">
+        <v>387</v>
+      </c>
+      <c r="D33" s="15" t="s">
+        <v>388</v>
+      </c>
+      <c r="E33" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="F33" s="15">
+        <v>2</v>
+      </c>
+      <c r="G33" s="15" t="s">
+        <v>200</v>
+      </c>
+      <c r="H33" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I33" s="15" t="s">
+        <v>228</v>
+      </c>
+      <c r="J33" s="15"/>
+      <c r="K33" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" ht="198.6" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="11" t="s">
+        <v>394</v>
+      </c>
+      <c r="B34" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="C34" s="14" t="s">
+        <v>396</v>
+      </c>
+      <c r="D34" s="14" t="s">
+        <v>397</v>
+      </c>
+      <c r="E34" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="F34" s="14">
+        <v>4</v>
+      </c>
+      <c r="G34" s="14" t="s">
+        <v>398</v>
+      </c>
+      <c r="H34" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="I34" s="14" t="s">
+        <v>191</v>
+      </c>
+      <c r="J34" s="14" t="s">
+        <v>399</v>
+      </c>
+      <c r="K34" s="14" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" ht="93" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="9" t="s">
+        <v>402</v>
+      </c>
+      <c r="B35" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="C35" s="15" t="s">
+        <v>404</v>
+      </c>
+      <c r="D35" s="15" t="s">
+        <v>405</v>
+      </c>
+      <c r="E35" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="F35" s="15">
+        <v>3</v>
+      </c>
+      <c r="G35" s="15" t="s">
+        <v>200</v>
+      </c>
+      <c r="H35" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I35" s="15" t="s">
+        <v>206</v>
+      </c>
+      <c r="J35" s="15"/>
+      <c r="K35" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" ht="106.2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="9" t="s">
+        <v>411</v>
+      </c>
+      <c r="B36" s="9" t="s">
+        <v>167</v>
+      </c>
+      <c r="C36" s="15" t="s">
+        <v>413</v>
+      </c>
+      <c r="D36" s="15" t="s">
+        <v>414</v>
+      </c>
+      <c r="E36" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="F36" s="15">
+        <v>3</v>
+      </c>
+      <c r="G36" s="15" t="s">
+        <v>200</v>
+      </c>
+      <c r="H36" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I36" s="15" t="s">
+        <v>206</v>
+      </c>
+      <c r="J36" s="15"/>
+      <c r="K36" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" ht="277.8" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="11" t="s">
+        <v>431</v>
+      </c>
+      <c r="B37" s="11" t="s">
+        <v>431</v>
+      </c>
+      <c r="C37" s="14" t="s">
+        <v>438</v>
+      </c>
+      <c r="D37" s="14" t="s">
+        <v>439</v>
+      </c>
+      <c r="E37" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="F37" s="14">
+        <v>2</v>
+      </c>
+      <c r="G37" s="14" t="s">
+        <v>440</v>
+      </c>
+      <c r="H37" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="I37" s="14" t="s">
+        <v>191</v>
+      </c>
+      <c r="J37" s="14" t="s">
+        <v>441</v>
+      </c>
+      <c r="K37" s="14" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" ht="66.599999999999994" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="9" t="s">
+        <v>447</v>
+      </c>
+      <c r="B38" s="9" t="s">
+        <v>449</v>
+      </c>
+      <c r="C38" s="15" t="s">
+        <v>450</v>
+      </c>
+      <c r="D38" s="15" t="s">
+        <v>451</v>
+      </c>
+      <c r="E38" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="F38" s="15">
+        <v>2</v>
+      </c>
+      <c r="G38" s="15" t="s">
+        <v>200</v>
+      </c>
+      <c r="H38" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I38" s="15" t="s">
+        <v>206</v>
+      </c>
+      <c r="J38" s="15"/>
+      <c r="K38" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" ht="93" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="9" t="s">
+        <v>467</v>
+      </c>
+      <c r="B39" s="9" t="s">
+        <v>468</v>
+      </c>
+      <c r="C39" s="15" t="s">
+        <v>469</v>
+      </c>
+      <c r="D39" s="15" t="s">
+        <v>470</v>
+      </c>
+      <c r="E39" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="F39" s="15">
+        <v>1</v>
+      </c>
+      <c r="G39" s="15" t="s">
+        <v>237</v>
+      </c>
+      <c r="H39" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I39" s="15" t="s">
+        <v>228</v>
+      </c>
+      <c r="J39" s="15"/>
+      <c r="K39" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" ht="106.2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="9" t="s">
+        <v>475</v>
+      </c>
+      <c r="B40" s="9" t="s">
+        <v>477</v>
+      </c>
+      <c r="C40" s="15" t="s">
+        <v>478</v>
+      </c>
+      <c r="D40" s="15" t="s">
+        <v>479</v>
+      </c>
+      <c r="E40" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="F40" s="15">
+        <v>2</v>
+      </c>
+      <c r="G40" s="15" t="s">
+        <v>200</v>
+      </c>
+      <c r="H40" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I40" s="15" t="s">
+        <v>206</v>
+      </c>
+      <c r="J40" s="15"/>
+      <c r="K40" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" collapsed="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="24" t="s">
+        <v>70</v>
+      </c>
+      <c r="B41" s="22"/>
+      <c r="C41" s="25" t="s">
+        <v>528</v>
+      </c>
+      <c r="D41" s="23"/>
+      <c r="E41" s="23"/>
+      <c r="F41" s="23"/>
+      <c r="G41" s="23"/>
+      <c r="H41" s="23"/>
+      <c r="I41" s="23"/>
+      <c r="J41" s="23"/>
+      <c r="K41" s="23"/>
+    </row>
+    <row r="42" spans="1:11" ht="211.8" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="B42" s="11" t="s">
+        <v>186</v>
+      </c>
+      <c r="C42" s="14" t="s">
+        <v>187</v>
+      </c>
+      <c r="D42" s="14" t="s">
+        <v>188</v>
+      </c>
+      <c r="E42" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="F42" s="14">
+        <v>20</v>
+      </c>
+      <c r="G42" s="14" t="s">
+        <v>189</v>
+      </c>
+      <c r="H42" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="I42" s="14" t="s">
+        <v>191</v>
+      </c>
+      <c r="J42" s="14" t="s">
+        <v>192</v>
+      </c>
+      <c r="K42" s="14" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" ht="145.80000000000001" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="9" t="s">
+        <v>214</v>
+      </c>
+      <c r="B43" s="9" t="s">
+        <v>216</v>
+      </c>
+      <c r="C43" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="D43" s="15" t="s">
+        <v>218</v>
+      </c>
+      <c r="E43" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="F43" s="15">
+        <v>3</v>
+      </c>
+      <c r="G43" s="15" t="s">
+        <v>219</v>
+      </c>
+      <c r="H43" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I43" s="15" t="s">
+        <v>206</v>
+      </c>
+      <c r="J43" s="15" t="s">
+        <v>220</v>
+      </c>
+      <c r="K43" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" ht="119.4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="11" t="s">
+        <v>260</v>
+      </c>
+      <c r="B44" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="C44" s="14" t="s">
+        <v>262</v>
+      </c>
+      <c r="D44" s="14" t="s">
+        <v>263</v>
+      </c>
+      <c r="E44" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="F44" s="14">
+        <v>1</v>
+      </c>
+      <c r="G44" s="14" t="s">
+        <v>237</v>
+      </c>
+      <c r="H44" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="I44" s="14" t="s">
+        <v>191</v>
+      </c>
+      <c r="J44" s="14" t="s">
+        <v>124</v>
+      </c>
+      <c r="K44" s="14" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" ht="185.4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="11" t="s">
+        <v>260</v>
+      </c>
+      <c r="B45" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="C45" s="14" t="s">
+        <v>264</v>
+      </c>
+      <c r="D45" s="14" t="s">
+        <v>265</v>
+      </c>
+      <c r="E45" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="F45" s="14">
+        <v>1</v>
+      </c>
+      <c r="G45" s="14" t="s">
+        <v>237</v>
+      </c>
+      <c r="H45" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="I45" s="14" t="s">
+        <v>191</v>
+      </c>
+      <c r="J45" s="14" t="s">
+        <v>127</v>
+      </c>
+      <c r="K45" s="14" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" ht="159" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="11" t="s">
+        <v>260</v>
+      </c>
+      <c r="B46" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="C46" s="14" t="s">
+        <v>266</v>
+      </c>
+      <c r="D46" s="14" t="s">
+        <v>267</v>
+      </c>
+      <c r="E46" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="F46" s="14">
+        <v>1</v>
+      </c>
+      <c r="G46" s="14" t="s">
+        <v>237</v>
+      </c>
+      <c r="H46" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="I46" s="14" t="s">
+        <v>191</v>
+      </c>
+      <c r="J46" s="14" t="s">
+        <v>268</v>
+      </c>
+      <c r="K46" s="14" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" ht="132.6" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="11" t="s">
+        <v>260</v>
+      </c>
+      <c r="B47" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="C47" s="14" t="s">
+        <v>269</v>
+      </c>
+      <c r="D47" s="14" t="s">
+        <v>270</v>
+      </c>
+      <c r="E47" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="F47" s="14">
+        <v>2</v>
+      </c>
+      <c r="G47" s="14" t="s">
+        <v>237</v>
+      </c>
+      <c r="H47" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="I47" s="14" t="s">
+        <v>191</v>
+      </c>
+      <c r="J47" s="14" t="s">
+        <v>271</v>
+      </c>
+      <c r="K47" s="14" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" ht="93" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="11" t="s">
+        <v>282</v>
+      </c>
+      <c r="B48" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="C48" s="14" t="s">
+        <v>284</v>
+      </c>
+      <c r="D48" s="14" t="s">
+        <v>285</v>
+      </c>
+      <c r="E48" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="F48" s="14">
+        <v>1</v>
+      </c>
+      <c r="G48" s="14" t="s">
+        <v>237</v>
+      </c>
+      <c r="H48" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="I48" s="14" t="s">
+        <v>191</v>
+      </c>
+      <c r="J48" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="K48" s="14" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" ht="93" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="11" t="s">
+        <v>282</v>
+      </c>
+      <c r="B49" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="C49" s="14" t="s">
+        <v>286</v>
+      </c>
+      <c r="D49" s="14" t="s">
+        <v>287</v>
+      </c>
+      <c r="E49" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="F49" s="14">
+        <v>1</v>
+      </c>
+      <c r="G49" s="14" t="s">
+        <v>237</v>
+      </c>
+      <c r="H49" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="I49" s="14" t="s">
+        <v>191</v>
+      </c>
+      <c r="J49" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="K49" s="14" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" ht="93" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="11" t="s">
+        <v>282</v>
+      </c>
+      <c r="B50" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="C50" s="14" t="s">
+        <v>288</v>
+      </c>
+      <c r="D50" s="14" t="s">
+        <v>289</v>
+      </c>
+      <c r="E50" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="F50" s="14">
+        <v>1</v>
+      </c>
+      <c r="G50" s="14" t="s">
+        <v>237</v>
+      </c>
+      <c r="H50" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="I50" s="14" t="s">
+        <v>191</v>
+      </c>
+      <c r="J50" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="K50" s="14" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" ht="93" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="11" t="s">
+        <v>344</v>
+      </c>
+      <c r="B51" s="11" t="s">
+        <v>140</v>
+      </c>
+      <c r="C51" s="14" t="s">
+        <v>346</v>
+      </c>
+      <c r="D51" s="14" t="s">
+        <v>347</v>
+      </c>
+      <c r="E51" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="F51" s="14">
+        <v>1</v>
+      </c>
+      <c r="G51" s="14" t="s">
+        <v>237</v>
+      </c>
+      <c r="H51" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="I51" s="14" t="s">
+        <v>191</v>
+      </c>
+      <c r="J51" s="14" t="s">
+        <v>139</v>
+      </c>
+      <c r="K51" s="14" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" ht="106.2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="11" t="s">
+        <v>344</v>
+      </c>
+      <c r="B52" s="11" t="s">
+        <v>140</v>
+      </c>
+      <c r="C52" s="14" t="s">
+        <v>286</v>
+      </c>
+      <c r="D52" s="14" t="s">
+        <v>348</v>
+      </c>
+      <c r="E52" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="F52" s="14">
+        <v>1</v>
+      </c>
+      <c r="G52" s="14" t="s">
+        <v>237</v>
+      </c>
+      <c r="H52" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="I52" s="14" t="s">
+        <v>191</v>
+      </c>
+      <c r="J52" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="K52" s="14" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" ht="66.599999999999994" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="11" t="s">
+        <v>344</v>
+      </c>
+      <c r="B53" s="11" t="s">
+        <v>140</v>
+      </c>
+      <c r="C53" s="14" t="s">
+        <v>145</v>
+      </c>
+      <c r="D53" s="14" t="s">
+        <v>349</v>
+      </c>
+      <c r="E53" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="F53" s="14">
+        <v>1</v>
+      </c>
+      <c r="G53" s="14" t="s">
+        <v>237</v>
+      </c>
+      <c r="H53" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="I53" s="14" t="s">
+        <v>191</v>
+      </c>
+      <c r="J53" s="14" t="s">
+        <v>144</v>
+      </c>
+      <c r="K53" s="14" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" ht="225" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="9" t="s">
+        <v>431</v>
+      </c>
+      <c r="B54" s="9" t="s">
+        <v>431</v>
+      </c>
+      <c r="C54" s="15" t="s">
+        <v>442</v>
+      </c>
+      <c r="D54" s="15" t="s">
+        <v>443</v>
+      </c>
+      <c r="E54" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="F54" s="15">
+        <v>3</v>
+      </c>
+      <c r="G54" s="15" t="s">
+        <v>444</v>
+      </c>
+      <c r="H54" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I54" s="15" t="s">
+        <v>206</v>
+      </c>
+      <c r="J54" s="15" t="s">
+        <v>445</v>
+      </c>
+      <c r="K54" s="15" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" ht="93" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="9" t="s">
+        <v>491</v>
+      </c>
+      <c r="B55" s="9" t="s">
+        <v>492</v>
+      </c>
+      <c r="C55" s="15" t="s">
+        <v>493</v>
+      </c>
+      <c r="D55" s="15" t="s">
+        <v>494</v>
+      </c>
+      <c r="E55" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="F55" s="15">
+        <v>1</v>
+      </c>
+      <c r="G55" s="15" t="s">
+        <v>237</v>
+      </c>
+      <c r="H55" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I55" s="15" t="s">
+        <v>228</v>
+      </c>
+      <c r="J55" s="15"/>
+      <c r="K55" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" collapsed="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="24" t="s">
+        <v>107</v>
+      </c>
+      <c r="B56" s="22"/>
+      <c r="C56" s="25" t="s">
+        <v>529</v>
+      </c>
+      <c r="D56" s="23"/>
+      <c r="E56" s="23"/>
+      <c r="F56" s="23"/>
+      <c r="G56" s="23"/>
+      <c r="H56" s="23"/>
+      <c r="I56" s="23"/>
+      <c r="J56" s="23"/>
+      <c r="K56" s="23"/>
+    </row>
+    <row r="57" spans="1:11" ht="132.6" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A57" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="B57" s="11" t="s">
+        <v>186</v>
+      </c>
+      <c r="C57" s="14" t="s">
+        <v>194</v>
+      </c>
+      <c r="D57" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="E57" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="F57" s="14">
+        <v>1</v>
+      </c>
+      <c r="G57" s="14" t="s">
+        <v>196</v>
+      </c>
+      <c r="H57" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="I57" s="14" t="s">
+        <v>191</v>
+      </c>
+      <c r="J57" s="14" t="s">
+        <v>197</v>
+      </c>
+      <c r="K57" s="14" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" ht="93" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="9" t="s">
+        <v>232</v>
+      </c>
+      <c r="B58" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="C58" s="15" t="s">
+        <v>235</v>
+      </c>
+      <c r="D58" s="15" t="s">
+        <v>236</v>
+      </c>
+      <c r="E58" s="15" t="s">
+        <v>107</v>
+      </c>
+      <c r="F58" s="15">
+        <v>1</v>
+      </c>
+      <c r="G58" s="15" t="s">
+        <v>237</v>
+      </c>
+      <c r="H58" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I58" s="15" t="s">
+        <v>206</v>
+      </c>
+      <c r="J58" s="15" t="s">
+        <v>238</v>
+      </c>
+      <c r="K58" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" ht="93" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="9" t="s">
+        <v>232</v>
+      </c>
+      <c r="B59" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="C59" s="15" t="s">
+        <v>239</v>
+      </c>
+      <c r="D59" s="15" t="s">
+        <v>240</v>
+      </c>
+      <c r="E59" s="15" t="s">
+        <v>107</v>
+      </c>
+      <c r="F59" s="15">
+        <v>2</v>
+      </c>
+      <c r="G59" s="15" t="s">
+        <v>241</v>
+      </c>
+      <c r="H59" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I59" s="15" t="s">
+        <v>228</v>
+      </c>
+      <c r="J59" s="15"/>
+      <c r="K59" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" ht="185.4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="11" t="s">
+        <v>282</v>
+      </c>
+      <c r="B60" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="C60" s="14" t="s">
+        <v>294</v>
+      </c>
+      <c r="D60" s="14" t="s">
+        <v>295</v>
+      </c>
+      <c r="E60" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="F60" s="14">
+        <v>1</v>
+      </c>
+      <c r="G60" s="14" t="s">
+        <v>237</v>
+      </c>
+      <c r="H60" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="I60" s="14" t="s">
+        <v>191</v>
+      </c>
+      <c r="J60" s="14" t="s">
+        <v>296</v>
+      </c>
+      <c r="K60" s="14" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" ht="106.2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A61" s="9" t="s">
+        <v>383</v>
+      </c>
+      <c r="B61" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="C61" s="15" t="s">
+        <v>385</v>
+      </c>
+      <c r="D61" s="15" t="s">
+        <v>386</v>
+      </c>
+      <c r="E61" s="15" t="s">
+        <v>107</v>
+      </c>
+      <c r="F61" s="15">
+        <v>1</v>
+      </c>
+      <c r="G61" s="15" t="s">
+        <v>237</v>
+      </c>
+      <c r="H61" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I61" s="15" t="s">
+        <v>206</v>
+      </c>
+      <c r="J61" s="15"/>
+      <c r="K61" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" ht="106.2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A62" s="9" t="s">
+        <v>411</v>
+      </c>
+      <c r="B62" s="9" t="s">
+        <v>167</v>
+      </c>
+      <c r="C62" s="15" t="s">
+        <v>415</v>
+      </c>
+      <c r="D62" s="15" t="s">
+        <v>416</v>
+      </c>
+      <c r="E62" s="15" t="s">
+        <v>107</v>
+      </c>
+      <c r="F62" s="15">
+        <v>2</v>
+      </c>
+      <c r="G62" s="15" t="s">
+        <v>317</v>
+      </c>
+      <c r="H62" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I62" s="15" t="s">
+        <v>206</v>
+      </c>
+      <c r="J62" s="15"/>
+      <c r="K62" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" ht="119.4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A63" s="9" t="s">
+        <v>457</v>
+      </c>
+      <c r="B63" s="9" t="s">
+        <v>458</v>
+      </c>
+      <c r="C63" s="15" t="s">
+        <v>459</v>
+      </c>
+      <c r="D63" s="15" t="s">
+        <v>460</v>
+      </c>
+      <c r="E63" s="15" t="s">
+        <v>107</v>
+      </c>
+      <c r="F63" s="15">
+        <v>1</v>
+      </c>
+      <c r="G63" s="15" t="s">
+        <v>237</v>
+      </c>
+      <c r="H63" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I63" s="15" t="s">
+        <v>228</v>
+      </c>
+      <c r="J63" s="15"/>
+      <c r="K63" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" ht="79.8" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A64" s="9" t="s">
+        <v>483</v>
+      </c>
+      <c r="B64" s="9" t="s">
+        <v>484</v>
+      </c>
+      <c r="C64" s="15" t="s">
+        <v>485</v>
+      </c>
+      <c r="D64" s="15" t="s">
+        <v>486</v>
+      </c>
+      <c r="E64" s="15" t="s">
+        <v>107</v>
+      </c>
+      <c r="F64" s="15">
+        <v>1</v>
+      </c>
+      <c r="G64" s="15" t="s">
+        <v>237</v>
+      </c>
+      <c r="H64" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I64" s="15" t="s">
+        <v>228</v>
+      </c>
+      <c r="J64" s="15"/>
+      <c r="K64" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" ht="93" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A65" s="9" t="s">
+        <v>503</v>
+      </c>
+      <c r="B65" s="9" t="s">
+        <v>505</v>
+      </c>
+      <c r="C65" s="15" t="s">
+        <v>506</v>
+      </c>
+      <c r="D65" s="15" t="s">
+        <v>507</v>
+      </c>
+      <c r="E65" s="15" t="s">
+        <v>107</v>
+      </c>
+      <c r="F65" s="15">
+        <v>2</v>
+      </c>
+      <c r="G65" s="15" t="s">
+        <v>508</v>
+      </c>
+      <c r="H65" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I65" s="15" t="s">
+        <v>206</v>
+      </c>
+      <c r="J65" s="15"/>
+      <c r="K65" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" ht="93" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A66" s="9" t="s">
+        <v>511</v>
+      </c>
+      <c r="B66" s="9" t="s">
+        <v>512</v>
+      </c>
+      <c r="C66" s="15" t="s">
+        <v>513</v>
+      </c>
+      <c r="D66" s="15" t="s">
+        <v>514</v>
+      </c>
+      <c r="E66" s="15" t="s">
+        <v>107</v>
+      </c>
+      <c r="F66" s="15">
+        <v>2</v>
+      </c>
+      <c r="G66" s="15" t="s">
+        <v>200</v>
+      </c>
+      <c r="H66" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I66" s="15" t="s">
+        <v>228</v>
+      </c>
+      <c r="J66" s="15"/>
+      <c r="K66" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" collapsed="1" x14ac:dyDescent="0.3">
+      <c r="A67" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="B67" s="22"/>
+      <c r="C67" s="25" t="s">
+        <v>530</v>
+      </c>
+      <c r="D67" s="23"/>
+      <c r="E67" s="23"/>
+      <c r="F67" s="23"/>
+      <c r="G67" s="23"/>
+      <c r="H67" s="23"/>
+      <c r="I67" s="23"/>
+      <c r="J67" s="23"/>
+      <c r="K67" s="23"/>
+    </row>
+    <row r="68" spans="1:11" ht="119.4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A68" s="9" t="s">
+        <v>214</v>
+      </c>
+      <c r="B68" s="9" t="s">
+        <v>216</v>
+      </c>
+      <c r="C68" s="15" t="s">
+        <v>230</v>
+      </c>
+      <c r="D68" s="15" t="s">
+        <v>231</v>
+      </c>
+      <c r="E68" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="F68" s="15">
+        <v>2</v>
+      </c>
+      <c r="G68" s="15" t="s">
+        <v>200</v>
+      </c>
+      <c r="H68" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I68" s="15" t="s">
+        <v>228</v>
+      </c>
+      <c r="J68" s="15"/>
+      <c r="K68" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" ht="172.2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A69" s="9" t="s">
+        <v>260</v>
+      </c>
+      <c r="B69" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="C69" s="15" t="s">
+        <v>279</v>
+      </c>
+      <c r="D69" s="15" t="s">
+        <v>280</v>
+      </c>
+      <c r="E69" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="F69" s="15">
+        <v>3</v>
+      </c>
+      <c r="G69" s="15" t="s">
+        <v>281</v>
+      </c>
+      <c r="H69" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I69" s="15" t="s">
+        <v>206</v>
+      </c>
+      <c r="J69" s="15"/>
+      <c r="K69" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" ht="119.4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A70" s="9" t="s">
+        <v>406</v>
+      </c>
+      <c r="B70" s="9" t="s">
+        <v>408</v>
+      </c>
+      <c r="C70" s="15" t="s">
+        <v>409</v>
+      </c>
+      <c r="D70" s="15" t="s">
+        <v>410</v>
+      </c>
+      <c r="E70" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="F70" s="15">
+        <v>2</v>
+      </c>
+      <c r="G70" s="15" t="s">
+        <v>200</v>
+      </c>
+      <c r="H70" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I70" s="15" t="s">
+        <v>228</v>
+      </c>
+      <c r="J70" s="15"/>
+      <c r="K70" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" ht="106.2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A71" s="9" t="s">
+        <v>499</v>
+      </c>
+      <c r="B71" s="9" t="s">
+        <v>500</v>
+      </c>
+      <c r="C71" s="15" t="s">
+        <v>501</v>
+      </c>
+      <c r="D71" s="15" t="s">
+        <v>502</v>
+      </c>
+      <c r="E71" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="F71" s="15">
+        <v>1</v>
+      </c>
+      <c r="G71" s="15" t="s">
+        <v>237</v>
+      </c>
+      <c r="H71" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I71" s="15" t="s">
+        <v>228</v>
+      </c>
+      <c r="J71" s="15"/>
+      <c r="K71" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11" ht="119.4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A72" s="9" t="s">
+        <v>515</v>
+      </c>
+      <c r="B72" s="9" t="s">
+        <v>516</v>
+      </c>
+      <c r="C72" s="15" t="s">
+        <v>517</v>
+      </c>
+      <c r="D72" s="15" t="s">
+        <v>518</v>
+      </c>
+      <c r="E72" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="F72" s="15">
+        <v>1</v>
+      </c>
+      <c r="G72" s="15" t="s">
+        <v>237</v>
+      </c>
+      <c r="H72" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I72" s="15" t="s">
+        <v>228</v>
+      </c>
+      <c r="J72" s="15"/>
+      <c r="K72" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" collapsed="1" x14ac:dyDescent="0.3">
+      <c r="A73" s="24" t="s">
+        <v>256</v>
+      </c>
+      <c r="B73" s="22"/>
+      <c r="C73" s="25" t="s">
+        <v>531</v>
+      </c>
+      <c r="D73" s="23"/>
+      <c r="E73" s="23"/>
+      <c r="F73" s="23"/>
+      <c r="G73" s="23"/>
+      <c r="H73" s="23"/>
+      <c r="I73" s="23"/>
+      <c r="J73" s="23"/>
+      <c r="K73" s="23"/>
+    </row>
+    <row r="74" spans="1:11" ht="159" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A74" s="9" t="s">
+        <v>247</v>
+      </c>
+      <c r="B74" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="C74" s="15" t="s">
+        <v>254</v>
+      </c>
+      <c r="D74" s="15" t="s">
+        <v>255</v>
+      </c>
+      <c r="E74" s="15" t="s">
+        <v>256</v>
+      </c>
+      <c r="F74" s="15">
+        <v>2</v>
+      </c>
+      <c r="G74" s="15" t="s">
+        <v>257</v>
+      </c>
+      <c r="H74" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I74" s="15" t="s">
+        <v>228</v>
+      </c>
+      <c r="J74" s="15"/>
+      <c r="K74" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="75" spans="1:11" ht="93" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A75" s="9" t="s">
+        <v>389</v>
+      </c>
+      <c r="B75" s="9" t="s">
+        <v>158</v>
+      </c>
+      <c r="C75" s="15" t="s">
+        <v>390</v>
+      </c>
+      <c r="D75" s="15" t="s">
+        <v>391</v>
+      </c>
+      <c r="E75" s="15" t="s">
+        <v>256</v>
+      </c>
+      <c r="F75" s="15">
+        <v>1</v>
+      </c>
+      <c r="G75" s="15" t="s">
+        <v>237</v>
+      </c>
+      <c r="H75" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I75" s="15" t="s">
+        <v>206</v>
+      </c>
+      <c r="J75" s="15"/>
+      <c r="K75" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11" ht="66.599999999999994" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A76" s="9" t="s">
+        <v>417</v>
+      </c>
+      <c r="B76" s="9" t="s">
+        <v>170</v>
+      </c>
+      <c r="C76" s="15" t="s">
+        <v>418</v>
+      </c>
+      <c r="D76" s="15" t="s">
+        <v>419</v>
+      </c>
+      <c r="E76" s="15" t="s">
+        <v>256</v>
+      </c>
+      <c r="F76" s="15">
+        <v>1</v>
+      </c>
+      <c r="G76" s="15" t="s">
+        <v>237</v>
+      </c>
+      <c r="H76" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I76" s="15" t="s">
+        <v>228</v>
+      </c>
+      <c r="J76" s="15"/>
+      <c r="K76" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="77" spans="1:11" ht="145.80000000000001" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A77" s="9" t="s">
+        <v>426</v>
+      </c>
+      <c r="B77" s="9" t="s">
+        <v>428</v>
+      </c>
+      <c r="C77" s="15" t="s">
+        <v>429</v>
+      </c>
+      <c r="D77" s="15" t="s">
+        <v>430</v>
+      </c>
+      <c r="E77" s="15" t="s">
+        <v>256</v>
+      </c>
+      <c r="F77" s="15">
+        <v>1</v>
+      </c>
+      <c r="G77" s="15" t="s">
+        <v>237</v>
+      </c>
+      <c r="H77" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I77" s="15" t="s">
+        <v>228</v>
+      </c>
+      <c r="J77" s="15"/>
+      <c r="K77" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11" collapsed="1" x14ac:dyDescent="0.3">
+      <c r="A78" s="24" t="s">
+        <v>226</v>
+      </c>
+      <c r="B78" s="22"/>
+      <c r="C78" s="25" t="s">
+        <v>532</v>
+      </c>
+      <c r="D78" s="23"/>
+      <c r="E78" s="23"/>
+      <c r="F78" s="23"/>
+      <c r="G78" s="23"/>
+      <c r="H78" s="23"/>
+      <c r="I78" s="23"/>
+      <c r="J78" s="23"/>
+      <c r="K78" s="23"/>
+    </row>
+    <row r="79" spans="1:11" ht="159" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A79" s="9" t="s">
+        <v>214</v>
+      </c>
+      <c r="B79" s="9" t="s">
+        <v>216</v>
+      </c>
+      <c r="C79" s="15" t="s">
+        <v>224</v>
+      </c>
+      <c r="D79" s="15" t="s">
+        <v>225</v>
+      </c>
+      <c r="E79" s="15" t="s">
+        <v>226</v>
+      </c>
+      <c r="F79" s="15">
+        <v>2</v>
+      </c>
+      <c r="G79" s="15" t="s">
+        <v>227</v>
+      </c>
+      <c r="H79" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I79" s="15" t="s">
+        <v>228</v>
+      </c>
+      <c r="J79" s="15" t="s">
+        <v>229</v>
+      </c>
+      <c r="K79" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="80" spans="1:11" ht="132.6" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A80" s="9" t="s">
+        <v>232</v>
+      </c>
+      <c r="B80" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="C80" s="15" t="s">
+        <v>242</v>
+      </c>
+      <c r="D80" s="15" t="s">
+        <v>243</v>
+      </c>
+      <c r="E80" s="15" t="s">
+        <v>226</v>
+      </c>
+      <c r="F80" s="15">
+        <v>3</v>
+      </c>
+      <c r="G80" s="15" t="s">
+        <v>244</v>
+      </c>
+      <c r="H80" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I80" s="15" t="s">
+        <v>228</v>
+      </c>
+      <c r="J80" s="15"/>
+      <c r="K80" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="81" spans="1:11" ht="185.4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A81" s="9" t="s">
+        <v>260</v>
+      </c>
+      <c r="B81" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="C81" s="15" t="s">
+        <v>276</v>
+      </c>
+      <c r="D81" s="15" t="s">
+        <v>277</v>
+      </c>
+      <c r="E81" s="15" t="s">
+        <v>226</v>
+      </c>
+      <c r="F81" s="15">
+        <v>2</v>
+      </c>
+      <c r="G81" s="15" t="s">
+        <v>278</v>
+      </c>
+      <c r="H81" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I81" s="15" t="s">
+        <v>206</v>
+      </c>
+      <c r="J81" s="15"/>
+      <c r="K81" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="82" spans="1:11" ht="93" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A82" s="11" t="s">
+        <v>359</v>
+      </c>
+      <c r="B82" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="C82" s="14" t="s">
+        <v>361</v>
+      </c>
+      <c r="D82" s="14" t="s">
+        <v>362</v>
+      </c>
+      <c r="E82" s="14" t="s">
+        <v>226</v>
+      </c>
+      <c r="F82" s="14">
+        <v>2</v>
+      </c>
+      <c r="G82" s="14" t="s">
+        <v>241</v>
+      </c>
+      <c r="H82" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="I82" s="14" t="s">
+        <v>191</v>
+      </c>
+      <c r="J82" s="14" t="s">
+        <v>363</v>
+      </c>
+      <c r="K82" s="14" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="83" spans="1:11" collapsed="1" x14ac:dyDescent="0.3">
+      <c r="A83" s="24" t="s">
+        <v>42</v>
+      </c>
+      <c r="B83" s="22"/>
+      <c r="C83" s="25" t="s">
+        <v>533</v>
+      </c>
+      <c r="D83" s="23"/>
+      <c r="E83" s="23"/>
+      <c r="F83" s="23"/>
+      <c r="G83" s="23"/>
+      <c r="H83" s="23"/>
+      <c r="I83" s="23"/>
+      <c r="J83" s="23"/>
+      <c r="K83" s="23"/>
+    </row>
+    <row r="84" spans="1:11" ht="198.6" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A84" s="9" t="s">
+        <v>184</v>
+      </c>
+      <c r="B84" s="9" t="s">
+        <v>186</v>
+      </c>
+      <c r="C84" s="15" t="s">
+        <v>202</v>
+      </c>
+      <c r="D84" s="15" t="s">
+        <v>203</v>
+      </c>
+      <c r="E84" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="F84" s="15">
+        <v>4</v>
+      </c>
+      <c r="G84" s="15" t="s">
+        <v>204</v>
+      </c>
+      <c r="H84" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I84" s="15" t="s">
+        <v>206</v>
+      </c>
+      <c r="J84" s="15" t="s">
+        <v>207</v>
+      </c>
+      <c r="K84" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="85" spans="1:11" ht="225" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A85" s="9" t="s">
+        <v>305</v>
+      </c>
+      <c r="B85" s="9" t="s">
+        <v>307</v>
+      </c>
+      <c r="C85" s="15" t="s">
+        <v>339</v>
+      </c>
+      <c r="D85" s="15" t="s">
+        <v>340</v>
+      </c>
+      <c r="E85" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="F85" s="15">
+        <v>12</v>
+      </c>
+      <c r="G85" s="15" t="s">
+        <v>341</v>
+      </c>
+      <c r="H85" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I85" s="15" t="s">
+        <v>206</v>
+      </c>
+      <c r="J85" s="15" t="s">
+        <v>342</v>
+      </c>
+      <c r="K85" s="15" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="86" spans="1:11" ht="79.8" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A86" s="9" t="s">
+        <v>431</v>
+      </c>
+      <c r="B86" s="9" t="s">
+        <v>431</v>
+      </c>
+      <c r="C86" s="15" t="s">
+        <v>435</v>
+      </c>
+      <c r="D86" s="15" t="s">
+        <v>436</v>
+      </c>
+      <c r="E86" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="F86" s="15">
+        <v>3</v>
+      </c>
+      <c r="G86" s="15" t="s">
+        <v>200</v>
+      </c>
+      <c r="H86" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I86" s="15" t="s">
+        <v>228</v>
+      </c>
+      <c r="J86" s="15"/>
+      <c r="K86" s="15" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="87" spans="1:11" ht="106.2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A87" s="9" t="s">
+        <v>457</v>
+      </c>
+      <c r="B87" s="9" t="s">
+        <v>458</v>
+      </c>
+      <c r="C87" s="15" t="s">
+        <v>461</v>
+      </c>
+      <c r="D87" s="15" t="s">
+        <v>462</v>
+      </c>
+      <c r="E87" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="F87" s="15">
+        <v>2</v>
+      </c>
+      <c r="G87" s="15" t="s">
+        <v>200</v>
+      </c>
+      <c r="H87" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I87" s="15" t="s">
+        <v>206</v>
+      </c>
+      <c r="J87" s="15"/>
+      <c r="K87" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="88" spans="1:11" collapsed="1" x14ac:dyDescent="0.3">
+      <c r="A88" s="24" t="s">
+        <v>37</v>
+      </c>
+      <c r="B88" s="22"/>
+      <c r="C88" s="25" t="s">
+        <v>534</v>
+      </c>
+      <c r="D88" s="23"/>
+      <c r="E88" s="23"/>
+      <c r="F88" s="23"/>
+      <c r="G88" s="23"/>
+      <c r="H88" s="23"/>
+      <c r="I88" s="23"/>
+      <c r="J88" s="23"/>
+      <c r="K88" s="23"/>
+    </row>
+    <row r="89" spans="1:11" ht="119.4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A89" s="9" t="s">
+        <v>282</v>
+      </c>
+      <c r="B89" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="C89" s="15" t="s">
+        <v>302</v>
+      </c>
+      <c r="D89" s="15" t="s">
+        <v>303</v>
+      </c>
+      <c r="E89" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="F89" s="15">
+        <v>4</v>
+      </c>
+      <c r="G89" s="15" t="s">
+        <v>200</v>
+      </c>
+      <c r="H89" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I89" s="15" t="s">
+        <v>206</v>
+      </c>
+      <c r="J89" s="15"/>
+      <c r="K89" s="15" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="90" spans="1:11" ht="132.6" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A90" s="11" t="s">
+        <v>305</v>
+      </c>
+      <c r="B90" s="11" t="s">
+        <v>307</v>
+      </c>
+      <c r="C90" s="14" t="s">
+        <v>334</v>
+      </c>
+      <c r="D90" s="14" t="s">
+        <v>335</v>
+      </c>
+      <c r="E90" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="F90" s="14">
+        <v>6</v>
+      </c>
+      <c r="G90" s="14" t="s">
+        <v>336</v>
+      </c>
+      <c r="H90" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="I90" s="14" t="s">
+        <v>191</v>
+      </c>
+      <c r="J90" s="14" t="s">
+        <v>337</v>
+      </c>
+      <c r="K90" s="14" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="91" spans="1:11" ht="106.2" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A91" s="9" t="s">
+        <v>359</v>
+      </c>
+      <c r="B91" s="9" t="s">
+        <v>147</v>
+      </c>
+      <c r="C91" s="15" t="s">
+        <v>371</v>
+      </c>
+      <c r="D91" s="15" t="s">
+        <v>372</v>
+      </c>
+      <c r="E91" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="F91" s="15">
+        <v>3</v>
+      </c>
+      <c r="G91" s="15" t="s">
+        <v>200</v>
+      </c>
+      <c r="H91" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I91" s="15" t="s">
+        <v>206</v>
+      </c>
+      <c r="J91" s="15"/>
+      <c r="K91" s="15" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="92" spans="1:11" collapsed="1" x14ac:dyDescent="0.3">
+      <c r="A92" s="24" t="s">
+        <v>326</v>
+      </c>
+      <c r="B92" s="22"/>
+      <c r="C92" s="25" t="s">
+        <v>535</v>
+      </c>
+      <c r="D92" s="23"/>
+      <c r="E92" s="23"/>
+      <c r="F92" s="23"/>
+      <c r="G92" s="23"/>
+      <c r="H92" s="23"/>
+      <c r="I92" s="23"/>
+      <c r="J92" s="23"/>
+      <c r="K92" s="23"/>
+    </row>
+    <row r="93" spans="1:11" ht="145.80000000000001" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A93" s="9" t="s">
+        <v>305</v>
+      </c>
+      <c r="B93" s="9" t="s">
+        <v>307</v>
+      </c>
+      <c r="C93" s="15" t="s">
+        <v>324</v>
+      </c>
+      <c r="D93" s="15" t="s">
+        <v>325</v>
+      </c>
+      <c r="E93" s="15" t="s">
+        <v>326</v>
+      </c>
+      <c r="F93" s="15">
+        <v>3</v>
+      </c>
+      <c r="G93" s="15" t="s">
+        <v>327</v>
+      </c>
+      <c r="H93" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I93" s="15" t="s">
+        <v>206</v>
+      </c>
+      <c r="J93" s="15" t="s">
+        <v>328</v>
+      </c>
+      <c r="K93" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="94" spans="1:11" ht="119.4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A94" s="9" t="s">
+        <v>374</v>
+      </c>
+      <c r="B94" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="C94" s="15" t="s">
+        <v>376</v>
+      </c>
+      <c r="D94" s="15" t="s">
+        <v>377</v>
+      </c>
+      <c r="E94" s="15" t="s">
+        <v>326</v>
+      </c>
+      <c r="F94" s="15">
+        <v>3</v>
+      </c>
+      <c r="G94" s="15" t="s">
+        <v>378</v>
+      </c>
+      <c r="H94" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I94" s="15" t="s">
+        <v>206</v>
+      </c>
+      <c r="J94" s="15"/>
+      <c r="K94" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="95" spans="1:11" collapsed="1" x14ac:dyDescent="0.3">
+      <c r="A95" s="24" t="s">
+        <v>47</v>
+      </c>
+      <c r="B95" s="22"/>
+      <c r="C95" s="25" t="s">
+        <v>536</v>
+      </c>
+      <c r="D95" s="23"/>
+      <c r="E95" s="23"/>
+      <c r="F95" s="23"/>
+      <c r="G95" s="23"/>
+      <c r="H95" s="23"/>
+      <c r="I95" s="23"/>
+      <c r="J95" s="23"/>
+      <c r="K95" s="23"/>
+    </row>
+    <row r="96" spans="1:11" ht="159" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A96" s="11" t="s">
+        <v>344</v>
+      </c>
+      <c r="B96" s="11" t="s">
+        <v>140</v>
+      </c>
+      <c r="C96" s="14" t="s">
+        <v>350</v>
+      </c>
+      <c r="D96" s="14" t="s">
+        <v>351</v>
+      </c>
+      <c r="E96" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="F96" s="14">
+        <v>1</v>
+      </c>
+      <c r="G96" s="14" t="s">
+        <v>237</v>
+      </c>
+      <c r="H96" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="I96" s="14" t="s">
+        <v>191</v>
+      </c>
+      <c r="J96" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="K96" s="14" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="97" spans="1:11" ht="145.80000000000001" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A97" s="9" t="s">
+        <v>495</v>
+      </c>
+      <c r="B97" s="9" t="s">
+        <v>496</v>
+      </c>
+      <c r="C97" s="15" t="s">
+        <v>497</v>
+      </c>
+      <c r="D97" s="15" t="s">
+        <v>498</v>
+      </c>
+      <c r="E97" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="F97" s="15">
+        <v>1</v>
+      </c>
+      <c r="G97" s="15" t="s">
+        <v>237</v>
+      </c>
+      <c r="H97" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I97" s="15" t="s">
+        <v>228</v>
+      </c>
+      <c r="J97" s="15"/>
+      <c r="K97" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="98" spans="1:11" collapsed="1" x14ac:dyDescent="0.3">
+      <c r="A98" s="24" t="s">
+        <v>321</v>
+      </c>
+      <c r="B98" s="22"/>
+      <c r="C98" s="25" t="s">
+        <v>537</v>
+      </c>
+      <c r="D98" s="23"/>
+      <c r="E98" s="23"/>
+      <c r="F98" s="23"/>
+      <c r="G98" s="23"/>
+      <c r="H98" s="23"/>
+      <c r="I98" s="23"/>
+      <c r="J98" s="23"/>
+      <c r="K98" s="23"/>
+    </row>
+    <row r="99" spans="1:11" ht="132.6" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A99" s="9" t="s">
+        <v>305</v>
+      </c>
+      <c r="B99" s="9" t="s">
+        <v>307</v>
+      </c>
+      <c r="C99" s="15" t="s">
+        <v>319</v>
+      </c>
+      <c r="D99" s="15" t="s">
+        <v>320</v>
+      </c>
+      <c r="E99" s="15" t="s">
+        <v>321</v>
+      </c>
+      <c r="F99" s="15">
+        <v>2</v>
+      </c>
+      <c r="G99" s="15" t="s">
+        <v>322</v>
+      </c>
+      <c r="H99" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="I99" s="15" t="s">
+        <v>206</v>
+      </c>
+      <c r="J99" s="15" t="s">
+        <v>323</v>
+      </c>
+      <c r="K99" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="100" spans="1:11" collapsed="1" x14ac:dyDescent="0.3">
+      <c r="A100" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="B100" s="22"/>
+      <c r="C100" s="25" t="s">
+        <v>538</v>
+      </c>
+      <c r="D100" s="23"/>
+      <c r="E100" s="23"/>
+      <c r="F100" s="23"/>
+      <c r="G100" s="23"/>
+      <c r="H100" s="23"/>
+      <c r="I100" s="23"/>
+      <c r="J100" s="23"/>
+      <c r="K100" s="23"/>
+    </row>
+    <row r="101" spans="1:11" ht="159" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A101" s="13" t="s">
+        <v>184</v>
+      </c>
+      <c r="B101" s="13" t="s">
+        <v>186</v>
+      </c>
+      <c r="C101" s="17" t="s">
+        <v>208</v>
+      </c>
+      <c r="D101" s="17" t="s">
+        <v>209</v>
+      </c>
+      <c r="E101" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="F101" s="17">
+        <v>6</v>
+      </c>
+      <c r="G101" s="17" t="s">
+        <v>210</v>
+      </c>
+      <c r="H101" s="17" t="s">
+        <v>211</v>
+      </c>
+      <c r="I101" s="17" t="s">
+        <v>212</v>
+      </c>
+      <c r="J101" s="17" t="s">
+        <v>213</v>
+      </c>
+      <c r="K101" s="17" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="102" spans="1:11" collapsed="1" x14ac:dyDescent="0.3">
+      <c r="A102" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="B102" s="22"/>
+      <c r="C102" s="25" t="s">
+        <v>539</v>
+      </c>
+      <c r="D102" s="23"/>
+      <c r="E102" s="23"/>
+      <c r="F102" s="23"/>
+      <c r="G102" s="23"/>
+      <c r="H102" s="23"/>
+      <c r="I102" s="23"/>
+      <c r="J102" s="23"/>
+      <c r="K102" s="23"/>
+    </row>
+    <row r="103" spans="1:11" ht="159" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A103" s="13" t="s">
+        <v>247</v>
+      </c>
+      <c r="B103" s="13" t="s">
+        <v>249</v>
+      </c>
+      <c r="C103" s="17" t="s">
+        <v>250</v>
+      </c>
+      <c r="D103" s="17" t="s">
+        <v>251</v>
+      </c>
+      <c r="E103" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="F103" s="17">
+        <v>1</v>
+      </c>
+      <c r="G103" s="17" t="s">
+        <v>252</v>
+      </c>
+      <c r="H103" s="17" t="s">
+        <v>211</v>
+      </c>
+      <c r="I103" s="17" t="s">
+        <v>212</v>
+      </c>
+      <c r="J103" s="17" t="s">
+        <v>253</v>
+      </c>
+      <c r="K103" s="17" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="104" spans="1:11" collapsed="1" x14ac:dyDescent="0.3">
+      <c r="A104" s="24" t="s">
+        <v>56</v>
+      </c>
+      <c r="B104" s="22"/>
+      <c r="C104" s="25" t="s">
+        <v>540</v>
+      </c>
+      <c r="D104" s="23"/>
+      <c r="E104" s="23"/>
+      <c r="F104" s="23"/>
+      <c r="G104" s="23"/>
+      <c r="H104" s="23"/>
+      <c r="I104" s="23"/>
+      <c r="J104" s="23"/>
+      <c r="K104" s="23"/>
+    </row>
+    <row r="105" spans="1:11" ht="145.80000000000001" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A105" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="B105" s="11" t="s">
+        <v>186</v>
+      </c>
+      <c r="C105" s="14" t="s">
+        <v>198</v>
+      </c>
+      <c r="D105" s="14" t="s">
+        <v>199</v>
+      </c>
+      <c r="E105" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="F105" s="14">
+        <v>1</v>
+      </c>
+      <c r="G105" s="14" t="s">
+        <v>200</v>
+      </c>
+      <c r="H105" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="I105" s="14" t="s">
+        <v>191</v>
+      </c>
+      <c r="J105" s="14" t="s">
+        <v>201</v>
+      </c>
+      <c r="K105" s="14" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="106" spans="1:11" collapsed="1" x14ac:dyDescent="0.3">
+      <c r="A106" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="B106" s="22"/>
+      <c r="C106" s="25" t="s">
+        <v>540</v>
+      </c>
+      <c r="D106" s="23"/>
+      <c r="E106" s="23"/>
+      <c r="F106" s="23"/>
+      <c r="G106" s="23"/>
+      <c r="H106" s="23"/>
+      <c r="I106" s="23"/>
+      <c r="J106" s="23"/>
+      <c r="K106" s="23"/>
+    </row>
+    <row r="107" spans="1:11" ht="159" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A107" s="11" t="s">
+        <v>305</v>
+      </c>
+      <c r="B107" s="11" t="s">
+        <v>307</v>
+      </c>
+      <c r="C107" s="14" t="s">
+        <v>308</v>
+      </c>
+      <c r="D107" s="14" t="s">
+        <v>309</v>
+      </c>
+      <c r="E107" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="F107" s="14">
+        <v>1</v>
+      </c>
+      <c r="G107" s="14" t="s">
+        <v>237</v>
+      </c>
+      <c r="H107" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="I107" s="14" t="s">
+        <v>191</v>
+      </c>
+      <c r="J107" s="14" t="s">
+        <v>310</v>
+      </c>
+      <c r="K107" s="14" t="s">
+        <v>193</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A3:K3" xr:uid="{4D3B3E0A-BA90-4939-991F-4C9A794F6191}"/>
+  <mergeCells count="17">
+    <mergeCell ref="C98:K98"/>
+    <mergeCell ref="C100:K100"/>
+    <mergeCell ref="C102:K102"/>
+    <mergeCell ref="C104:K104"/>
+    <mergeCell ref="C106:K106"/>
+    <mergeCell ref="C73:K73"/>
+    <mergeCell ref="C78:K78"/>
+    <mergeCell ref="C83:K83"/>
+    <mergeCell ref="C88:K88"/>
+    <mergeCell ref="C92:K92"/>
+    <mergeCell ref="C95:K95"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="C4:K4"/>
+    <mergeCell ref="C25:K25"/>
+    <mergeCell ref="C41:K41"/>
+    <mergeCell ref="C56:K56"/>
+    <mergeCell ref="C67:K67"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3EFFE12F-C7B1-4BC5-A174-5F3ED5AFF8E4}">
   <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -7600,7 +11017,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:E3" xr:uid="{27130E95-0811-4A0B-A01B-CAF6D9C8D224}"/>
+  <autoFilter ref="A3:E3" xr:uid="{3EFFE12F-C7B1-4BC5-A174-5F3ED5AFF8E4}"/>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
   </mergeCells>
@@ -7608,8 +11025,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C0CE624-02A4-4A49-BA11-9CC2BF6D3829}">
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9103D5F2-0E5E-48DC-B076-0498D1ABAC3E}">
   <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -7814,8 +11231,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C044133-EC9A-474B-9594-6BDAFD92E6A6}">
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BD161C2-1547-4072-8859-8A842F755591}">
   <dimension ref="A1:D47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -7826,7 +11243,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="18" x14ac:dyDescent="0.35">
       <c r="A1" s="20" t="s">
-        <v>525</v>
+        <v>541</v>
       </c>
       <c r="B1" s="20"/>
       <c r="C1" s="20"/>
@@ -7839,106 +11256,106 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
-        <v>526</v>
+        <v>542</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>527</v>
+        <v>543</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>528</v>
+        <v>544</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
-        <v>529</v>
+        <v>545</v>
       </c>
       <c r="B4" s="27" t="s">
-        <v>530</v>
+        <v>546</v>
       </c>
       <c r="C4" s="27" t="s">
-        <v>531</v>
+        <v>547</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
-        <v>532</v>
+        <v>548</v>
       </c>
       <c r="B5" s="27" t="s">
-        <v>533</v>
+        <v>549</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>534</v>
+        <v>550</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
-        <v>535</v>
+        <v>551</v>
       </c>
       <c r="B6" s="27" t="s">
-        <v>536</v>
+        <v>552</v>
       </c>
       <c r="C6" s="27" t="s">
-        <v>537</v>
+        <v>553</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
-        <v>538</v>
+        <v>554</v>
       </c>
       <c r="B7" s="27" t="s">
-        <v>539</v>
+        <v>555</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>540</v>
+        <v>556</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
-        <v>541</v>
+        <v>557</v>
       </c>
       <c r="B8" s="27" t="s">
-        <v>542</v>
+        <v>558</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>543</v>
+        <v>559</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
-        <v>544</v>
+        <v>560</v>
       </c>
       <c r="B9" s="27" t="s">
-        <v>545</v>
+        <v>561</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>546</v>
+        <v>562</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
-        <v>547</v>
+        <v>563</v>
       </c>
       <c r="B10" s="27" t="s">
-        <v>548</v>
+        <v>564</v>
       </c>
       <c r="C10" s="27" t="s">
-        <v>549</v>
+        <v>565</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="7" t="s">
-        <v>550</v>
+        <v>566</v>
       </c>
       <c r="B11" s="27" t="s">
-        <v>551</v>
+        <v>567</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>552</v>
+        <v>568</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="21" t="s">
-        <v>553</v>
+        <v>569</v>
       </c>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
@@ -7948,7 +11365,7 @@
         <v>180</v>
       </c>
       <c r="B14" s="28" t="s">
-        <v>554</v>
+        <v>570</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
@@ -7977,153 +11394,153 @@
     </row>
     <row r="28" spans="1:3" ht="17.399999999999999" x14ac:dyDescent="0.35">
       <c r="A28" s="5" t="s">
-        <v>555</v>
+        <v>571</v>
       </c>
       <c r="B28" s="5"/>
       <c r="C28" s="5"/>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" s="10" t="s">
-        <v>556</v>
+        <v>572</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>557</v>
+        <v>573</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="11" t="s">
-        <v>558</v>
+        <v>574</v>
       </c>
       <c r="B31" s="14" t="s">
-        <v>559</v>
+        <v>575</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="11" t="s">
-        <v>560</v>
+        <v>576</v>
       </c>
       <c r="B32" s="14" t="s">
-        <v>561</v>
+        <v>577</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="11" t="s">
-        <v>551</v>
+        <v>567</v>
       </c>
       <c r="B33" s="14" t="s">
-        <v>562</v>
+        <v>578</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="11" t="s">
-        <v>563</v>
+        <v>579</v>
       </c>
       <c r="B34" s="14" t="s">
-        <v>564</v>
+        <v>580</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="11" t="s">
-        <v>565</v>
+        <v>581</v>
       </c>
       <c r="B35" s="14" t="s">
-        <v>566</v>
+        <v>582</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="11" t="s">
-        <v>567</v>
+        <v>583</v>
       </c>
       <c r="B36" s="14" t="s">
-        <v>568</v>
+        <v>584</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="11" t="s">
-        <v>569</v>
+        <v>585</v>
       </c>
       <c r="B37" s="14" t="s">
-        <v>570</v>
+        <v>586</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="11" t="s">
-        <v>571</v>
+        <v>587</v>
       </c>
       <c r="B38" s="14" t="s">
-        <v>572</v>
+        <v>588</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="11" t="s">
-        <v>573</v>
+        <v>589</v>
       </c>
       <c r="B39" s="14" t="s">
-        <v>574</v>
+        <v>590</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="11" t="s">
-        <v>575</v>
+        <v>591</v>
       </c>
       <c r="B40" s="14" t="s">
-        <v>576</v>
+        <v>592</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="11" t="s">
-        <v>577</v>
+        <v>593</v>
       </c>
       <c r="B41" s="14" t="s">
-        <v>578</v>
+        <v>594</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="9" t="s">
-        <v>579</v>
+        <v>595</v>
       </c>
       <c r="B42" s="15" t="s">
-        <v>580</v>
+        <v>596</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="9" t="s">
-        <v>581</v>
+        <v>597</v>
       </c>
       <c r="B43" s="15" t="s">
-        <v>582</v>
+        <v>598</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="11" t="s">
-        <v>583</v>
+        <v>599</v>
       </c>
       <c r="B44" s="14" t="s">
-        <v>584</v>
+        <v>600</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="9" t="s">
-        <v>585</v>
+        <v>601</v>
       </c>
       <c r="B45" s="15" t="s">
-        <v>586</v>
+        <v>602</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="9" t="s">
-        <v>587</v>
+        <v>603</v>
       </c>
       <c r="B46" s="15" t="s">
-        <v>588</v>
+        <v>604</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="9" t="s">
-        <v>589</v>
+        <v>605</v>
       </c>
       <c r="B47" s="15" t="s">
-        <v>590</v>
+        <v>606</v>
       </c>
     </row>
   </sheetData>
@@ -8137,8 +11554,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98C3FB85-BA0C-4991-974E-308CF7363756}">
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67772A58-931E-42F5-8F04-7CACE6B453D1}">
   <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -8666,7 +12083,7 @@
       <c r="G25" s="1"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:G3" xr:uid="{98C3FB85-BA0C-4991-974E-308CF7363756}"/>
+  <autoFilter ref="A3:G3" xr:uid="{67772A58-931E-42F5-8F04-7CACE6B453D1}"/>
   <mergeCells count="2">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A25:G25"/>

</xml_diff>